<commit_message>
Update 2 terms in BCIO_Upper_Defs.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
@@ -451,77 +451,77 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Parent</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Synonyms</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Examples</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>BFO entity</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Sub-ontology</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'has process part'</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'realises'</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Curator note</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Curation status</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Definition source</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Cross reference</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>To be reviewed by</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>Informal definition</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Logical definition</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Parent</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Synonyms</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>BFO entity</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Examples</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'has process part'</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'realises'</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Comment</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Sub-ontology</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Definition source</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Cross reference</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Curator note</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Curation status</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>To be reviewed by</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
@@ -563,32 +563,32 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>An attribute of a behaviour change intervention.</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
           <t>process attribute</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>behaviour change intervention attribute</t>
         </is>
       </c>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="I2" s="2" t="n"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
       <c r="L2" s="2" t="n"/>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N2" s="2" t="n"/>
@@ -596,7 +596,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Published</t>
+          <t>An attribute of a behaviour change intervention.</t>
         </is>
       </c>
       <c r="R2" s="2" t="n"/>
@@ -631,28 +631,28 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>A criterion for selecting people for a BCI population.</t>
+          <t>information content entity</t>
         </is>
       </c>
       <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>information content entity</t>
-        </is>
-      </c>
+      <c r="F3" s="2" t="n"/>
       <c r="G3" s="2" t="n"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
           <t>information content entity</t>
         </is>
       </c>
-      <c r="I3" s="2" t="n"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J3" s="2" t="n"/>
       <c r="K3" s="2" t="n"/>
       <c r="L3" s="2" t="n"/>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N3" s="2" t="n"/>
@@ -660,7 +660,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>Published</t>
+          <t>A criterion for selecting people for a BCI population.</t>
         </is>
       </c>
       <c r="R3" s="2" t="n"/>
@@ -693,18 +693,22 @@
           <t>An intervention that has the aim of influencing human behaviour.</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>intervention</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>BCI</t>
+        </is>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>intervention</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>BCI</t>
-        </is>
-      </c>
+          <t>Involves use of products, services, activities, rules or environmental objects.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
           <t>process</t>
@@ -712,7 +716,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Involves use of products, services, activities, rules or environmental objects.</t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -728,17 +732,13 @@
       <c r="L4" s="2" t="n"/>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N4" s="2" t="n"/>
       <c r="O4" s="2" t="n"/>
       <c r="P4" s="2" t="n"/>
-      <c r="Q4" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q4" s="2" t="n"/>
       <c r="R4" s="2" t="n"/>
       <c r="S4" s="2" t="n"/>
       <c r="T4" s="2" t="inlineStr">
@@ -769,18 +769,22 @@
           <t xml:space="preserve">A BCI evaluation study that involves comparison between two or more BCI scenarios to produce one or more BCI effect estimates. </t>
         </is>
       </c>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>behaviour change intervention evaluation study</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>BCI comparison evaluation study</t>
+        </is>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention evaluation study</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>BCI comparison evaluation study</t>
-        </is>
-      </c>
+          <t>Comparison involves identifying differences between the entities in the scenarios.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n"/>
       <c r="H5" s="2" t="inlineStr">
         <is>
           <t>process</t>
@@ -788,7 +792,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Comparison involves identifying differences between the entities in the scenarios.</t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J5" s="2" t="n"/>
@@ -796,17 +800,13 @@
       <c r="L5" s="2" t="n"/>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N5" s="2" t="n"/>
       <c r="O5" s="2" t="n"/>
       <c r="P5" s="2" t="n"/>
-      <c r="Q5" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q5" s="2" t="n"/>
       <c r="R5" s="2" t="n"/>
       <c r="S5" s="2" t="n"/>
       <c r="T5" s="2" t="inlineStr">
@@ -837,18 +837,22 @@
           <t>An intervention content that is part of a behaviour change intervention.</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>intervention content</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>BCI content</t>
+        </is>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>intervention content</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>BCI content</t>
-        </is>
-      </c>
+          <t xml:space="preserve">Consists of BCTs that can be classified using a BCT taxonomy. </t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n"/>
       <c r="H6" s="2" t="inlineStr">
         <is>
           <t>process</t>
@@ -856,7 +860,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Consists of BCTs that can be classified using a BCT taxonomy. </t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J6" s="2" t="n"/>
@@ -864,17 +868,13 @@
       <c r="L6" s="2" t="n"/>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N6" s="2" t="n"/>
       <c r="O6" s="2" t="n"/>
       <c r="P6" s="2" t="n"/>
-      <c r="Q6" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q6" s="2" t="n"/>
       <c r="R6" s="2" t="n"/>
       <c r="S6" s="2" t="n"/>
       <c r="T6" s="2" t="inlineStr">
@@ -905,18 +905,22 @@
           <t>An intervention context in which the process is a behaviour change intervention.</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>intervention context</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> BCI context</t>
+        </is>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>intervention context</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> BCI context</t>
-        </is>
-      </c>
+          <t>Includes as part BCI population and BCI setting. Use of the word ‘may’ conveys a non-zero probability given available information.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n"/>
       <c r="H7" s="2" t="inlineStr">
         <is>
           <t>object aggregate</t>
@@ -924,7 +928,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Includes as part BCI population and BCI setting. Use of the word ‘may’ conveys a non-zero probability given available information.</t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J7" s="2" t="n"/>
@@ -932,17 +936,13 @@
       <c r="L7" s="2" t="n"/>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N7" s="2" t="n"/>
       <c r="O7" s="2" t="n"/>
       <c r="P7" s="2" t="n"/>
-      <c r="Q7" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q7" s="2" t="n"/>
       <c r="R7" s="2" t="n"/>
       <c r="S7" s="2" t="n"/>
       <c r="T7" s="2" t="inlineStr">
@@ -973,40 +973,40 @@
           <t>An intervention delivery in which the intervention is a behaviour change intervention.</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>intervention delivery</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> BCI delivery</t>
         </is>
       </c>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="I8" s="2" t="n"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="n"/>
       <c r="L8" s="2" t="n"/>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="n"/>
       <c r="P8" s="2" t="n"/>
-      <c r="Q8" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q8" s="2" t="n"/>
       <c r="R8" s="2" t="n"/>
       <c r="S8" s="2" t="n"/>
       <c r="T8" s="2" t="inlineStr">
@@ -1037,16 +1037,24 @@
           <t>A BCI content attribute that is its amount.</t>
         </is>
       </c>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>BCI attribute</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> BCI dose</t>
+        </is>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>BCI attribute</t>
+          <t xml:space="preserve">The dose of an active ingredient in a pharmacological intervention; the number of behaviour change techniques included in an intervention. </t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> BCI dose</t>
+          <t xml:space="preserve">This class requires further specification when it is used because specific BCI content instances may vary in amount in different ways. </t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1056,29 +1064,21 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The dose of an active ingredient in a pharmacological intervention; the number of behaviour change techniques included in an intervention. </t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J9" s="2" t="n"/>
       <c r="K9" s="2" t="n"/>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">This class requires further specification when it is used because specific BCI content instances may vary in amount in different ways. </t>
-        </is>
-      </c>
+      <c r="L9" s="2" t="n"/>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N9" s="2" t="n"/>
       <c r="O9" s="2" t="n"/>
       <c r="P9" s="2" t="n"/>
-      <c r="Q9" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q9" s="2" t="n"/>
       <c r="R9" s="2" t="n"/>
       <c r="S9" s="2" t="n"/>
       <c r="T9" s="2" t="inlineStr">
@@ -1109,18 +1109,22 @@
           <t xml:space="preserve">A behaviour change intervention evaluation finding that characterises the difference between BCI outcome estimates of two BCI scenarios. </t>
         </is>
       </c>
-      <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="n"/>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>behaviour change intervention evaluation finding</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> BCI effect estimate</t>
+        </is>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention evaluation finding</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> BCI effect estimate</t>
-        </is>
-      </c>
+          <t>This includes the following subclasses: 1) BCI effect estimate type -the type of statistic used to represent the difference (e.g. odds ratio, mean difference), 2) BCI effect estimate value – the datum that represents the difference (e.g. 1.35), 3)  BCI effect estimate uncertainty type – the type of statistic used to represent the range of uncertainty of the value (e.g. 95% confidence interval see STATO), and 4) the BCI effect estimate uncertainty value  - the datum representing the uncertainty (e.g. 1.20-1.55).</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
           <t>information content entity</t>
@@ -1128,7 +1132,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>This includes the following subclasses: 1) BCI effect estimate type -the type of statistic used to represent the difference (e.g. odds ratio, mean difference), 2) BCI effect estimate value – the datum that represents the difference (e.g. 1.35), 3)  BCI effect estimate uncertainty type – the type of statistic used to represent the range of uncertainty of the value (e.g. 95% confidence interval see STATO), and 4) the BCI effect estimate uncertainty value  - the datum representing the uncertainty (e.g. 1.20-1.55).</t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J10" s="2" t="n"/>
@@ -1136,17 +1140,13 @@
       <c r="L10" s="2" t="n"/>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N10" s="2" t="n"/>
       <c r="O10" s="2" t="n"/>
       <c r="P10" s="2" t="n"/>
-      <c r="Q10" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q10" s="2" t="n"/>
       <c r="R10" s="2" t="n"/>
       <c r="S10" s="2" t="n"/>
       <c r="T10" s="2" t="inlineStr">
@@ -1177,40 +1177,40 @@
           <t>An evaluation finding that is the output of a BCI evaluation study.</t>
         </is>
       </c>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>evaluation finding</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>intervention evaluation finding</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>BCI evaluation finding</t>
         </is>
       </c>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
       <c r="H11" s="2" t="inlineStr">
         <is>
           <t>information content entoty</t>
         </is>
       </c>
-      <c r="I11" s="2" t="n"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="n"/>
       <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="n"/>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N11" s="2" t="n"/>
       <c r="O11" s="2" t="n"/>
       <c r="P11" s="2" t="n"/>
-      <c r="Q11" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q11" s="2" t="n"/>
       <c r="R11" s="2" t="n"/>
       <c r="S11" s="2" t="n"/>
       <c r="T11" s="2" t="inlineStr">
@@ -1241,18 +1241,22 @@
           <t>A report that is a description of a BCI evaluation study.</t>
         </is>
       </c>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>report</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>BCI evaluation report</t>
+        </is>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>report</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>BCI evaluation report</t>
-        </is>
-      </c>
+          <t>Includes entities that stand in direct relation to the study e.g. authors, findings, funding, aims.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
           <t>generally dependent continuant</t>
@@ -1260,7 +1264,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Includes entities that stand in direct relation to the study e.g. authors, findings, funding, aims.</t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J12" s="2" t="n"/>
@@ -1268,17 +1272,13 @@
       <c r="L12" s="2" t="n"/>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N12" s="2" t="n"/>
       <c r="O12" s="2" t="n"/>
       <c r="P12" s="2" t="n"/>
-      <c r="Q12" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q12" s="2" t="n"/>
       <c r="R12" s="2" t="n"/>
       <c r="S12" s="2" t="n"/>
       <c r="T12" s="2" t="inlineStr">
@@ -1309,40 +1309,40 @@
           <t>An intervention evaluation study of a BCI scenario.</t>
         </is>
       </c>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>intervention evaluation study</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>BCI evaluation study</t>
         </is>
       </c>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
       <c r="H13" s="2" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="I13" s="2" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="n"/>
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="n"/>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N13" s="2" t="n"/>
       <c r="O13" s="2" t="n"/>
       <c r="P13" s="2" t="n"/>
-      <c r="Q13" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q13" s="2" t="n"/>
       <c r="R13" s="2" t="n"/>
       <c r="S13" s="2" t="n"/>
       <c r="T13" s="2" t="inlineStr">
@@ -1373,40 +1373,40 @@
           <t>A plan for a BCI evaluation study.</t>
         </is>
       </c>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>plan</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>BCI evaluation study plan</t>
         </is>
       </c>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
       <c r="H14" s="2" t="inlineStr">
         <is>
           <t>information content entity</t>
         </is>
       </c>
-      <c r="I14" s="2" t="n"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J14" s="2" t="n"/>
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="n"/>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N14" s="2" t="n"/>
       <c r="O14" s="2" t="n"/>
       <c r="P14" s="2" t="n"/>
-      <c r="Q14" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q14" s="2" t="n"/>
       <c r="R14" s="2" t="n"/>
       <c r="S14" s="2" t="n"/>
       <c r="T14" s="2" t="inlineStr">
@@ -1437,40 +1437,40 @@
           <t>An information content entity that is about the likelihood of the BCI evaluation finding misrepresenting the outcome behaviour.</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>information content entity</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>BCI evaluation study risk of bias or error</t>
         </is>
       </c>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
       <c r="H15" s="2" t="inlineStr">
         <is>
           <t>information content entity</t>
         </is>
       </c>
-      <c r="I15" s="2" t="n"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="n"/>
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="n"/>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N15" s="2" t="n"/>
       <c r="O15" s="2" t="n"/>
       <c r="P15" s="2" t="n"/>
-      <c r="Q15" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q15" s="2" t="n"/>
       <c r="R15" s="2" t="n"/>
       <c r="S15" s="2" t="n"/>
       <c r="T15" s="2" t="inlineStr">
@@ -1501,40 +1501,40 @@
           <t xml:space="preserve">A process that is causally active in the relationship between a BCI scenario and its outcome behaviour. </t>
         </is>
       </c>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>BCI mechanism of action; MOA; BCI MOA</t>
         </is>
       </c>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
       <c r="H16" s="2" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="I16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J16" s="2" t="n"/>
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="n"/>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N16" s="2" t="n"/>
       <c r="O16" s="2" t="n"/>
       <c r="P16" s="2" t="n"/>
-      <c r="Q16" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q16" s="2" t="n"/>
       <c r="R16" s="2" t="n"/>
       <c r="S16" s="2" t="n"/>
       <c r="T16" s="2" t="inlineStr">
@@ -1565,40 +1565,40 @@
           <t>An attribute of a BCI delivery that is the physical or informational medium through which a BCI is provided.</t>
         </is>
       </c>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>BCI attribute</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>BCI mode of delivery; BCI MOD; MOD</t>
         </is>
       </c>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
       <c r="H17" s="2" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="I17" s="2" t="n"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J17" s="2" t="n"/>
       <c r="K17" s="2" t="n"/>
       <c r="L17" s="2" t="n"/>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N17" s="2" t="n"/>
       <c r="O17" s="2" t="n"/>
       <c r="P17" s="2" t="n"/>
-      <c r="Q17" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q17" s="2" t="n"/>
       <c r="R17" s="2" t="n"/>
       <c r="S17" s="2" t="n"/>
       <c r="T17" s="2" t="inlineStr">
@@ -1629,37 +1629,37 @@
           <t>Human behaviour that is an intervention outcome.</t>
         </is>
       </c>
-      <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>'individual human behaviour' AND 'intervention outcome'</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>individual human behaviour</t>
         </is>
       </c>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="n"/>
       <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="n"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n"/>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N18" s="2" t="n"/>
       <c r="O18" s="2" t="n"/>
       <c r="P18" s="2" t="n"/>
-      <c r="Q18" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R18" s="2" t="n"/>
+      <c r="Q18" s="2" t="n"/>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>'individual human behaviour' AND 'intervention outcome'</t>
+        </is>
+      </c>
       <c r="S18" s="2" t="n"/>
       <c r="T18" s="2" t="inlineStr">
         <is>
@@ -1689,18 +1689,22 @@
           <t>A BCI evaluation finding that is about an outcome behaviour.</t>
         </is>
       </c>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>behaviour change intervention evaluation finding</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>BCI outcome estimate</t>
+        </is>
+      </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention evaluation finding</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>BCI outcome estimate</t>
-        </is>
-      </c>
+          <t>This includes as subclasses 1) type of outcome estimate (e.g. mean, percentage), 2) value of outcome estimate (e.g. 1.5 cigs per day, 23%), 3) uncertainty estimate type (e.g. 95% CI), and 4) uncertainty estimate value (e.g. 12.0%-45.0%).</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n"/>
       <c r="H19" s="2" t="inlineStr">
         <is>
           <t>information content entoty</t>
@@ -1708,7 +1712,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>This includes as subclasses 1) type of outcome estimate (e.g. mean, percentage), 2) value of outcome estimate (e.g. 1.5 cigs per day, 23%), 3) uncertainty estimate type (e.g. 95% CI), and 4) uncertainty estimate value (e.g. 12.0%-45.0%).</t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J19" s="2" t="n"/>
@@ -1716,17 +1720,13 @@
       <c r="L19" s="2" t="n"/>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N19" s="2" t="n"/>
       <c r="O19" s="2" t="n"/>
       <c r="P19" s="2" t="n"/>
-      <c r="Q19" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q19" s="2" t="n"/>
       <c r="R19" s="2" t="n"/>
       <c r="S19" s="2" t="n"/>
       <c r="T19" s="2" t="inlineStr">
@@ -1757,36 +1757,36 @@
           <t>A physical environment in which a BCI is delivered.</t>
         </is>
       </c>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>environmental system</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>BCI physical setting</t>
         </is>
       </c>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
       <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J20" s="2" t="n"/>
       <c r="K20" s="2" t="n"/>
       <c r="L20" s="2" t="n"/>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N20" s="2" t="n"/>
       <c r="O20" s="2" t="n"/>
       <c r="P20" s="2" t="n"/>
-      <c r="Q20" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q20" s="2" t="n"/>
       <c r="R20" s="2" t="n"/>
       <c r="S20" s="2" t="n"/>
       <c r="T20" s="2" t="inlineStr">
@@ -1817,36 +1817,36 @@
           <t>An intervention population who are exposed to a behaviour change intervention.</t>
         </is>
       </c>
-      <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>intervention population</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>BCI population</t>
         </is>
       </c>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
       <c r="H21" s="2" t="n"/>
-      <c r="I21" s="2" t="n"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J21" s="2" t="n"/>
       <c r="K21" s="2" t="n"/>
       <c r="L21" s="2" t="n"/>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N21" s="2" t="n"/>
       <c r="O21" s="2" t="n"/>
       <c r="P21" s="2" t="n"/>
-      <c r="Q21" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q21" s="2" t="n"/>
       <c r="R21" s="2" t="n"/>
       <c r="S21" s="2" t="n"/>
       <c r="T21" s="2" t="inlineStr">
@@ -1877,20 +1877,24 @@
           <t>A planned process in which a BCI is applied in a given context, including BCI engagement and outcome behaviour.</t>
         </is>
       </c>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>planned process</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>BCI scenario</t>
         </is>
       </c>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
       <c r="H22" s="2" t="n"/>
-      <c r="I22" s="2" t="n"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
           <t>behaviour change intervention outcome behaviour</t>
@@ -1900,17 +1904,13 @@
       <c r="L22" s="2" t="n"/>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N22" s="2" t="n"/>
       <c r="O22" s="2" t="n"/>
       <c r="P22" s="2" t="n"/>
-      <c r="Q22" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q22" s="2" t="n"/>
       <c r="R22" s="2" t="n"/>
       <c r="S22" s="2" t="n"/>
       <c r="T22" s="2" t="inlineStr">
@@ -1941,36 +1941,36 @@
           <t>A plan that is realized in a BCI scenario process.</t>
         </is>
       </c>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>plan</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>BCI scenario plan</t>
         </is>
       </c>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
       <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="n"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J23" s="2" t="n"/>
       <c r="K23" s="2" t="n"/>
       <c r="L23" s="2" t="n"/>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N23" s="2" t="n"/>
       <c r="O23" s="2" t="n"/>
       <c r="P23" s="2" t="n"/>
-      <c r="Q23" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q23" s="2" t="n"/>
       <c r="R23" s="2" t="n"/>
       <c r="S23" s="2" t="n"/>
       <c r="T23" s="2" t="inlineStr">
@@ -2001,36 +2001,36 @@
           <t>A report that describes a BCI scenario.</t>
         </is>
       </c>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>report</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>BCI scenario report</t>
         </is>
       </c>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
       <c r="H24" s="2" t="n"/>
-      <c r="I24" s="2" t="n"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J24" s="2" t="n"/>
       <c r="K24" s="2" t="n"/>
       <c r="L24" s="2" t="n"/>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N24" s="2" t="n"/>
       <c r="O24" s="2" t="n"/>
       <c r="P24" s="2" t="n"/>
-      <c r="Q24" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q24" s="2" t="n"/>
       <c r="R24" s="2" t="n"/>
       <c r="S24" s="2" t="n"/>
       <c r="T24" s="2" t="inlineStr">
@@ -2061,22 +2061,26 @@
           <t>A BCI attribute that involves its temporal organisation.</t>
         </is>
       </c>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>BCI attribute</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>BCI schedule of delivery</t>
+        </is>
+      </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>BCI attribute</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>BCI schedule of delivery</t>
-        </is>
-      </c>
+          <t>Includes the start and end of the BCI and its parts.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n"/>
       <c r="H25" s="2" t="n"/>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Includes the start and end of the BCI and its parts.</t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J25" s="2" t="n"/>
@@ -2084,17 +2088,13 @@
       <c r="L25" s="2" t="n"/>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N25" s="2" t="n"/>
       <c r="O25" s="2" t="n"/>
       <c r="P25" s="2" t="n"/>
-      <c r="Q25" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q25" s="2" t="n"/>
       <c r="R25" s="2" t="n"/>
       <c r="S25" s="2" t="n"/>
       <c r="T25" s="2" t="inlineStr">
@@ -2125,22 +2125,26 @@
           <t xml:space="preserve">An aggregate of entities that form the environment in which a BCI is provided. </t>
         </is>
       </c>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="n"/>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>object aggregate</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>BCI setting</t>
+        </is>
+      </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>object aggregate</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>BCI setting</t>
-        </is>
-      </c>
+          <t>Includes as parts social setting and physical setting.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n"/>
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Includes as parts social setting and physical setting.</t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J26" s="2" t="n"/>
@@ -2148,17 +2152,13 @@
       <c r="L26" s="2" t="n"/>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N26" s="2" t="n"/>
       <c r="O26" s="2" t="n"/>
       <c r="P26" s="2" t="n"/>
-      <c r="Q26" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q26" s="2" t="n"/>
       <c r="R26" s="2" t="n"/>
       <c r="S26" s="2" t="n"/>
       <c r="T26" s="2" t="inlineStr">
@@ -2189,36 +2189,36 @@
           <t>An aggregate of people with whom a BCI population interacts.</t>
         </is>
       </c>
-      <c r="D27" s="2" t="n"/>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>human population</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>BCI social setting</t>
         </is>
       </c>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
       <c r="H27" s="2" t="n"/>
-      <c r="I27" s="2" t="n"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J27" s="2" t="n"/>
       <c r="K27" s="2" t="n"/>
       <c r="L27" s="2" t="n"/>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N27" s="2" t="n"/>
       <c r="O27" s="2" t="n"/>
       <c r="P27" s="2" t="n"/>
-      <c r="Q27" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q27" s="2" t="n"/>
       <c r="R27" s="2" t="n"/>
       <c r="S27" s="2" t="n"/>
       <c r="T27" s="2" t="inlineStr">
@@ -2249,22 +2249,26 @@
           <t>A role played by a person, population or organisation that provides a BCI.</t>
         </is>
       </c>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="n"/>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>BCI source</t>
+        </is>
+      </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>role</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>BCI source</t>
-        </is>
-      </c>
+          <t>This includes individual people, groups of people, and organisations.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n"/>
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>This includes individual people, groups of people, and organisations.</t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J28" s="2" t="n"/>
@@ -2272,17 +2276,13 @@
       <c r="L28" s="2" t="n"/>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N28" s="2" t="n"/>
       <c r="O28" s="2" t="n"/>
       <c r="P28" s="2" t="n"/>
-      <c r="Q28" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q28" s="2" t="n"/>
       <c r="R28" s="2" t="n"/>
       <c r="S28" s="2" t="n"/>
       <c r="T28" s="2" t="inlineStr">
@@ -2313,22 +2313,26 @@
           <t>A role played by a person that contributes substantively to production or reporting of a BCI evaluation study.</t>
         </is>
       </c>
-      <c r="D29" s="2" t="n"/>
-      <c r="E29" s="2" t="n"/>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>BCI study investigator</t>
+        </is>
+      </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>role</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>BCI study investigator</t>
-        </is>
-      </c>
+          <t xml:space="preserve">What counts as substantively is subject to judgement. The level and nature of the contribution can be defined using the CReDiT taxonomy (https://casrai.org/credit/). </t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n"/>
       <c r="H29" s="2" t="n"/>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">What counts as substantively is subject to judgement. The level and nature of the contribution can be defined using the CReDiT taxonomy (https://casrai.org/credit/). </t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J29" s="2" t="n"/>
@@ -2336,17 +2340,13 @@
       <c r="L29" s="2" t="n"/>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N29" s="2" t="n"/>
       <c r="O29" s="2" t="n"/>
       <c r="P29" s="2" t="n"/>
-      <c r="Q29" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q29" s="2" t="n"/>
       <c r="R29" s="2" t="n"/>
       <c r="S29" s="2" t="n"/>
       <c r="T29" s="2" t="inlineStr">
@@ -2377,36 +2377,36 @@
           <t>A research study sample whose behaviour is studied in a BCI evaluation study.</t>
         </is>
       </c>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>research study participants</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>BCI study sample</t>
         </is>
       </c>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="n"/>
       <c r="H30" s="2" t="n"/>
-      <c r="I30" s="2" t="n"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J30" s="2" t="n"/>
       <c r="K30" s="2" t="n"/>
       <c r="L30" s="2" t="n"/>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N30" s="2" t="n"/>
       <c r="O30" s="2" t="n"/>
       <c r="P30" s="2" t="n"/>
-      <c r="Q30" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q30" s="2" t="n"/>
       <c r="R30" s="2" t="n"/>
       <c r="S30" s="2" t="n"/>
       <c r="T30" s="2" t="inlineStr">
@@ -2437,22 +2437,26 @@
           <t>A communication style that is an attribute of a BCI content communication process.</t>
         </is>
       </c>
-      <c r="D31" s="2" t="n"/>
-      <c r="E31" s="2" t="n"/>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>communication style</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>BCI style of delivery</t>
+        </is>
+      </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>communication style</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>BCI style of delivery</t>
-        </is>
-      </c>
+          <t>An example is cold and distant vs. warm and accepting.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n"/>
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>An example is cold and distant vs. warm and accepting.</t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J31" s="2" t="n"/>
@@ -2460,17 +2464,13 @@
       <c r="L31" s="2" t="n"/>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N31" s="2" t="n"/>
       <c r="O31" s="2" t="n"/>
       <c r="P31" s="2" t="n"/>
-      <c r="Q31" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q31" s="2" t="n"/>
       <c r="R31" s="2" t="n"/>
       <c r="S31" s="2" t="n"/>
       <c r="T31" s="2" t="inlineStr">
@@ -2503,36 +2503,36 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>An attribute of a behaviour change intervention (BCI) or a BCI component whereby its content or delivery is varied according to characteristics of members of the target population or setting.</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="n"/>
+          <t>BCI attribute</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>BCI tailoring</t>
+        </is>
+      </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>BCI attribute</t>
+          <t>Tailoring the dose of pharmacotherapy for smoking cessation to the prior level of nicotine dependence of the smoker (static) or to the smokers' current strength of urges to smoke during a quit attempt (dynamic).</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>BCI tailoring</t>
+          <t>Tailoring can be static (i.e., conducted before intervention delivery in a case case), or dynamic (i.e., conducted one or more times after the intervention has started in a given case based on population or setting characteristics present at that time. Population and setting characteristics include the historical factors such as prior exposure to the intervention.</t>
         </is>
       </c>
       <c r="H32" s="2" t="n"/>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Tailoring the dose of pharmacotherapy for smoking cessation to the prior level of nicotine dependence of the smoker (static) or to the smokers' current strength of urges to smoke during a quit attempt (dynamic).</t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J32" s="2" t="n"/>
       <c r="K32" s="2" t="n"/>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>Tailoring can be static (i.e., conducted before intervention delivery in a case case), or dynamic (i.e., conducted one or more times after the intervention has started in a given case based on population or setting characteristics present at that time. Population and setting characteristics include the historical factors such as prior exposure to the intervention.</t>
-        </is>
-      </c>
+      <c r="L32" s="2" t="n"/>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N32" s="2" t="n"/>
@@ -2540,7 +2540,7 @@
       <c r="P32" s="2" t="n"/>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>Published</t>
+          <t>An attribute of a behaviour change intervention (BCI) or a BCI component whereby its content or delivery is varied according to characteristics of members of the target population or setting.</t>
         </is>
       </c>
       <c r="R32" s="2" t="n"/>
@@ -2573,36 +2573,36 @@
           <t>The intervention temporal context where the process is the behaviour change intervention</t>
         </is>
       </c>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>intervention temporal context</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>BCI temporal context</t>
         </is>
       </c>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="n"/>
       <c r="H33" s="2" t="n"/>
-      <c r="I33" s="2" t="n"/>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J33" s="2" t="n"/>
       <c r="K33" s="2" t="n"/>
       <c r="L33" s="2" t="n"/>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N33" s="2" t="n"/>
       <c r="O33" s="2" t="n"/>
       <c r="P33" s="2" t="n"/>
-      <c r="Q33" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q33" s="2" t="n"/>
       <c r="R33" s="2" t="n"/>
       <c r="S33" s="2" t="n"/>
       <c r="T33" s="2" t="inlineStr">
@@ -2633,36 +2633,36 @@
           <t xml:space="preserve">An event which occurs during a behaviour change intervention temporal context. </t>
         </is>
       </c>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>behaviour change intervention temporal context</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>BCI temporal context event</t>
         </is>
       </c>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
       <c r="H34" s="2" t="n"/>
-      <c r="I34" s="2" t="n"/>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J34" s="2" t="n"/>
       <c r="K34" s="2" t="n"/>
       <c r="L34" s="2" t="n"/>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N34" s="2" t="n"/>
       <c r="O34" s="2" t="n"/>
       <c r="P34" s="2" t="n"/>
-      <c r="Q34" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q34" s="2" t="n"/>
       <c r="R34" s="2" t="n"/>
       <c r="S34" s="2" t="n"/>
       <c r="T34" s="2" t="inlineStr">
@@ -2693,36 +2693,36 @@
           <t>A &lt;planned process&gt; that is the smallest part of BCI content that is observable, replicable and on its own has the potential to bring about behaviour change.</t>
         </is>
       </c>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>planned process</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>BCT</t>
         </is>
       </c>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
       <c r="H35" s="2" t="n"/>
-      <c r="I35" s="2" t="n"/>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J35" s="2" t="n"/>
       <c r="K35" s="2" t="n"/>
       <c r="L35" s="2" t="n"/>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N35" s="2" t="n"/>
       <c r="O35" s="2" t="n"/>
       <c r="P35" s="2" t="n"/>
-      <c r="Q35" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q35" s="2" t="n"/>
       <c r="R35" s="2" t="n"/>
       <c r="S35" s="2" t="n"/>
       <c r="T35" s="2" t="inlineStr">
@@ -2753,32 +2753,32 @@
           <t>An attribute of a communication process.</t>
         </is>
       </c>
-      <c r="D36" s="2" t="n"/>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>process attribute</t>
+        </is>
+      </c>
       <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>process attribute</t>
-        </is>
-      </c>
+      <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="n"/>
       <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="n"/>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J36" s="2" t="n"/>
       <c r="K36" s="2" t="n"/>
       <c r="L36" s="2" t="n"/>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N36" s="2" t="n"/>
       <c r="O36" s="2" t="n"/>
       <c r="P36" s="2" t="n"/>
-      <c r="Q36" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q36" s="2" t="n"/>
       <c r="R36" s="2" t="n"/>
       <c r="S36" s="2" t="n"/>
       <c r="T36" s="2" t="inlineStr">
@@ -2809,32 +2809,32 @@
           <t>A particular manner of communicating aimed at inducing or avoiding certain kinds of responses in others, or demonstrating certain characteristics of the initiator.</t>
         </is>
       </c>
-      <c r="D37" s="2" t="n"/>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>communication process attribute</t>
+        </is>
+      </c>
       <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>communication process attribute</t>
-        </is>
-      </c>
+      <c r="F37" s="2" t="n"/>
       <c r="G37" s="2" t="n"/>
       <c r="H37" s="2" t="n"/>
-      <c r="I37" s="2" t="n"/>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J37" s="2" t="n"/>
       <c r="K37" s="2" t="n"/>
       <c r="L37" s="2" t="n"/>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N37" s="2" t="n"/>
       <c r="O37" s="2" t="n"/>
       <c r="P37" s="2" t="n"/>
-      <c r="Q37" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q37" s="2" t="n"/>
       <c r="R37" s="2" t="n"/>
       <c r="S37" s="2" t="n"/>
       <c r="T37" s="2" t="inlineStr">
@@ -2850,107 +2850,111 @@
       <c r="V37" s="2" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:035000</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>evaluation finding</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>A data item that is the output of an intervention evaluation study.</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>data item</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="n"/>
-      <c r="H38" s="2" t="n"/>
-      <c r="I38" s="2" t="n"/>
-      <c r="J38" s="2" t="n"/>
-      <c r="K38" s="2" t="n"/>
-      <c r="L38" s="2" t="n"/>
-      <c r="M38" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
-      <c r="N38" s="2" t="n"/>
-      <c r="O38" s="2" t="n"/>
-      <c r="P38" s="2" t="n"/>
-      <c r="Q38" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R38" s="2" t="n"/>
-      <c r="S38" s="2" t="n"/>
-      <c r="T38" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
-      <c r="U38" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V38" s="2" t="n"/>
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:050462</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>high cognitive exertion expended on a behaviour</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Cognitive exertion expended on a behaviour that is high.</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>cognitive exertion expended on a behaviour</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="n"/>
+      <c r="F38" s="3" t="n"/>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>High cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="n"/>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="n"/>
+      <c r="K38" s="3" t="n"/>
+      <c r="L38" s="3" t="n"/>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="N38" s="3" t="n"/>
+      <c r="O38" s="3" t="n"/>
+      <c r="P38" s="3" t="n"/>
+      <c r="Q38" s="3" t="n"/>
+      <c r="R38" s="3" t="n"/>
+      <c r="S38" s="3" t="n"/>
+      <c r="T38" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U38" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="V38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050462</t>
+          <t>BCIO:050463</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>high cognitive exertion expended on a behaviour</t>
+          <t>high emotional management  exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Cognitive exertion expended on a behaviour that is high.</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="n"/>
+          <t>Emotional management exertion expended on a behaviour that is high.</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>emotional management exertion expended on a behaviour</t>
+        </is>
+      </c>
       <c r="E39" s="3" t="n"/>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>cognitive exertion expended on a behaviour</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="n"/>
+      <c r="F39" s="3" t="n"/>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>High emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
+        </is>
+      </c>
       <c r="H39" s="3" t="n"/>
-      <c r="I39" s="3" t="n"/>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
       <c r="J39" s="3" t="n"/>
       <c r="K39" s="3" t="n"/>
-      <c r="L39" s="3" t="inlineStr">
-        <is>
-          <t>High cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="L39" s="3" t="n"/>
       <c r="M39" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="N39" s="3" t="n"/>
       <c r="O39" s="3" t="n"/>
       <c r="P39" s="3" t="n"/>
-      <c r="Q39" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="Q39" s="3" t="n"/>
       <c r="R39" s="3" t="n"/>
       <c r="S39" s="3" t="n"/>
       <c r="T39" s="3" t="inlineStr">
@@ -2968,49 +2972,49 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050463</t>
+          <t>BCIO:050464</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>high emotional management  exertion expended on a behaviour</t>
+          <t>high mental exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Emotional management exertion expended on a behaviour that is high.</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="n"/>
+          <t>Mental exertion expended on a behaviour that is high.</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>mental exertion expended on a behaviour</t>
+        </is>
+      </c>
       <c r="E40" s="3" t="n"/>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>emotional management exertion expended on a behaviour</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="n"/>
+      <c r="F40" s="3" t="n"/>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>High mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
+        </is>
+      </c>
       <c r="H40" s="3" t="n"/>
-      <c r="I40" s="3" t="n"/>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
       <c r="J40" s="3" t="n"/>
       <c r="K40" s="3" t="n"/>
-      <c r="L40" s="3" t="inlineStr">
-        <is>
-          <t>High emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="L40" s="3" t="n"/>
       <c r="M40" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="N40" s="3" t="n"/>
       <c r="O40" s="3" t="n"/>
       <c r="P40" s="3" t="n"/>
-      <c r="Q40" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="Q40" s="3" t="n"/>
       <c r="R40" s="3" t="n"/>
       <c r="S40" s="3" t="n"/>
       <c r="T40" s="3" t="inlineStr">
@@ -3028,49 +3032,49 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050464</t>
+          <t>BCIO:050465</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>high mental exertion expended on a behaviour</t>
+          <t>high physical exertion expended on behaviour</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Mental exertion expended on a behaviour that is high.</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="n"/>
+          <t>Physical exertion expended on a behaviour that is high</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>physical exertion expended on a behaviour</t>
+        </is>
+      </c>
       <c r="E41" s="3" t="n"/>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>mental exertion expended on a behaviour</t>
-        </is>
-      </c>
-      <c r="G41" s="3" t="n"/>
+      <c r="F41" s="3" t="n"/>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>High physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
+        </is>
+      </c>
       <c r="H41" s="3" t="n"/>
-      <c r="I41" s="3" t="n"/>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
       <c r="J41" s="3" t="n"/>
       <c r="K41" s="3" t="n"/>
-      <c r="L41" s="3" t="inlineStr">
-        <is>
-          <t>High mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="L41" s="3" t="n"/>
       <c r="M41" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="N41" s="3" t="n"/>
       <c r="O41" s="3" t="n"/>
       <c r="P41" s="3" t="n"/>
-      <c r="Q41" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="Q41" s="3" t="n"/>
       <c r="R41" s="3" t="n"/>
       <c r="S41" s="3" t="n"/>
       <c r="T41" s="3" t="inlineStr">
@@ -3088,170 +3092,166 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050465</t>
+          <t>BCIO:042000</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>high physical exertion expended on behaviour</t>
+          <t>human behaviour</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Physical exertion expended on a behaviour that is high</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="n"/>
+          <t>A process that is an individual human behaviour or a population behaviour.</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
       <c r="E42" s="3" t="n"/>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>physical exertion expended on a behaviour</t>
-        </is>
-      </c>
+      <c r="F42" s="3" t="n"/>
       <c r="G42" s="3" t="n"/>
       <c r="H42" s="3" t="n"/>
-      <c r="I42" s="3" t="n"/>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J42" s="3" t="n"/>
       <c r="K42" s="3" t="n"/>
-      <c r="L42" s="3" t="inlineStr">
-        <is>
-          <t>High physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="L42" s="3" t="n"/>
       <c r="M42" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="N42" s="3" t="n"/>
       <c r="O42" s="3" t="n"/>
       <c r="P42" s="3" t="n"/>
-      <c r="Q42" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="R42" s="3" t="n"/>
+      <c r="Q42" s="3" t="n"/>
+      <c r="R42" s="3" t="inlineStr">
+        <is>
+          <t>"individual human behaviour" OR "population behaviour"</t>
+        </is>
+      </c>
       <c r="S42" s="3" t="n"/>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>BG; PS</t>
         </is>
       </c>
       <c r="U42" s="3" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>0</t>
         </is>
       </c>
       <c r="V42" s="3" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:042000</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>human behaviour</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>A process that is an individual human behaviour or a population behaviour.</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="n"/>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>"individual human behaviour" OR "population behaviour"</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="G43" s="3" t="n"/>
-      <c r="H43" s="3" t="n"/>
-      <c r="I43" s="3" t="n"/>
-      <c r="J43" s="3" t="n"/>
-      <c r="K43" s="3" t="n"/>
-      <c r="L43" s="3" t="n"/>
-      <c r="M43" s="3" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
-      <c r="N43" s="3" t="n"/>
-      <c r="O43" s="3" t="n"/>
-      <c r="P43" s="3" t="n"/>
-      <c r="Q43" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="R43" s="3" t="n"/>
-      <c r="S43" s="3" t="n"/>
-      <c r="T43" s="3" t="inlineStr">
-        <is>
-          <t>BG; PS</t>
-        </is>
-      </c>
-      <c r="U43" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V43" s="3" t="n"/>
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:041000</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>human population</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>An object aggregate that consists of two or more people.</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>object aggregate</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+      <c r="G43" s="2" t="n"/>
+      <c r="H43" s="2" t="n"/>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="n"/>
+      <c r="K43" s="2" t="n"/>
+      <c r="L43" s="2" t="n"/>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="n"/>
+      <c r="O43" s="2" t="n"/>
+      <c r="P43" s="2" t="n"/>
+      <c r="Q43" s="2" t="n"/>
+      <c r="R43" s="2" t="n"/>
+      <c r="S43" s="2" t="n"/>
+      <c r="T43" s="2" t="inlineStr">
+        <is>
+          <t>JH; AW</t>
+        </is>
+      </c>
+      <c r="U43" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>BCIO:041000</t>
+          <t>BCIO:040000</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>human population</t>
+          <t>individual human activity</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>An object aggregate that consists of two or more people.</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="n"/>
+          <t>A process that is produced by a person.</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
       <c r="E44" s="2" t="n"/>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>object aggregate</t>
-        </is>
-      </c>
+      <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="n"/>
       <c r="H44" s="2" t="n"/>
-      <c r="I44" s="2" t="n"/>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J44" s="2" t="n"/>
       <c r="K44" s="2" t="n"/>
       <c r="L44" s="2" t="n"/>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N44" s="2" t="n"/>
       <c r="O44" s="2" t="n"/>
       <c r="P44" s="2" t="n"/>
-      <c r="Q44" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q44" s="2" t="n"/>
       <c r="R44" s="2" t="n"/>
       <c r="S44" s="2" t="n"/>
       <c r="T44" s="2" t="inlineStr">
         <is>
-          <t>JH; AW</t>
+          <t>JH</t>
         </is>
       </c>
       <c r="U44" s="2" t="inlineStr">
@@ -3264,45 +3264,53 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>BCIO:040000</t>
+          <t>BCIO:036000</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>individual human activity</t>
+          <t>individual human behaviour</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>A process that is produced by a person.</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="n"/>
-      <c r="E45" s="2" t="n"/>
+          <t xml:space="preserve">A bodily process of a human that involves co-ordinated contraction of striated muscles controlled by the brain. </t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>bodily process</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>human behaviour</t>
+        </is>
+      </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>process</t>
+          <t>Also referred to in definitions as human behaviour or just behaviour.</t>
         </is>
       </c>
       <c r="G45" s="2" t="n"/>
       <c r="H45" s="2" t="n"/>
-      <c r="I45" s="2" t="n"/>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J45" s="2" t="n"/>
       <c r="K45" s="2" t="n"/>
       <c r="L45" s="2" t="n"/>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N45" s="2" t="n"/>
       <c r="O45" s="2" t="n"/>
       <c r="P45" s="2" t="n"/>
-      <c r="Q45" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q45" s="2" t="n"/>
       <c r="R45" s="2" t="n"/>
       <c r="S45" s="2" t="n"/>
       <c r="T45" s="2" t="inlineStr">
@@ -3320,35 +3328,35 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>BCIO:036000</t>
+          <t>BCIO:037000</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>individual human behaviour</t>
+          <t>intervention</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A bodily process of a human that involves co-ordinated contraction of striated muscles controlled by the brain. </t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="n"/>
+          <t>A planned process that has the aim of influencing an outcome.</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>planned process</t>
+        </is>
+      </c>
       <c r="E46" s="2" t="n"/>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>bodily process</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>human behaviour</t>
-        </is>
-      </c>
+          <t>Examples of interventions are putting health warnings on cigarette packets, providing free stop smoking services and banning smoking in public places.</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="n"/>
       <c r="H46" s="2" t="n"/>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Also referred to in definitions as human behaviour or just behaviour.</t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J46" s="2" t="n"/>
@@ -3356,22 +3364,18 @@
       <c r="L46" s="2" t="n"/>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N46" s="2" t="n"/>
       <c r="O46" s="2" t="n"/>
       <c r="P46" s="2" t="n"/>
-      <c r="Q46" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q46" s="2" t="n"/>
       <c r="R46" s="2" t="n"/>
       <c r="S46" s="2" t="n"/>
       <c r="T46" s="2" t="inlineStr">
         <is>
-          <t>JH</t>
+          <t>JH; RW</t>
         </is>
       </c>
       <c r="U46" s="2" t="inlineStr">
@@ -3384,31 +3388,31 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>BCIO:037000</t>
+          <t>BCIO:046000</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>intervention</t>
+          <t>intervention content</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>A planned process that has the aim of influencing an outcome.</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="n"/>
+          <t>A planned process that is part of an intervention and is intended to be causally active in influencing the intervention outcome.</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>planned process</t>
+        </is>
+      </c>
       <c r="E47" s="2" t="n"/>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>planned process</t>
-        </is>
-      </c>
+      <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="n"/>
       <c r="H47" s="2" t="n"/>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>Examples of interventions are putting health warnings on cigarette packets, providing free stop smoking services and banning smoking in public places.</t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J47" s="2" t="n"/>
@@ -3416,22 +3420,18 @@
       <c r="L47" s="2" t="n"/>
       <c r="M47" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N47" s="2" t="n"/>
       <c r="O47" s="2" t="n"/>
       <c r="P47" s="2" t="n"/>
-      <c r="Q47" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q47" s="2" t="n"/>
       <c r="R47" s="2" t="n"/>
       <c r="S47" s="2" t="n"/>
       <c r="T47" s="2" t="inlineStr">
         <is>
-          <t>JH; RW</t>
+          <t>RW</t>
         </is>
       </c>
       <c r="U47" s="2" t="inlineStr">
@@ -3442,133 +3442,133 @@
       <c r="V47" s="2" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:046000</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>intervention content</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>A planned process that is part of an intervention and is intended to be causally active in influencing the intervention outcome.</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="n"/>
-      <c r="E48" s="2" t="n"/>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>GMHO:0000253</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>intervention context</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>process context</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="U48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:045000</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>intervention delivery</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>A planned process by which intervention content is delivered.</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>planned process</t>
         </is>
       </c>
-      <c r="G48" s="2" t="n"/>
-      <c r="H48" s="2" t="n"/>
-      <c r="I48" s="2" t="n"/>
-      <c r="J48" s="2" t="n"/>
-      <c r="K48" s="2" t="n"/>
-      <c r="L48" s="2" t="n"/>
-      <c r="M48" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
-      <c r="N48" s="2" t="n"/>
-      <c r="O48" s="2" t="n"/>
-      <c r="P48" s="2" t="n"/>
-      <c r="Q48" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="R48" s="2" t="n"/>
-      <c r="S48" s="2" t="n"/>
-      <c r="T48" s="2" t="inlineStr">
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="2" t="n"/>
+      <c r="G49" s="2" t="n"/>
+      <c r="H49" s="2" t="n"/>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="n"/>
+      <c r="K49" s="2" t="n"/>
+      <c r="L49" s="2" t="n"/>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="n"/>
+      <c r="O49" s="2" t="n"/>
+      <c r="P49" s="2" t="n"/>
+      <c r="Q49" s="2" t="n"/>
+      <c r="R49" s="2" t="n"/>
+      <c r="S49" s="2" t="n"/>
+      <c r="T49" s="2" t="inlineStr">
         <is>
           <t>RW</t>
         </is>
       </c>
-      <c r="U48" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V48" s="2" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>GMHO:0000253</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>intervention context</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>process context</t>
-        </is>
-      </c>
-      <c r="Q49" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="U49" t="n">
-        <v>0</v>
-      </c>
+      <c r="U49" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>BCIO:045000</t>
+          <t>BCIO:035000</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>intervention delivery</t>
+          <t>intervention evaluation finding</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>A planned process by which intervention content is delivered.</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="n"/>
+          <t>A data item that is the output of an intervention evaluation study.</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
       <c r="E50" s="2" t="n"/>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>planned process</t>
-        </is>
-      </c>
+      <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="n"/>
       <c r="H50" s="2" t="n"/>
-      <c r="I50" s="2" t="n"/>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J50" s="2" t="n"/>
       <c r="K50" s="2" t="n"/>
       <c r="L50" s="2" t="n"/>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N50" s="2" t="n"/>
       <c r="O50" s="2" t="n"/>
       <c r="P50" s="2" t="n"/>
-      <c r="Q50" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q50" s="2" t="n"/>
       <c r="R50" s="2" t="n"/>
       <c r="S50" s="2" t="n"/>
       <c r="T50" s="2" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>JH; RW</t>
         </is>
       </c>
       <c r="U50" s="2" t="inlineStr">
@@ -3594,32 +3594,32 @@
           <t>A research study that aims to assess attributes of an intervention with regards to their positive or negative value.</t>
         </is>
       </c>
-      <c r="D51" s="2" t="n"/>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>research study</t>
+        </is>
+      </c>
       <c r="E51" s="2" t="n"/>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>research study</t>
-        </is>
-      </c>
+      <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="n"/>
       <c r="H51" s="2" t="n"/>
-      <c r="I51" s="2" t="n"/>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J51" s="2" t="n"/>
       <c r="K51" s="2" t="n"/>
       <c r="L51" s="2" t="n"/>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N51" s="2" t="n"/>
       <c r="O51" s="2" t="n"/>
       <c r="P51" s="2" t="n"/>
-      <c r="Q51" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q51" s="2" t="n"/>
       <c r="R51" s="2" t="n"/>
       <c r="S51" s="2" t="n"/>
       <c r="T51" s="2" t="inlineStr">
@@ -3650,18 +3650,22 @@
           <t>An entity that is influenced by an intervention</t>
         </is>
       </c>
-      <c r="D52" s="2" t="n"/>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>entity</t>
+        </is>
+      </c>
       <c r="E52" s="2" t="n"/>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>entity</t>
+          <t xml:space="preserve">Includes individual human behaviour, mental activity and physiological activity. Also includes undesirable outcomes, such as treatment side effects, and unintended negative consequences of the intervention. </t>
         </is>
       </c>
       <c r="G52" s="2" t="n"/>
       <c r="H52" s="2" t="n"/>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Includes individual human behaviour, mental activity and physiological activity. Also includes undesirable outcomes, such as treatment side effects, and unintended negative consequences of the intervention. </t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J52" s="2" t="n"/>
@@ -3669,17 +3673,13 @@
       <c r="L52" s="2" t="n"/>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N52" s="2" t="n"/>
       <c r="O52" s="2" t="n"/>
       <c r="P52" s="2" t="n"/>
-      <c r="Q52" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q52" s="2" t="n"/>
       <c r="R52" s="2" t="n"/>
       <c r="S52" s="2" t="n"/>
       <c r="T52" s="2" t="inlineStr">
@@ -3710,32 +3710,32 @@
           <t>A human population who are exposed to an intervention.</t>
         </is>
       </c>
-      <c r="D53" s="2" t="n"/>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>human population</t>
+        </is>
+      </c>
       <c r="E53" s="2" t="n"/>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>human population</t>
-        </is>
-      </c>
+      <c r="F53" s="2" t="n"/>
       <c r="G53" s="2" t="n"/>
       <c r="H53" s="2" t="n"/>
-      <c r="I53" s="2" t="n"/>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J53" s="2" t="n"/>
       <c r="K53" s="2" t="n"/>
       <c r="L53" s="2" t="n"/>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N53" s="2" t="n"/>
       <c r="O53" s="2" t="n"/>
       <c r="P53" s="2" t="n"/>
-      <c r="Q53" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q53" s="2" t="n"/>
       <c r="R53" s="2" t="n"/>
       <c r="S53" s="2" t="n"/>
       <c r="T53" s="2" t="inlineStr">
@@ -3761,12 +3761,12 @@
           <t>intervention temporal context</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>intervention context</t>
         </is>
       </c>
-      <c r="Q54" t="inlineStr">
+      <c r="M54" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -3791,36 +3791,36 @@
           <t>Cognitive exertion expended on a behaviour that is low.</t>
         </is>
       </c>
-      <c r="D55" s="3" t="n"/>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>cognitive exertion expended on a behaviour</t>
+        </is>
+      </c>
       <c r="E55" s="3" t="n"/>
-      <c r="F55" s="3" t="inlineStr">
-        <is>
-          <t>cognitive exertion expended on a behaviour</t>
-        </is>
-      </c>
-      <c r="G55" s="3" t="n"/>
+      <c r="F55" s="3" t="n"/>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>Low cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
+        </is>
+      </c>
       <c r="H55" s="3" t="n"/>
-      <c r="I55" s="3" t="n"/>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
       <c r="J55" s="3" t="n"/>
       <c r="K55" s="3" t="n"/>
-      <c r="L55" s="3" t="inlineStr">
-        <is>
-          <t>Low cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="L55" s="3" t="n"/>
       <c r="M55" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="N55" s="3" t="n"/>
       <c r="O55" s="3" t="n"/>
       <c r="P55" s="3" t="n"/>
-      <c r="Q55" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="Q55" s="3" t="n"/>
       <c r="R55" s="3" t="n"/>
       <c r="S55" s="3" t="n"/>
       <c r="T55" s="3" t="inlineStr">
@@ -3851,36 +3851,36 @@
           <t>Emotional management exertion expended on a behaviour that is low.</t>
         </is>
       </c>
-      <c r="D56" s="3" t="n"/>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>emotional management exertion expended on a behaviour</t>
+        </is>
+      </c>
       <c r="E56" s="3" t="n"/>
-      <c r="F56" s="3" t="inlineStr">
-        <is>
-          <t>emotional management exertion expended on a behaviour</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="n"/>
+      <c r="F56" s="3" t="n"/>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>Low emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
+        </is>
+      </c>
       <c r="H56" s="3" t="n"/>
-      <c r="I56" s="3" t="n"/>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
       <c r="J56" s="3" t="n"/>
       <c r="K56" s="3" t="n"/>
-      <c r="L56" s="3" t="inlineStr">
-        <is>
-          <t>Low emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="L56" s="3" t="n"/>
       <c r="M56" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="N56" s="3" t="n"/>
       <c r="O56" s="3" t="n"/>
       <c r="P56" s="3" t="n"/>
-      <c r="Q56" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="Q56" s="3" t="n"/>
       <c r="R56" s="3" t="n"/>
       <c r="S56" s="3" t="n"/>
       <c r="T56" s="3" t="inlineStr">
@@ -3911,36 +3911,36 @@
           <t>Mental exertion expended on a behaviour that is low.</t>
         </is>
       </c>
-      <c r="D57" s="3" t="n"/>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>mental exertion expended on a behaviour</t>
+        </is>
+      </c>
       <c r="E57" s="3" t="n"/>
-      <c r="F57" s="3" t="inlineStr">
-        <is>
-          <t>mental exertion expended on a behaviour</t>
-        </is>
-      </c>
-      <c r="G57" s="3" t="n"/>
+      <c r="F57" s="3" t="n"/>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>Low mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
+        </is>
+      </c>
       <c r="H57" s="3" t="n"/>
-      <c r="I57" s="3" t="n"/>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
       <c r="J57" s="3" t="n"/>
       <c r="K57" s="3" t="n"/>
-      <c r="L57" s="3" t="inlineStr">
-        <is>
-          <t>Low mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="L57" s="3" t="n"/>
       <c r="M57" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="N57" s="3" t="n"/>
       <c r="O57" s="3" t="n"/>
       <c r="P57" s="3" t="n"/>
-      <c r="Q57" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="Q57" s="3" t="n"/>
       <c r="R57" s="3" t="n"/>
       <c r="S57" s="3" t="n"/>
       <c r="T57" s="3" t="inlineStr">
@@ -3971,36 +3971,36 @@
           <t>Physical exertion expended on a behaviour that is low.</t>
         </is>
       </c>
-      <c r="D58" s="3" t="n"/>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>physical exertion expended on a behaviour</t>
+        </is>
+      </c>
       <c r="E58" s="3" t="n"/>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
-          <t>physical exertion expended on a behaviour</t>
-        </is>
-      </c>
-      <c r="G58" s="3" t="n"/>
+      <c r="F58" s="3" t="n"/>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means </t>
+        </is>
+      </c>
       <c r="H58" s="3" t="n"/>
-      <c r="I58" s="3" t="n"/>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
       <c r="J58" s="3" t="n"/>
       <c r="K58" s="3" t="n"/>
-      <c r="L58" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Low physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means </t>
-        </is>
-      </c>
+      <c r="L58" s="3" t="n"/>
       <c r="M58" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="N58" s="3" t="n"/>
       <c r="O58" s="3" t="n"/>
       <c r="P58" s="3" t="n"/>
-      <c r="Q58" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="Q58" s="3" t="n"/>
       <c r="R58" s="3" t="n"/>
       <c r="S58" s="3" t="n"/>
       <c r="T58" s="3" t="inlineStr">
@@ -4031,36 +4031,36 @@
           <t>Cognitive exertion expended on a behaviour that is medium.</t>
         </is>
       </c>
-      <c r="D59" s="3" t="n"/>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>cognitive exertion expended on a behaviour</t>
+        </is>
+      </c>
       <c r="E59" s="3" t="n"/>
-      <c r="F59" s="3" t="inlineStr">
-        <is>
-          <t>cognitive exertion expended on a behaviour</t>
-        </is>
-      </c>
-      <c r="G59" s="3" t="n"/>
+      <c r="F59" s="3" t="n"/>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>Moderate cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
+        </is>
+      </c>
       <c r="H59" s="3" t="n"/>
-      <c r="I59" s="3" t="n"/>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
       <c r="J59" s="3" t="n"/>
       <c r="K59" s="3" t="n"/>
-      <c r="L59" s="3" t="inlineStr">
-        <is>
-          <t>Moderate cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="L59" s="3" t="n"/>
       <c r="M59" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="N59" s="3" t="n"/>
       <c r="O59" s="3" t="n"/>
       <c r="P59" s="3" t="n"/>
-      <c r="Q59" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="Q59" s="3" t="n"/>
       <c r="R59" s="3" t="n"/>
       <c r="S59" s="3" t="n"/>
       <c r="T59" s="3" t="inlineStr">
@@ -4091,36 +4091,36 @@
           <t>Emotional management exertion expended on a behaviour that is medium.</t>
         </is>
       </c>
-      <c r="D60" s="3" t="n"/>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>emotional management exertion expended on a behaviour</t>
+        </is>
+      </c>
       <c r="E60" s="3" t="n"/>
-      <c r="F60" s="3" t="inlineStr">
-        <is>
-          <t>emotional management exertion expended on a behaviour</t>
-        </is>
-      </c>
-      <c r="G60" s="3" t="n"/>
+      <c r="F60" s="3" t="n"/>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>Moderate emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
+        </is>
+      </c>
       <c r="H60" s="3" t="n"/>
-      <c r="I60" s="3" t="n"/>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
       <c r="J60" s="3" t="n"/>
       <c r="K60" s="3" t="n"/>
-      <c r="L60" s="3" t="inlineStr">
-        <is>
-          <t>Moderate emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="L60" s="3" t="n"/>
       <c r="M60" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="N60" s="3" t="n"/>
       <c r="O60" s="3" t="n"/>
       <c r="P60" s="3" t="n"/>
-      <c r="Q60" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="Q60" s="3" t="n"/>
       <c r="R60" s="3" t="n"/>
       <c r="S60" s="3" t="n"/>
       <c r="T60" s="3" t="inlineStr">
@@ -4151,36 +4151,36 @@
           <t>Mental exertion expended on a behaviour that is medium.</t>
         </is>
       </c>
-      <c r="D61" s="3" t="n"/>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>mental exertion expended on a behaviour</t>
+        </is>
+      </c>
       <c r="E61" s="3" t="n"/>
-      <c r="F61" s="3" t="inlineStr">
-        <is>
-          <t>mental exertion expended on a behaviour</t>
-        </is>
-      </c>
-      <c r="G61" s="3" t="n"/>
+      <c r="F61" s="3" t="n"/>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>Moderate mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
+        </is>
+      </c>
       <c r="H61" s="3" t="n"/>
-      <c r="I61" s="3" t="n"/>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
       <c r="J61" s="3" t="n"/>
       <c r="K61" s="3" t="n"/>
-      <c r="L61" s="3" t="inlineStr">
-        <is>
-          <t>Moderate mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="L61" s="3" t="n"/>
       <c r="M61" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="N61" s="3" t="n"/>
       <c r="O61" s="3" t="n"/>
       <c r="P61" s="3" t="n"/>
-      <c r="Q61" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="Q61" s="3" t="n"/>
       <c r="R61" s="3" t="n"/>
       <c r="S61" s="3" t="n"/>
       <c r="T61" s="3" t="inlineStr">
@@ -4211,36 +4211,36 @@
           <t>Physical exertion expended on a behaviour that is medium.</t>
         </is>
       </c>
-      <c r="D62" s="3" t="n"/>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>physical exertion expended on a behaviour</t>
+        </is>
+      </c>
       <c r="E62" s="3" t="n"/>
-      <c r="F62" s="3" t="inlineStr">
-        <is>
-          <t>physical exertion expended on a behaviour</t>
-        </is>
-      </c>
-      <c r="G62" s="3" t="n"/>
+      <c r="F62" s="3" t="n"/>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>Moderate physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
+        </is>
+      </c>
       <c r="H62" s="3" t="n"/>
-      <c r="I62" s="3" t="n"/>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
       <c r="J62" s="3" t="n"/>
       <c r="K62" s="3" t="n"/>
-      <c r="L62" s="3" t="inlineStr">
-        <is>
-          <t>Moderate physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="L62" s="3" t="n"/>
       <c r="M62" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Obsolete</t>
         </is>
       </c>
       <c r="N62" s="3" t="n"/>
       <c r="O62" s="3" t="n"/>
       <c r="P62" s="3" t="n"/>
-      <c r="Q62" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="Q62" s="3" t="n"/>
       <c r="R62" s="3" t="n"/>
       <c r="S62" s="3" t="n"/>
       <c r="T62" s="3" t="inlineStr">
@@ -4271,18 +4271,22 @@
           <t>Participant engagement with intervention, where the intervention focuses on changing behaviour.</t>
         </is>
       </c>
-      <c r="D63" s="2" t="n"/>
-      <c r="E63" s="2" t="n"/>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>participant engagement with intervention</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>BCI engagement</t>
+        </is>
+      </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>participant engagement with intervention</t>
-        </is>
-      </c>
-      <c r="G63" s="2" t="inlineStr">
-        <is>
-          <t>BCI engagement</t>
-        </is>
-      </c>
+          <t>Includes mental activities and behaviours.</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="n"/>
       <c r="H63" s="2" t="inlineStr">
         <is>
           <t>process</t>
@@ -4290,7 +4294,7 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>Includes mental activities and behaviours.</t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J63" s="2" t="n"/>
@@ -4298,17 +4302,13 @@
       <c r="L63" s="2" t="n"/>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N63" s="2" t="n"/>
       <c r="O63" s="2" t="n"/>
       <c r="P63" s="2" t="n"/>
-      <c r="Q63" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q63" s="2" t="n"/>
       <c r="R63" s="2" t="n"/>
       <c r="S63" s="2" t="n"/>
       <c r="T63" s="2" t="inlineStr">
@@ -4341,24 +4341,24 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>The extend to someone interacts with an intervention, including their cognitive, emotional and behavioural response (e.g., attending intervention session) to the intervention itself.</t>
+          <t>individual human activity</t>
         </is>
       </c>
       <c r="E64" s="2" t="n"/>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
-          <t>individual human activity</t>
-        </is>
-      </c>
+      <c r="F64" s="2" t="n"/>
       <c r="G64" s="2" t="n"/>
       <c r="H64" s="2" t="n"/>
-      <c r="I64" s="2" t="n"/>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J64" s="2" t="n"/>
       <c r="K64" s="2" t="n"/>
       <c r="L64" s="2" t="n"/>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N64" s="2" t="n"/>
@@ -4366,7 +4366,7 @@
       <c r="P64" s="2" t="n"/>
       <c r="Q64" s="2" t="inlineStr">
         <is>
-          <t>Published</t>
+          <t>The extend to someone interacts with an intervention, including their cognitive, emotional and behavioural response (e.g., attending intervention session) to the intervention itself.</t>
         </is>
       </c>
       <c r="R64" s="2" t="n"/>
@@ -4397,36 +4397,36 @@
           <t>An aggregate of individual human behaviours of members of a population.</t>
         </is>
       </c>
-      <c r="D65" s="2" t="n"/>
-      <c r="E65" s="2" t="n"/>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="G65" s="2" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>human behaviour</t>
         </is>
       </c>
+      <c r="F65" s="2" t="n"/>
+      <c r="G65" s="2" t="n"/>
       <c r="H65" s="2" t="n"/>
-      <c r="I65" s="2" t="n"/>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J65" s="2" t="n"/>
       <c r="K65" s="2" t="n"/>
       <c r="L65" s="2" t="n"/>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N65" s="2" t="n"/>
       <c r="O65" s="2" t="n"/>
       <c r="P65" s="2" t="n"/>
-      <c r="Q65" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q65" s="2" t="n"/>
       <c r="R65" s="2" t="n"/>
       <c r="S65" s="2" t="n"/>
       <c r="T65" s="2" t="inlineStr">
@@ -4459,20 +4459,20 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>An attribute of a process.</t>
+          <t>process profile</t>
         </is>
       </c>
       <c r="E66" s="2" t="n"/>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>process profile</t>
+          <t>This is intended to provide a user-friendly way of representing the way in which processes are manifest. This is somewhat similar to, but not the same as, the class 'specifically dependent continuant' in Basic Formal Ontology which provides a way of representing features of material entities such as age and size. It is formally equivalent to process profile in Basic Formal Ontology.</t>
         </is>
       </c>
       <c r="G66" s="2" t="n"/>
       <c r="H66" s="2" t="n"/>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>This is intended to provide a user-friendly way of representing the way in which processes are manifest. This is somewhat similar to, but not the same as, the class 'specifically dependent continuant' in Basic Formal Ontology which provides a way of representing features of material entities such as age and size. It is formally equivalent to process profile in Basic Formal Ontology.</t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J66" s="2" t="n"/>
@@ -4480,7 +4480,7 @@
       <c r="L66" s="2" t="n"/>
       <c r="M66" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N66" s="2" t="n"/>
@@ -4488,7 +4488,7 @@
       <c r="P66" s="2" t="n"/>
       <c r="Q66" s="2" t="inlineStr">
         <is>
-          <t>Published</t>
+          <t>An attribute of a process.</t>
         </is>
       </c>
       <c r="R66" s="2" t="n"/>
@@ -4516,12 +4516,12 @@
           <t>process context</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
+      <c r="D67" t="inlineStr">
         <is>
           <t>entity</t>
         </is>
       </c>
-      <c r="Q67" t="inlineStr">
+      <c r="M67" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -4546,32 +4546,32 @@
           <t>A population that is studied in a research study.</t>
         </is>
       </c>
-      <c r="D68" s="2" t="n"/>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>human population</t>
+        </is>
+      </c>
       <c r="E68" s="2" t="n"/>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>human population</t>
-        </is>
-      </c>
+      <c r="F68" s="2" t="n"/>
       <c r="G68" s="2" t="n"/>
       <c r="H68" s="2" t="n"/>
-      <c r="I68" s="2" t="n"/>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="J68" s="2" t="n"/>
       <c r="K68" s="2" t="n"/>
       <c r="L68" s="2" t="n"/>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Published</t>
         </is>
       </c>
       <c r="N68" s="2" t="n"/>
       <c r="O68" s="2" t="n"/>
       <c r="P68" s="2" t="n"/>
-      <c r="Q68" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="Q68" s="2" t="n"/>
       <c r="R68" s="2" t="n"/>
       <c r="S68" s="2" t="n"/>
       <c r="T68" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Edit BCIO_Upper_Defs.xlsx: update 1, add 1
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
@@ -30,7 +30,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +47,11 @@
         <fgColor rgb="002f4f4f"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ffffff"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -60,11 +65,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V68"/>
+  <dimension ref="A1:V69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,17 +517,17 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>Logical definition</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Informal definition</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
           <t>To be reviewed by</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Informal definition</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Logical definition</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
@@ -1653,13 +1659,13 @@
       </c>
       <c r="N18" s="2" t="n"/>
       <c r="O18" s="2" t="n"/>
-      <c r="P18" s="2" t="n"/>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>'individual human behaviour' AND 'intervention outcome'</t>
+        </is>
+      </c>
       <c r="Q18" s="2" t="n"/>
-      <c r="R18" s="2" t="inlineStr">
-        <is>
-          <t>'individual human behaviour' AND 'intervention outcome'</t>
-        </is>
-      </c>
+      <c r="R18" s="2" t="n"/>
       <c r="S18" s="2" t="n"/>
       <c r="T18" s="2" t="inlineStr">
         <is>
@@ -2048,32 +2054,32 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>BCIO:009000</t>
+          <t>BCIO:014000</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention schedule of delivery</t>
+          <t>behaviour change intervention setting</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>A BCI attribute that involves its temporal organisation.</t>
+          <t xml:space="preserve">An aggregate of entities that form the environment in which a BCI is provided. </t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>BCI attribute</t>
+          <t>object aggregate</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>BCI schedule of delivery</t>
+          <t>BCI setting</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Includes the start and end of the BCI and its parts.</t>
+          <t>Includes as parts social setting and physical setting.</t>
         </is>
       </c>
       <c r="G25" s="2" t="n"/>
@@ -2112,34 +2118,30 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>BCIO:014000</t>
+          <t>BCIO:029000</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention setting</t>
+          <t>behaviour change intervention social setting</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">An aggregate of entities that form the environment in which a BCI is provided. </t>
+          <t>An aggregate of people with whom a BCI population interacts.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>object aggregate</t>
+          <t>human population</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>BCI setting</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Includes as parts social setting and physical setting.</t>
-        </is>
-      </c>
+          <t>BCI social setting</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="n"/>
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="2" t="inlineStr">
@@ -2176,30 +2178,34 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>BCIO:029000</t>
+          <t>BCIO:010000</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention social setting</t>
+          <t>behaviour change intervention source</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>An aggregate of people with whom a BCI population interacts.</t>
+          <t>A role played by a person, population or organisation that provides a BCI.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>human population</t>
+          <t>role</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>BCI social setting</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="n"/>
+          <t>BCI source</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>This includes individual people, groups of people, and organisations.</t>
+        </is>
+      </c>
       <c r="G27" s="2" t="n"/>
       <c r="H27" s="2" t="n"/>
       <c r="I27" s="2" t="inlineStr">
@@ -2236,17 +2242,17 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>BCIO:010000</t>
+          <t>BCIO:030000</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention source</t>
+          <t>behaviour change intervention study investigator</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>A role played by a person, population or organisation that provides a BCI.</t>
+          <t>A role played by a person that contributes substantively to production or reporting of a BCI evaluation study.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -2256,12 +2262,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>BCI source</t>
+          <t>BCI study investigator</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>This includes individual people, groups of people, and organisations.</t>
+          <t xml:space="preserve">What counts as substantively is subject to judgement. The level and nature of the contribution can be defined using the CReDiT taxonomy (https://casrai.org/credit/). </t>
         </is>
       </c>
       <c r="G28" s="2" t="n"/>
@@ -2300,34 +2306,30 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>BCIO:030000</t>
+          <t>BCIO:031000</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention study investigator</t>
+          <t>behaviour change intervention study sample</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>A role played by a person that contributes substantively to production or reporting of a BCI evaluation study.</t>
+          <t>A research study sample whose behaviour is studied in a BCI evaluation study.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>role</t>
+          <t>research study participants</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>BCI study investigator</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">What counts as substantively is subject to judgement. The level and nature of the contribution can be defined using the CReDiT taxonomy (https://casrai.org/credit/). </t>
-        </is>
-      </c>
+          <t>BCI study sample</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="n"/>
       <c r="H29" s="2" t="n"/>
       <c r="I29" s="2" t="inlineStr">
@@ -2351,7 +2353,7 @@
       <c r="S29" s="2" t="n"/>
       <c r="T29" s="2" t="inlineStr">
         <is>
-          <t>JH; RW</t>
+          <t>JH; RW; PS</t>
         </is>
       </c>
       <c r="U29" s="2" t="inlineStr">
@@ -2364,30 +2366,34 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>BCIO:031000</t>
+          <t>BCIO:044000</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention study sample</t>
+          <t>behaviour change intervention style of delivery</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>A research study sample whose behaviour is studied in a BCI evaluation study.</t>
+          <t>A communication style that is an attribute of a BCI content communication process.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>research study participants</t>
+          <t>communication style</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>BCI study sample</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="n"/>
+          <t>BCI style of delivery</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>An example is cold and distant vs. warm and accepting.</t>
+        </is>
+      </c>
       <c r="G30" s="2" t="n"/>
       <c r="H30" s="2" t="n"/>
       <c r="I30" s="2" t="inlineStr">
@@ -2411,7 +2417,7 @@
       <c r="S30" s="2" t="n"/>
       <c r="T30" s="2" t="inlineStr">
         <is>
-          <t>JH; RW; PS</t>
+          <t>JH; RW</t>
         </is>
       </c>
       <c r="U30" s="2" t="inlineStr">
@@ -2424,35 +2430,39 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>BCIO:044000</t>
+          <t>BCIO:032000</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention style of delivery</t>
+          <t>behaviour change intervention tailoring</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>A communication style that is an attribute of a BCI content communication process.</t>
+          <t>A BCI attribute in which the content or delivery of a BCI for some member of the BCI population varies according to their characteristics or setting.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>communication style</t>
+          <t>BCI attribute</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>BCI style of delivery</t>
+          <t>BCI tailoring</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>An example is cold and distant vs. warm and accepting.</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="n"/>
+          <t>Tailoring the dose of pharmacotherapy for smoking cessation to the prior level of nicotine dependence of the smoker (static) or to the smokers' current strength of urges to smoke during a quit attempt (dynamic).</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Tailoring can be static (i.e., conducted before intervention delivery in a case case), or dynamic (i.e., conducted one or more times after the intervention has started in a given case based on population or setting characteristics present at that time. Population and setting characteristics include the historical factors such as prior exposure to the intervention.</t>
+        </is>
+      </c>
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="2" t="inlineStr">
         <is>
@@ -2470,7 +2480,11 @@
       <c r="N31" s="2" t="n"/>
       <c r="O31" s="2" t="n"/>
       <c r="P31" s="2" t="n"/>
-      <c r="Q31" s="2" t="n"/>
+      <c r="Q31" s="2" t="inlineStr">
+        <is>
+          <t>An attribute of a behaviour change intervention (BCI) or a BCI component whereby its content or delivery is varied according to characteristics of members of the target population or setting.</t>
+        </is>
+      </c>
       <c r="R31" s="2" t="n"/>
       <c r="S31" s="2" t="n"/>
       <c r="T31" s="2" t="inlineStr">
@@ -2488,39 +2502,31 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>BCIO:032000</t>
+          <t>BCIO:047000</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention tailoring</t>
+          <t xml:space="preserve">behaviour change intervention temporal context </t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>A BCI attribute in which the content or delivery of a BCI for some member of the BCI population varies according to their characteristics or setting.</t>
+          <t>The intervention temporal context where the process is the behaviour change intervention</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>BCI attribute</t>
+          <t>intervention temporal context</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>BCI tailoring</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Tailoring the dose of pharmacotherapy for smoking cessation to the prior level of nicotine dependence of the smoker (static) or to the smokers' current strength of urges to smoke during a quit attempt (dynamic).</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>Tailoring can be static (i.e., conducted before intervention delivery in a case case), or dynamic (i.e., conducted one or more times after the intervention has started in a given case based on population or setting characteristics present at that time. Population and setting characteristics include the historical factors such as prior exposure to the intervention.</t>
-        </is>
-      </c>
+          <t>BCI temporal context</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
       <c r="H32" s="2" t="n"/>
       <c r="I32" s="2" t="inlineStr">
         <is>
@@ -2538,11 +2544,7 @@
       <c r="N32" s="2" t="n"/>
       <c r="O32" s="2" t="n"/>
       <c r="P32" s="2" t="n"/>
-      <c r="Q32" s="2" t="inlineStr">
-        <is>
-          <t>An attribute of a behaviour change intervention (BCI) or a BCI component whereby its content or delivery is varied according to characteristics of members of the target population or setting.</t>
-        </is>
-      </c>
+      <c r="Q32" s="2" t="n"/>
       <c r="R32" s="2" t="n"/>
       <c r="S32" s="2" t="n"/>
       <c r="T32" s="2" t="inlineStr">
@@ -2560,27 +2562,27 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>BCIO:047000</t>
+          <t>BCIO:047001</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">behaviour change intervention temporal context </t>
+          <t>behaviour change intervention temporal context event</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>The intervention temporal context where the process is the behaviour change intervention</t>
+          <t xml:space="preserve">An event which occurs during a behaviour change intervention temporal context. </t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal context</t>
+          <t>behaviour change intervention temporal context</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal context</t>
+          <t>BCI temporal context event</t>
         </is>
       </c>
       <c r="F33" s="2" t="n"/>
@@ -2620,27 +2622,27 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>BCIO:047001</t>
+          <t>BCIO:033000</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention temporal context event</t>
+          <t>behaviour change technique</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">An event which occurs during a behaviour change intervention temporal context. </t>
+          <t>A &lt;planned process&gt; that is the smallest part of BCI content that is observable, replicable and on its own has the potential to bring about behaviour change.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention temporal context</t>
+          <t>planned process</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal context event</t>
+          <t>BCT</t>
         </is>
       </c>
       <c r="F34" s="2" t="n"/>
@@ -2667,7 +2669,7 @@
       <c r="S34" s="2" t="n"/>
       <c r="T34" s="2" t="inlineStr">
         <is>
-          <t>JH; RW</t>
+          <t>JH; RW; PS</t>
         </is>
       </c>
       <c r="U34" s="2" t="inlineStr">
@@ -2680,29 +2682,25 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>BCIO:033000</t>
+          <t>BCIO:044003</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>behaviour change technique</t>
+          <t>communication process attribute</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>A &lt;planned process&gt; that is the smallest part of BCI content that is observable, replicable and on its own has the potential to bring about behaviour change.</t>
+          <t>An attribute of a communication process.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>planned process</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>BCT</t>
-        </is>
-      </c>
+          <t>process attribute</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n"/>
       <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="n"/>
       <c r="H35" s="2" t="n"/>
@@ -2727,7 +2725,7 @@
       <c r="S35" s="2" t="n"/>
       <c r="T35" s="2" t="inlineStr">
         <is>
-          <t>JH; RW; PS</t>
+          <t>JH; PS</t>
         </is>
       </c>
       <c r="U35" s="2" t="inlineStr">
@@ -2740,22 +2738,22 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>BCIO:044003</t>
+          <t>BCIO:044004</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
+          <t>communication style</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>A particular manner of communicating aimed at inducing or avoiding certain kinds of responses in others, or demonstrating certain characteristics of the initiator.</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
           <t>communication process attribute</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>An attribute of a communication process.</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>process attribute</t>
         </is>
       </c>
       <c r="E36" s="2" t="n"/>
@@ -2783,7 +2781,7 @@
       <c r="S36" s="2" t="n"/>
       <c r="T36" s="2" t="inlineStr">
         <is>
-          <t>JH; PS</t>
+          <t>JH</t>
         </is>
       </c>
       <c r="U36" s="2" t="inlineStr">
@@ -2794,87 +2792,91 @@
       <c r="V36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:044004</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>communication style</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>A particular manner of communicating aimed at inducing or avoiding certain kinds of responses in others, or demonstrating certain characteristics of the initiator.</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>communication process attribute</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="n"/>
-      <c r="G37" s="2" t="n"/>
-      <c r="H37" s="2" t="n"/>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="n"/>
-      <c r="K37" s="2" t="n"/>
-      <c r="L37" s="2" t="n"/>
-      <c r="M37" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="N37" s="2" t="n"/>
-      <c r="O37" s="2" t="n"/>
-      <c r="P37" s="2" t="n"/>
-      <c r="Q37" s="2" t="n"/>
-      <c r="R37" s="2" t="n"/>
-      <c r="S37" s="2" t="n"/>
-      <c r="T37" s="2" t="inlineStr">
-        <is>
-          <t>JH</t>
-        </is>
-      </c>
-      <c r="U37" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V37" s="2" t="n"/>
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:050462</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>high cognitive exertion expended on a behaviour</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Cognitive exertion expended on a behaviour that is high.</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>cognitive exertion expended on a behaviour</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="n"/>
+      <c r="F37" s="3" t="n"/>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>High cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="n"/>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="J37" s="3" t="n"/>
+      <c r="K37" s="3" t="n"/>
+      <c r="L37" s="3" t="n"/>
+      <c r="M37" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="N37" s="3" t="n"/>
+      <c r="O37" s="3" t="n"/>
+      <c r="P37" s="3" t="n"/>
+      <c r="Q37" s="3" t="n"/>
+      <c r="R37" s="3" t="n"/>
+      <c r="S37" s="3" t="n"/>
+      <c r="T37" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U37" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="V37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050462</t>
+          <t>BCIO:050463</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>high cognitive exertion expended on a behaviour</t>
+          <t>high emotional management  exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Cognitive exertion expended on a behaviour that is high.</t>
+          <t>Emotional management exertion expended on a behaviour that is high.</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>cognitive exertion expended on a behaviour</t>
+          <t>emotional management exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E38" s="3" t="n"/>
       <c r="F38" s="3" t="n"/>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>High cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
+          <t>High emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="H38" s="3" t="n"/>
@@ -2912,29 +2914,29 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050463</t>
+          <t>BCIO:050464</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>high emotional management  exertion expended on a behaviour</t>
+          <t>high mental exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Emotional management exertion expended on a behaviour that is high.</t>
+          <t>Mental exertion expended on a behaviour that is high.</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>emotional management exertion expended on a behaviour</t>
+          <t>mental exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E39" s="3" t="n"/>
       <c r="F39" s="3" t="n"/>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>High emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
+          <t>High mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="H39" s="3" t="n"/>
@@ -2972,29 +2974,29 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050464</t>
+          <t>BCIO:050465</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>high mental exertion expended on a behaviour</t>
+          <t>high physical exertion expended on behaviour</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Mental exertion expended on a behaviour that is high.</t>
+          <t>Physical exertion expended on a behaviour that is high</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>mental exertion expended on a behaviour</t>
+          <t>physical exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E40" s="3" t="n"/>
       <c r="F40" s="3" t="n"/>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>High mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
+          <t>High physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="H40" s="3" t="n"/>
@@ -3032,35 +3034,31 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050465</t>
+          <t>BCIO:042000</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>high physical exertion expended on behaviour</t>
+          <t>human behaviour</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Physical exertion expended on a behaviour that is high</t>
+          <t>A process that is an individual human behaviour or a population behaviour.</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>physical exertion expended on a behaviour</t>
+          <t>process</t>
         </is>
       </c>
       <c r="E41" s="3" t="n"/>
       <c r="F41" s="3" t="n"/>
-      <c r="G41" s="3" t="inlineStr">
-        <is>
-          <t>High physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="G41" s="3" t="n"/>
       <c r="H41" s="3" t="n"/>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="J41" s="3" t="n"/>
@@ -3073,101 +3071,101 @@
       </c>
       <c r="N41" s="3" t="n"/>
       <c r="O41" s="3" t="n"/>
-      <c r="P41" s="3" t="n"/>
+      <c r="P41" s="3" t="inlineStr">
+        <is>
+          <t>"individual human behaviour" OR "population behaviour"</t>
+        </is>
+      </c>
       <c r="Q41" s="3" t="n"/>
       <c r="R41" s="3" t="n"/>
       <c r="S41" s="3" t="n"/>
       <c r="T41" s="3" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>BG; PS</t>
         </is>
       </c>
       <c r="U41" s="3" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>0</t>
         </is>
       </c>
       <c r="V41" s="3" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:042000</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>human behaviour</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>A process that is an individual human behaviour or a population behaviour.</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="n"/>
-      <c r="F42" s="3" t="n"/>
-      <c r="G42" s="3" t="n"/>
-      <c r="H42" s="3" t="n"/>
-      <c r="I42" s="3" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
-      <c r="J42" s="3" t="n"/>
-      <c r="K42" s="3" t="n"/>
-      <c r="L42" s="3" t="n"/>
-      <c r="M42" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="N42" s="3" t="n"/>
-      <c r="O42" s="3" t="n"/>
-      <c r="P42" s="3" t="n"/>
-      <c r="Q42" s="3" t="n"/>
-      <c r="R42" s="3" t="inlineStr">
-        <is>
-          <t>"individual human behaviour" OR "population behaviour"</t>
-        </is>
-      </c>
-      <c r="S42" s="3" t="n"/>
-      <c r="T42" s="3" t="inlineStr">
-        <is>
-          <t>BG; PS</t>
-        </is>
-      </c>
-      <c r="U42" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V42" s="3" t="n"/>
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:041000</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>human population</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>An object aggregate that consists of two or more people.</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>object aggregate</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="2" t="n"/>
+      <c r="G42" s="2" t="n"/>
+      <c r="H42" s="2" t="n"/>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="n"/>
+      <c r="K42" s="2" t="n"/>
+      <c r="L42" s="2" t="n"/>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="n"/>
+      <c r="O42" s="2" t="n"/>
+      <c r="P42" s="2" t="n"/>
+      <c r="Q42" s="2" t="n"/>
+      <c r="R42" s="2" t="n"/>
+      <c r="S42" s="2" t="n"/>
+      <c r="T42" s="2" t="inlineStr">
+        <is>
+          <t>JH; AW</t>
+        </is>
+      </c>
+      <c r="U42" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>BCIO:041000</t>
+          <t>BCIO:040000</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>human population</t>
+          <t>individual human activity</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>An object aggregate that consists of two or more people.</t>
+          <t>A process that is produced by a person.</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>object aggregate</t>
+          <t>process</t>
         </is>
       </c>
       <c r="E43" s="2" t="n"/>
@@ -3195,7 +3193,7 @@
       <c r="S43" s="2" t="n"/>
       <c r="T43" s="2" t="inlineStr">
         <is>
-          <t>JH; AW</t>
+          <t>JH</t>
         </is>
       </c>
       <c r="U43" s="2" t="inlineStr">
@@ -3208,26 +3206,34 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>BCIO:040000</t>
+          <t>BCIO:036000</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>individual human activity</t>
+          <t>individual human behaviour</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>A process that is produced by a person.</t>
+          <t xml:space="preserve">A bodily process of a human that involves co-ordinated contraction of striated muscles controlled by the brain. </t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="2" t="n"/>
+          <t>bodily process</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>human behaviour</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Also referred to in definitions as human behaviour or just behaviour.</t>
+        </is>
+      </c>
       <c r="G44" s="2" t="n"/>
       <c r="H44" s="2" t="n"/>
       <c r="I44" s="2" t="inlineStr">
@@ -3264,32 +3270,28 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>BCIO:036000</t>
+          <t>BCIO:037000</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>individual human behaviour</t>
+          <t>intervention</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A bodily process of a human that involves co-ordinated contraction of striated muscles controlled by the brain. </t>
+          <t>A planned process that has the aim of influencing an outcome.</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>bodily process</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>human behaviour</t>
-        </is>
-      </c>
+          <t>planned process</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="n"/>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Also referred to in definitions as human behaviour or just behaviour.</t>
+          <t>Examples of interventions are putting health warnings on cigarette packets, providing free stop smoking services and banning smoking in public places.</t>
         </is>
       </c>
       <c r="G45" s="2" t="n"/>
@@ -3315,7 +3317,7 @@
       <c r="S45" s="2" t="n"/>
       <c r="T45" s="2" t="inlineStr">
         <is>
-          <t>JH</t>
+          <t>JH; RW</t>
         </is>
       </c>
       <c r="U45" s="2" t="inlineStr">
@@ -3326,64 +3328,50 @@
       <c r="V45" s="2" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:037000</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>intervention</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>A planned process that has the aim of influencing an outcome.</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>planned process</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="n"/>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>Examples of interventions are putting health warnings on cigarette packets, providing free stop smoking services and banning smoking in public places.</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="n"/>
-      <c r="H46" s="2" t="n"/>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
-      <c r="J46" s="2" t="n"/>
-      <c r="K46" s="2" t="n"/>
-      <c r="L46" s="2" t="n"/>
-      <c r="M46" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="N46" s="2" t="n"/>
-      <c r="O46" s="2" t="n"/>
-      <c r="P46" s="2" t="n"/>
-      <c r="Q46" s="2" t="n"/>
-      <c r="R46" s="2" t="n"/>
-      <c r="S46" s="2" t="n"/>
-      <c r="T46" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
-      <c r="U46" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V46" s="2" t="n"/>
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:051010</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>intervention attribute</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>A &lt;process attribute&gt; whose bearer is an intervention.</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>process attribute</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr"/>
+      <c r="F46" s="4" t="inlineStr"/>
+      <c r="G46" s="4" t="inlineStr"/>
+      <c r="H46" s="4" t="inlineStr"/>
+      <c r="I46" s="4" t="inlineStr"/>
+      <c r="J46" s="4" t="inlineStr"/>
+      <c r="K46" s="4" t="inlineStr"/>
+      <c r="L46" s="4" t="inlineStr"/>
+      <c r="M46" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="N46" s="4" t="inlineStr"/>
+      <c r="O46" s="4" t="inlineStr"/>
+      <c r="P46" s="4" t="inlineStr"/>
+      <c r="Q46" s="4" t="inlineStr"/>
+      <c r="R46" s="4" t="inlineStr"/>
+      <c r="S46" s="4" t="inlineStr"/>
+      <c r="T46" s="4" t="inlineStr"/>
+      <c r="U46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V46" s="4" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3751,116 +3739,124 @@
       <c r="V53" s="2" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:009000</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>intervention schedule of delivery</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>An intervention attribute that is its temporal organisation.</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>intervention attribute</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>BCI schedule of delivery</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Includes the start and end of the BCI and its parts.</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="n"/>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="n"/>
+      <c r="K54" s="2" t="n"/>
+      <c r="L54" s="2" t="n"/>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="n"/>
+      <c r="O54" s="2" t="n"/>
+      <c r="P54" s="2" t="n"/>
+      <c r="Q54" s="2" t="n"/>
+      <c r="R54" s="2" t="n"/>
+      <c r="S54" s="2" t="n"/>
+      <c r="T54" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
+      <c r="U54" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
         <is>
           <t>GMHO:0000254</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>intervention temporal context</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D55" t="inlineStr">
         <is>
           <t>intervention context</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr">
+      <c r="M55" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="U54" t="n">
+      <c r="U55" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:050466</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="inlineStr">
-        <is>
-          <t>low cognitive exertion expended on a behaviour</t>
-        </is>
-      </c>
-      <c r="C55" s="3" t="inlineStr">
-        <is>
-          <t>Cognitive exertion expended on a behaviour that is low.</t>
-        </is>
-      </c>
-      <c r="D55" s="3" t="inlineStr">
-        <is>
-          <t>cognitive exertion expended on a behaviour</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="n"/>
-      <c r="F55" s="3" t="n"/>
-      <c r="G55" s="3" t="inlineStr">
-        <is>
-          <t>Low cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
-        </is>
-      </c>
-      <c r="H55" s="3" t="n"/>
-      <c r="I55" s="3" t="inlineStr">
-        <is>
-          <t>behaviour</t>
-        </is>
-      </c>
-      <c r="J55" s="3" t="n"/>
-      <c r="K55" s="3" t="n"/>
-      <c r="L55" s="3" t="n"/>
-      <c r="M55" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="N55" s="3" t="n"/>
-      <c r="O55" s="3" t="n"/>
-      <c r="P55" s="3" t="n"/>
-      <c r="Q55" s="3" t="n"/>
-      <c r="R55" s="3" t="n"/>
-      <c r="S55" s="3" t="n"/>
-      <c r="T55" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="U55" s="3" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="V55" s="3" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050467</t>
+          <t>BCIO:050466</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>low emotional management exertion expended on a behaviour</t>
+          <t>low cognitive exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Emotional management exertion expended on a behaviour that is low.</t>
+          <t>Cognitive exertion expended on a behaviour that is low.</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>emotional management exertion expended on a behaviour</t>
+          <t>cognitive exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E56" s="3" t="n"/>
       <c r="F56" s="3" t="n"/>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>Low emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
+          <t>Low cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="H56" s="3" t="n"/>
@@ -3898,29 +3894,29 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050468</t>
+          <t>BCIO:050467</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>low mental exertion expended on a behaviour</t>
+          <t>low emotional management exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Mental exertion expended on a behaviour that is low.</t>
+          <t>Emotional management exertion expended on a behaviour that is low.</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>mental exertion expended on a behaviour</t>
+          <t>emotional management exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E57" s="3" t="n"/>
       <c r="F57" s="3" t="n"/>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>Low mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
+          <t>Low emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="H57" s="3" t="n"/>
@@ -3958,29 +3954,29 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050469</t>
+          <t>BCIO:050468</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>low physical exertion expended on behaviour</t>
+          <t>low mental exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Physical exertion expended on a behaviour that is low.</t>
+          <t>Mental exertion expended on a behaviour that is low.</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>physical exertion expended on a behaviour</t>
+          <t>mental exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E58" s="3" t="n"/>
       <c r="F58" s="3" t="n"/>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means </t>
+          <t>Low mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="H58" s="3" t="n"/>
@@ -4018,29 +4014,29 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050470</t>
+          <t>BCIO:050469</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>moderate cognitive exertion expended on a behaviour</t>
+          <t>low physical exertion expended on behaviour</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Cognitive exertion expended on a behaviour that is medium.</t>
+          <t>Physical exertion expended on a behaviour that is low.</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>cognitive exertion expended on a behaviour</t>
+          <t>physical exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E59" s="3" t="n"/>
       <c r="F59" s="3" t="n"/>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>Moderate cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
+          <t xml:space="preserve">Low physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means </t>
         </is>
       </c>
       <c r="H59" s="3" t="n"/>
@@ -4078,29 +4074,29 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050471</t>
+          <t>BCIO:050470</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>moderate emotional management exertion expended on a behaviour</t>
+          <t>moderate cognitive exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Emotional management exertion expended on a behaviour that is medium.</t>
+          <t>Cognitive exertion expended on a behaviour that is medium.</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>emotional management exertion expended on a behaviour</t>
+          <t>cognitive exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E60" s="3" t="n"/>
       <c r="F60" s="3" t="n"/>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>Moderate emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
+          <t>Moderate cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="H60" s="3" t="n"/>
@@ -4138,29 +4134,29 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050472</t>
+          <t>BCIO:050471</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>moderate mental exertion expended on a behaviour</t>
+          <t>moderate emotional management exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Mental exertion expended on a behaviour that is medium.</t>
+          <t>Emotional management exertion expended on a behaviour that is medium.</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>mental exertion expended on a behaviour</t>
+          <t>emotional management exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E61" s="3" t="n"/>
       <c r="F61" s="3" t="n"/>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>Moderate mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
+          <t>Moderate emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="H61" s="3" t="n"/>
@@ -4198,29 +4194,29 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050473</t>
+          <t>BCIO:050472</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>moderate physical exertion expended on behaviour</t>
+          <t>moderate mental exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Physical exertion expended on a behaviour that is medium.</t>
+          <t>Mental exertion expended on a behaviour that is medium.</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>physical exertion expended on a behaviour</t>
+          <t>mental exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E62" s="3" t="n"/>
       <c r="F62" s="3" t="n"/>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>Moderate physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
+          <t>Moderate mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="H62" s="3" t="n"/>
@@ -4256,98 +4252,102 @@
       <c r="V62" s="3" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:013000</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>participant engagement with behaviour change intervention</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>Participant engagement with intervention, where the intervention focuses on changing behaviour.</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>participant engagement with intervention</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>BCI engagement</t>
-        </is>
-      </c>
-      <c r="F63" s="2" t="inlineStr">
-        <is>
-          <t>Includes mental activities and behaviours.</t>
-        </is>
-      </c>
-      <c r="G63" s="2" t="n"/>
-      <c r="H63" s="2" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="I63" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
-      <c r="J63" s="2" t="n"/>
-      <c r="K63" s="2" t="n"/>
-      <c r="L63" s="2" t="n"/>
-      <c r="M63" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="N63" s="2" t="n"/>
-      <c r="O63" s="2" t="n"/>
-      <c r="P63" s="2" t="n"/>
-      <c r="Q63" s="2" t="n"/>
-      <c r="R63" s="2" t="n"/>
-      <c r="S63" s="2" t="n"/>
-      <c r="T63" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW; PS</t>
-        </is>
-      </c>
-      <c r="U63" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V63" s="2" t="n"/>
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:050473</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>moderate physical exertion expended on behaviour</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Physical exertion expended on a behaviour that is medium.</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>physical exertion expended on a behaviour</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="n"/>
+      <c r="F63" s="3" t="n"/>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>Moderate physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="n"/>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="n"/>
+      <c r="K63" s="3" t="n"/>
+      <c r="L63" s="3" t="n"/>
+      <c r="M63" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="N63" s="3" t="n"/>
+      <c r="O63" s="3" t="n"/>
+      <c r="P63" s="3" t="n"/>
+      <c r="Q63" s="3" t="n"/>
+      <c r="R63" s="3" t="n"/>
+      <c r="S63" s="3" t="n"/>
+      <c r="T63" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U63" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="V63" s="3" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050916</t>
+          <t>BCIO:013000</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
+          <t>participant engagement with behaviour change intervention</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Participant engagement with intervention, where the intervention focuses on changing behaviour.</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
           <t>participant engagement with intervention</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>An individual human activity of an intervention participant within one or more parts of the intervention.</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>individual human activity</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="n"/>
-      <c r="F64" s="2" t="n"/>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>BCI engagement</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Includes mental activities and behaviours.</t>
+        </is>
+      </c>
       <c r="G64" s="2" t="n"/>
-      <c r="H64" s="2" t="n"/>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
           <t>Upper level</t>
@@ -4364,49 +4364,43 @@
       <c r="N64" s="2" t="n"/>
       <c r="O64" s="2" t="n"/>
       <c r="P64" s="2" t="n"/>
-      <c r="Q64" s="2" t="inlineStr">
-        <is>
-          <t>The extend to someone interacts with an intervention, including their cognitive, emotional and behavioural response (e.g., attending intervention session) to the intervention itself.</t>
-        </is>
-      </c>
+      <c r="Q64" s="2" t="n"/>
       <c r="R64" s="2" t="n"/>
       <c r="S64" s="2" t="n"/>
       <c r="T64" s="2" t="inlineStr">
         <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="U64" s="2" t="n">
-        <v>0</v>
+          <t>JH; RW; PS</t>
+        </is>
+      </c>
+      <c r="U64" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="V64" s="2" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>BCIO:034000</t>
+          <t>BCIO:050916</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>population behaviour</t>
+          <t>participant engagement with intervention</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>An aggregate of individual human behaviours of members of a population.</t>
+          <t>An individual human activity of an intervention participant within one or more parts of the intervention.</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t>human behaviour</t>
-        </is>
-      </c>
+          <t>individual human activity</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="n"/>
       <c r="F65" s="2" t="n"/>
       <c r="G65" s="2" t="n"/>
       <c r="H65" s="2" t="n"/>
@@ -4426,48 +4420,50 @@
       <c r="N65" s="2" t="n"/>
       <c r="O65" s="2" t="n"/>
       <c r="P65" s="2" t="n"/>
-      <c r="Q65" s="2" t="n"/>
+      <c r="Q65" s="2" t="inlineStr">
+        <is>
+          <t>The extend to someone interacts with an intervention, including their cognitive, emotional and behavioural response (e.g., attending intervention session) to the intervention itself.</t>
+        </is>
+      </c>
       <c r="R65" s="2" t="n"/>
       <c r="S65" s="2" t="n"/>
       <c r="T65" s="2" t="inlineStr">
         <is>
-          <t>JH</t>
-        </is>
-      </c>
-      <c r="U65" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U65" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="V65" s="2" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>BCIO:043000</t>
+          <t>BCIO:034000</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>process attribute</t>
+          <t>population behaviour</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>A process profile that is an attribute of a process.</t>
+          <t>An aggregate of individual human behaviours of members of a population.</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>process profile</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="n"/>
-      <c r="F66" s="2" t="inlineStr">
-        <is>
-          <t>This is intended to provide a user-friendly way of representing the way in which processes are manifest. This is somewhat similar to, but not the same as, the class 'specifically dependent continuant' in Basic Formal Ontology which provides a way of representing features of material entities such as age and size. It is formally equivalent to process profile in Basic Formal Ontology.</t>
-        </is>
-      </c>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>human behaviour</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="n"/>
       <c r="G66" s="2" t="n"/>
       <c r="H66" s="2" t="n"/>
       <c r="I66" s="2" t="inlineStr">
@@ -4486,11 +4482,7 @@
       <c r="N66" s="2" t="n"/>
       <c r="O66" s="2" t="n"/>
       <c r="P66" s="2" t="n"/>
-      <c r="Q66" s="2" t="inlineStr">
-        <is>
-          <t>An attribute of a process.</t>
-        </is>
-      </c>
+      <c r="Q66" s="2" t="n"/>
       <c r="R66" s="2" t="n"/>
       <c r="S66" s="2" t="n"/>
       <c r="T66" s="2" t="inlineStr">
@@ -4506,85 +4498,149 @@
       <c r="V66" s="2" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:043000</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>process attribute</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>A process profile that is an attribute of a process.</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>process profile</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="n"/>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>This is intended to provide a user-friendly way of representing the way in which processes are manifest. This is somewhat similar to, but not the same as, the class 'specifically dependent continuant' in Basic Formal Ontology which provides a way of representing features of material entities such as age and size. It is formally equivalent to process profile in Basic Formal Ontology.</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="n"/>
+      <c r="H67" s="2" t="n"/>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="n"/>
+      <c r="K67" s="2" t="n"/>
+      <c r="L67" s="2" t="n"/>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="n"/>
+      <c r="O67" s="2" t="n"/>
+      <c r="P67" s="2" t="n"/>
+      <c r="Q67" s="2" t="inlineStr">
+        <is>
+          <t>An attribute of a process.</t>
+        </is>
+      </c>
+      <c r="R67" s="2" t="n"/>
+      <c r="S67" s="2" t="n"/>
+      <c r="T67" s="2" t="inlineStr">
+        <is>
+          <t>JH</t>
+        </is>
+      </c>
+      <c r="U67" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V67" s="2" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
         <is>
           <t>GMHO:0000268</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B68" t="inlineStr">
         <is>
           <t>process context</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="D68" t="inlineStr">
         <is>
           <t>entity</t>
         </is>
       </c>
-      <c r="M67" t="inlineStr">
+      <c r="M68" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="U67" t="n">
+      <c r="U68" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>BCIO:050551</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>research study participants</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
         <is>
           <t>A population that is studied in a research study.</t>
         </is>
       </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>human population</t>
         </is>
       </c>
-      <c r="E68" s="2" t="n"/>
-      <c r="F68" s="2" t="n"/>
-      <c r="G68" s="2" t="n"/>
-      <c r="H68" s="2" t="n"/>
-      <c r="I68" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
-      <c r="J68" s="2" t="n"/>
-      <c r="K68" s="2" t="n"/>
-      <c r="L68" s="2" t="n"/>
-      <c r="M68" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="N68" s="2" t="n"/>
-      <c r="O68" s="2" t="n"/>
-      <c r="P68" s="2" t="n"/>
-      <c r="Q68" s="2" t="n"/>
-      <c r="R68" s="2" t="n"/>
-      <c r="S68" s="2" t="n"/>
-      <c r="T68" s="2" t="inlineStr">
+      <c r="E69" s="2" t="n"/>
+      <c r="F69" s="2" t="n"/>
+      <c r="G69" s="2" t="n"/>
+      <c r="H69" s="2" t="n"/>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="n"/>
+      <c r="K69" s="2" t="n"/>
+      <c r="L69" s="2" t="n"/>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="n"/>
+      <c r="O69" s="2" t="n"/>
+      <c r="P69" s="2" t="n"/>
+      <c r="Q69" s="2" t="n"/>
+      <c r="R69" s="2" t="n"/>
+      <c r="S69" s="2" t="n"/>
+      <c r="T69" s="2" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="U68" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V68" s="2" t="n"/>
+      <c r="U69" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V69" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update behaviour change intervention study investigator role in BCIO_Upper_Defs.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
@@ -467,77 +467,77 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Logical definition</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Examples</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>BFO entity</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Comment</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>BFO entity</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'has process part'</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>REL 'realises'</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Sub-ontology</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'has process part'</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>REL 'realises'</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Curator note</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Definition source</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Cross reference</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Curator</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Informal definition</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Curation status</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Definition source</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Cross reference</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Logical definition</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Informal definition</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>To be reviewed by</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Reviewer query</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Curator</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
@@ -584,34 +584,34 @@
           <t>process</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="n"/>
       <c r="N2" s="2" t="n"/>
       <c r="O2" s="2" t="n"/>
-      <c r="P2" s="2" t="n"/>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>An attribute of a behaviour change intervention.</t>
         </is>
       </c>
-      <c r="R2" s="2" t="n"/>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="inlineStr">
-        <is>
-          <t>RW</t>
-        </is>
-      </c>
+      <c r="T2" s="2" t="n"/>
       <c r="U2" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -648,34 +648,34 @@
           <t>information content entity</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I3" s="2" t="n"/>
       <c r="J3" s="2" t="n"/>
       <c r="K3" s="2" t="n"/>
-      <c r="L3" s="2" t="n"/>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="n"/>
       <c r="N3" s="2" t="n"/>
       <c r="O3" s="2" t="n"/>
-      <c r="P3" s="2" t="n"/>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>RW; JH</t>
+        </is>
+      </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
           <t>A criterion for selecting people for a BCI population.</t>
         </is>
       </c>
-      <c r="R3" s="2" t="n"/>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S3" s="2" t="n"/>
-      <c r="T3" s="2" t="inlineStr">
-        <is>
-          <t>RW; JH</t>
-        </is>
-      </c>
+      <c r="T3" s="2" t="n"/>
       <c r="U3" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -709,22 +709,18 @@
           <t>BCI</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Involves use of products, services, activities, rules or environmental objects.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I4" s="2" t="n"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
           <t>behaviour change intervention content; participant engagement with behaviour change intervention; behaviour change intervention mechanism of action; behaviour change intervention outcome behaviour</t>
@@ -735,23 +731,27 @@
           <t>behaviour change intervention scenario plan</t>
         </is>
       </c>
-      <c r="L4" s="2" t="n"/>
-      <c r="M4" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="n"/>
       <c r="N4" s="2" t="n"/>
       <c r="O4" s="2" t="n"/>
-      <c r="P4" s="2" t="n"/>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>JH; BG; PS</t>
+        </is>
+      </c>
       <c r="Q4" s="2" t="n"/>
-      <c r="R4" s="2" t="n"/>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S4" s="2" t="n"/>
-      <c r="T4" s="2" t="inlineStr">
-        <is>
-          <t>JH; BG; PS</t>
-        </is>
-      </c>
+      <c r="T4" s="2" t="n"/>
       <c r="U4" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -785,41 +785,41 @@
           <t>BCI comparison evaluation study</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Comparison involves identifying differences between the entities in the scenarios.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n"/>
       <c r="H5" s="2" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I5" s="2" t="n"/>
       <c r="J5" s="2" t="n"/>
       <c r="K5" s="2" t="n"/>
-      <c r="L5" s="2" t="n"/>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="n"/>
       <c r="N5" s="2" t="n"/>
       <c r="O5" s="2" t="n"/>
-      <c r="P5" s="2" t="n"/>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q5" s="2" t="n"/>
-      <c r="R5" s="2" t="n"/>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S5" s="2" t="n"/>
-      <c r="T5" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T5" s="2" t="n"/>
       <c r="U5" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -853,41 +853,41 @@
           <t>BCI content</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Consists of BCTs that can be classified using a BCT taxonomy. </t>
         </is>
       </c>
-      <c r="G6" s="2" t="n"/>
       <c r="H6" s="2" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I6" s="2" t="n"/>
       <c r="J6" s="2" t="n"/>
       <c r="K6" s="2" t="n"/>
-      <c r="L6" s="2" t="n"/>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="n"/>
       <c r="N6" s="2" t="n"/>
       <c r="O6" s="2" t="n"/>
-      <c r="P6" s="2" t="n"/>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
       <c r="Q6" s="2" t="n"/>
-      <c r="R6" s="2" t="n"/>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S6" s="2" t="n"/>
-      <c r="T6" s="2" t="inlineStr">
-        <is>
-          <t>RW</t>
-        </is>
-      </c>
+      <c r="T6" s="2" t="n"/>
       <c r="U6" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -921,41 +921,41 @@
           <t xml:space="preserve"> BCI context</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Includes as part BCI population and BCI setting. Use of the word ‘may’ conveys a non-zero probability given available information.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n"/>
       <c r="H7" s="2" t="inlineStr">
         <is>
           <t>object aggregate</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I7" s="2" t="n"/>
       <c r="J7" s="2" t="n"/>
       <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="n"/>
       <c r="N7" s="2" t="n"/>
       <c r="O7" s="2" t="n"/>
-      <c r="P7" s="2" t="n"/>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q7" s="2" t="n"/>
-      <c r="R7" s="2" t="n"/>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S7" s="2" t="n"/>
-      <c r="T7" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T7" s="2" t="n"/>
       <c r="U7" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -996,30 +996,30 @@
           <t>process</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I8" s="2" t="n"/>
       <c r="J8" s="2" t="n"/>
       <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="n"/>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="n"/>
       <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="n"/>
-      <c r="P8" s="2" t="n"/>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q8" s="2" t="n"/>
-      <c r="R8" s="2" t="n"/>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S8" s="2" t="n"/>
-      <c r="T8" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T8" s="2" t="n"/>
       <c r="U8" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1053,45 +1053,45 @@
           <t xml:space="preserve"> BCI dose</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The dose of an active ingredient in a pharmacological intervention; the number of behaviour change techniques included in an intervention. </t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">This class requires further specification when it is used because specific BCI content instances may vary in amount in different ways. </t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
         </is>
       </c>
       <c r="J9" s="2" t="n"/>
       <c r="K9" s="2" t="n"/>
-      <c r="L9" s="2" t="n"/>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="n"/>
       <c r="N9" s="2" t="n"/>
       <c r="O9" s="2" t="n"/>
-      <c r="P9" s="2" t="n"/>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q9" s="2" t="n"/>
-      <c r="R9" s="2" t="n"/>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S9" s="2" t="n"/>
-      <c r="T9" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T9" s="2" t="n"/>
       <c r="U9" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1125,41 +1125,41 @@
           <t xml:space="preserve"> BCI effect estimate</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>This includes the following subclasses: 1) BCI effect estimate type -the type of statistic used to represent the difference (e.g. odds ratio, mean difference), 2) BCI effect estimate value – the datum that represents the difference (e.g. 1.35), 3)  BCI effect estimate uncertainty type – the type of statistic used to represent the range of uncertainty of the value (e.g. 95% confidence interval see STATO), and 4) the BCI effect estimate uncertainty value  - the datum representing the uncertainty (e.g. 1.20-1.55).</t>
         </is>
       </c>
-      <c r="G10" s="2" t="n"/>
       <c r="H10" s="2" t="inlineStr">
         <is>
           <t>information content entity</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I10" s="2" t="n"/>
       <c r="J10" s="2" t="n"/>
       <c r="K10" s="2" t="n"/>
-      <c r="L10" s="2" t="n"/>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="n"/>
       <c r="N10" s="2" t="n"/>
       <c r="O10" s="2" t="n"/>
-      <c r="P10" s="2" t="n"/>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW; BG</t>
+        </is>
+      </c>
       <c r="Q10" s="2" t="n"/>
-      <c r="R10" s="2" t="n"/>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S10" s="2" t="n"/>
-      <c r="T10" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW; BG</t>
-        </is>
-      </c>
+      <c r="T10" s="2" t="n"/>
       <c r="U10" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1200,30 +1200,30 @@
           <t>information content entoty</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I11" s="2" t="n"/>
       <c r="J11" s="2" t="n"/>
       <c r="K11" s="2" t="n"/>
-      <c r="L11" s="2" t="n"/>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n"/>
       <c r="N11" s="2" t="n"/>
       <c r="O11" s="2" t="n"/>
-      <c r="P11" s="2" t="n"/>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW; BG</t>
+        </is>
+      </c>
       <c r="Q11" s="2" t="n"/>
-      <c r="R11" s="2" t="n"/>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S11" s="2" t="n"/>
-      <c r="T11" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW; BG</t>
-        </is>
-      </c>
+      <c r="T11" s="2" t="n"/>
       <c r="U11" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1257,41 +1257,41 @@
           <t>BCI evaluation report</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Includes entities that stand in direct relation to the study e.g. authors, findings, funding, aims.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="n"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
           <t>generally dependent continuant</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I12" s="2" t="n"/>
       <c r="J12" s="2" t="n"/>
       <c r="K12" s="2" t="n"/>
-      <c r="L12" s="2" t="n"/>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n"/>
       <c r="N12" s="2" t="n"/>
       <c r="O12" s="2" t="n"/>
-      <c r="P12" s="2" t="n"/>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q12" s="2" t="n"/>
-      <c r="R12" s="2" t="n"/>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S12" s="2" t="n"/>
-      <c r="T12" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T12" s="2" t="n"/>
       <c r="U12" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1332,30 +1332,30 @@
           <t>process</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I13" s="2" t="n"/>
       <c r="J13" s="2" t="n"/>
       <c r="K13" s="2" t="n"/>
-      <c r="L13" s="2" t="n"/>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="n"/>
       <c r="N13" s="2" t="n"/>
       <c r="O13" s="2" t="n"/>
-      <c r="P13" s="2" t="n"/>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q13" s="2" t="n"/>
-      <c r="R13" s="2" t="n"/>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S13" s="2" t="n"/>
-      <c r="T13" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T13" s="2" t="n"/>
       <c r="U13" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1396,30 +1396,30 @@
           <t>information content entity</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="n"/>
       <c r="K14" s="2" t="n"/>
-      <c r="L14" s="2" t="n"/>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n"/>
       <c r="N14" s="2" t="n"/>
       <c r="O14" s="2" t="n"/>
-      <c r="P14" s="2" t="n"/>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q14" s="2" t="n"/>
-      <c r="R14" s="2" t="n"/>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S14" s="2" t="n"/>
-      <c r="T14" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T14" s="2" t="n"/>
       <c r="U14" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1460,30 +1460,30 @@
           <t>information content entity</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="n"/>
       <c r="K15" s="2" t="n"/>
-      <c r="L15" s="2" t="n"/>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n"/>
       <c r="N15" s="2" t="n"/>
       <c r="O15" s="2" t="n"/>
-      <c r="P15" s="2" t="n"/>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q15" s="2" t="n"/>
-      <c r="R15" s="2" t="n"/>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S15" s="2" t="n"/>
-      <c r="T15" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T15" s="2" t="n"/>
       <c r="U15" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1524,30 +1524,30 @@
           <t>process</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I16" s="2" t="n"/>
       <c r="J16" s="2" t="n"/>
       <c r="K16" s="2" t="n"/>
-      <c r="L16" s="2" t="n"/>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n"/>
       <c r="N16" s="2" t="n"/>
       <c r="O16" s="2" t="n"/>
-      <c r="P16" s="2" t="n"/>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>PS; JH; RW</t>
+        </is>
+      </c>
       <c r="Q16" s="2" t="n"/>
-      <c r="R16" s="2" t="n"/>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S16" s="2" t="n"/>
-      <c r="T16" s="2" t="inlineStr">
-        <is>
-          <t>PS; JH; RW</t>
-        </is>
-      </c>
+      <c r="T16" s="2" t="n"/>
       <c r="U16" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1588,30 +1588,30 @@
           <t>process</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I17" s="2" t="n"/>
       <c r="J17" s="2" t="n"/>
       <c r="K17" s="2" t="n"/>
-      <c r="L17" s="2" t="n"/>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n"/>
       <c r="N17" s="2" t="n"/>
       <c r="O17" s="2" t="n"/>
-      <c r="P17" s="2" t="n"/>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q17" s="2" t="n"/>
-      <c r="R17" s="2" t="n"/>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S17" s="2" t="n"/>
-      <c r="T17" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T17" s="2" t="n"/>
       <c r="U17" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1641,37 +1641,37 @@
         </is>
       </c>
       <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>'individual human behaviour' AND 'intervention outcome'</t>
+        </is>
+      </c>
       <c r="G18" s="2" t="n"/>
       <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I18" s="2" t="n"/>
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
-      <c r="L18" s="2" t="n"/>
-      <c r="M18" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n"/>
       <c r="N18" s="2" t="n"/>
       <c r="O18" s="2" t="n"/>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>'individual human behaviour' AND 'intervention outcome'</t>
+          <t>JH; BG; PS</t>
         </is>
       </c>
       <c r="Q18" s="2" t="n"/>
-      <c r="R18" s="2" t="n"/>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S18" s="2" t="n"/>
-      <c r="T18" s="2" t="inlineStr">
-        <is>
-          <t>JH; BG; PS</t>
-        </is>
-      </c>
+      <c r="T18" s="2" t="n"/>
       <c r="U18" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1705,41 +1705,41 @@
           <t>BCI outcome estimate</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>This includes as subclasses 1) type of outcome estimate (e.g. mean, percentage), 2) value of outcome estimate (e.g. 1.5 cigs per day, 23%), 3) uncertainty estimate type (e.g. 95% CI), and 4) uncertainty estimate value (e.g. 12.0%-45.0%).</t>
         </is>
       </c>
-      <c r="G19" s="2" t="n"/>
       <c r="H19" s="2" t="inlineStr">
         <is>
           <t>information content entoty</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I19" s="2" t="n"/>
       <c r="J19" s="2" t="n"/>
       <c r="K19" s="2" t="n"/>
-      <c r="L19" s="2" t="n"/>
-      <c r="M19" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n"/>
       <c r="N19" s="2" t="n"/>
       <c r="O19" s="2" t="n"/>
-      <c r="P19" s="2" t="n"/>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q19" s="2" t="n"/>
-      <c r="R19" s="2" t="n"/>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S19" s="2" t="n"/>
-      <c r="T19" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T19" s="2" t="n"/>
       <c r="U19" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1776,30 +1776,30 @@
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="n"/>
       <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I20" s="2" t="n"/>
       <c r="J20" s="2" t="n"/>
       <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="n"/>
-      <c r="M20" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="n"/>
       <c r="N20" s="2" t="n"/>
       <c r="O20" s="2" t="n"/>
-      <c r="P20" s="2" t="n"/>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q20" s="2" t="n"/>
-      <c r="R20" s="2" t="n"/>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S20" s="2" t="n"/>
-      <c r="T20" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T20" s="2" t="n"/>
       <c r="U20" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1836,30 +1836,30 @@
       <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="n"/>
       <c r="H21" s="2" t="n"/>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I21" s="2" t="n"/>
       <c r="J21" s="2" t="n"/>
       <c r="K21" s="2" t="n"/>
-      <c r="L21" s="2" t="n"/>
-      <c r="M21" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n"/>
       <c r="N21" s="2" t="n"/>
       <c r="O21" s="2" t="n"/>
-      <c r="P21" s="2" t="n"/>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW; PS</t>
+        </is>
+      </c>
       <c r="Q21" s="2" t="n"/>
-      <c r="R21" s="2" t="n"/>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S21" s="2" t="n"/>
-      <c r="T21" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW; PS</t>
-        </is>
-      </c>
+      <c r="T21" s="2" t="n"/>
       <c r="U21" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1896,34 +1896,34 @@
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="n"/>
       <c r="H22" s="2" t="n"/>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I22" s="2" t="n"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
           <t>behaviour change intervention outcome behaviour</t>
         </is>
       </c>
       <c r="K22" s="2" t="n"/>
-      <c r="L22" s="2" t="n"/>
-      <c r="M22" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="n"/>
       <c r="N22" s="2" t="n"/>
       <c r="O22" s="2" t="n"/>
-      <c r="P22" s="2" t="n"/>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q22" s="2" t="n"/>
-      <c r="R22" s="2" t="n"/>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S22" s="2" t="n"/>
-      <c r="T22" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T22" s="2" t="n"/>
       <c r="U22" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1960,30 +1960,30 @@
       <c r="F23" s="2" t="n"/>
       <c r="G23" s="2" t="n"/>
       <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I23" s="2" t="n"/>
       <c r="J23" s="2" t="n"/>
       <c r="K23" s="2" t="n"/>
-      <c r="L23" s="2" t="n"/>
-      <c r="M23" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="n"/>
       <c r="N23" s="2" t="n"/>
       <c r="O23" s="2" t="n"/>
-      <c r="P23" s="2" t="n"/>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q23" s="2" t="n"/>
-      <c r="R23" s="2" t="n"/>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S23" s="2" t="n"/>
-      <c r="T23" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T23" s="2" t="n"/>
       <c r="U23" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2020,30 +2020,30 @@
       <c r="F24" s="2" t="n"/>
       <c r="G24" s="2" t="n"/>
       <c r="H24" s="2" t="n"/>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I24" s="2" t="n"/>
       <c r="J24" s="2" t="n"/>
       <c r="K24" s="2" t="n"/>
-      <c r="L24" s="2" t="n"/>
-      <c r="M24" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="n"/>
       <c r="N24" s="2" t="n"/>
       <c r="O24" s="2" t="n"/>
-      <c r="P24" s="2" t="n"/>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q24" s="2" t="n"/>
-      <c r="R24" s="2" t="n"/>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S24" s="2" t="n"/>
-      <c r="T24" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T24" s="2" t="n"/>
       <c r="U24" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2077,37 +2077,37 @@
           <t>BCI setting</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>Includes as parts social setting and physical setting.</t>
         </is>
       </c>
-      <c r="G25" s="2" t="n"/>
       <c r="H25" s="2" t="n"/>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I25" s="2" t="n"/>
       <c r="J25" s="2" t="n"/>
       <c r="K25" s="2" t="n"/>
-      <c r="L25" s="2" t="n"/>
-      <c r="M25" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="n"/>
       <c r="N25" s="2" t="n"/>
       <c r="O25" s="2" t="n"/>
-      <c r="P25" s="2" t="n"/>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q25" s="2" t="n"/>
-      <c r="R25" s="2" t="n"/>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S25" s="2" t="n"/>
-      <c r="T25" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T25" s="2" t="n"/>
       <c r="U25" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2144,30 +2144,30 @@
       <c r="F26" s="2" t="n"/>
       <c r="G26" s="2" t="n"/>
       <c r="H26" s="2" t="n"/>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I26" s="2" t="n"/>
       <c r="J26" s="2" t="n"/>
       <c r="K26" s="2" t="n"/>
-      <c r="L26" s="2" t="n"/>
-      <c r="M26" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="n"/>
       <c r="N26" s="2" t="n"/>
       <c r="O26" s="2" t="n"/>
-      <c r="P26" s="2" t="n"/>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q26" s="2" t="n"/>
-      <c r="R26" s="2" t="n"/>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S26" s="2" t="n"/>
-      <c r="T26" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T26" s="2" t="n"/>
       <c r="U26" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2201,37 +2201,37 @@
           <t>BCI source</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>This includes individual people, groups of people, and organisations.</t>
         </is>
       </c>
-      <c r="G27" s="2" t="n"/>
       <c r="H27" s="2" t="n"/>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I27" s="2" t="n"/>
       <c r="J27" s="2" t="n"/>
       <c r="K27" s="2" t="n"/>
-      <c r="L27" s="2" t="n"/>
-      <c r="M27" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="n"/>
       <c r="N27" s="2" t="n"/>
       <c r="O27" s="2" t="n"/>
-      <c r="P27" s="2" t="n"/>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q27" s="2" t="n"/>
-      <c r="R27" s="2" t="n"/>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S27" s="2" t="n"/>
-      <c r="T27" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T27" s="2" t="n"/>
       <c r="U27" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2247,17 +2247,17 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention study investigator</t>
+          <t>behaviour change intervention study investigator role</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>A role played by a person that contributes substantively to production or reporting of a BCI evaluation study.</t>
+          <t>A researcher role played by a person that contributes substantively to production or reporting of a BCI evaluation study.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>role</t>
+          <t>researcher role</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2265,37 +2265,37 @@
           <t>BCI study investigator</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">What counts as substantively is subject to judgement. The level and nature of the contribution can be defined using the CReDiT taxonomy (https://casrai.org/credit/). </t>
         </is>
       </c>
-      <c r="G28" s="2" t="n"/>
       <c r="H28" s="2" t="n"/>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I28" s="2" t="n"/>
       <c r="J28" s="2" t="n"/>
       <c r="K28" s="2" t="n"/>
-      <c r="L28" s="2" t="n"/>
-      <c r="M28" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="n"/>
       <c r="N28" s="2" t="n"/>
       <c r="O28" s="2" t="n"/>
-      <c r="P28" s="2" t="n"/>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q28" s="2" t="n"/>
-      <c r="R28" s="2" t="n"/>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S28" s="2" t="n"/>
-      <c r="T28" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T28" s="2" t="n"/>
       <c r="U28" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2332,30 +2332,30 @@
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="2" t="n"/>
       <c r="H29" s="2" t="n"/>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I29" s="2" t="n"/>
       <c r="J29" s="2" t="n"/>
       <c r="K29" s="2" t="n"/>
-      <c r="L29" s="2" t="n"/>
-      <c r="M29" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="n"/>
       <c r="N29" s="2" t="n"/>
       <c r="O29" s="2" t="n"/>
-      <c r="P29" s="2" t="n"/>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW; PS</t>
+        </is>
+      </c>
       <c r="Q29" s="2" t="n"/>
-      <c r="R29" s="2" t="n"/>
+      <c r="R29" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S29" s="2" t="n"/>
-      <c r="T29" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW; PS</t>
-        </is>
-      </c>
+      <c r="T29" s="2" t="n"/>
       <c r="U29" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2389,37 +2389,37 @@
           <t>BCI style of delivery</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>An example is cold and distant vs. warm and accepting.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="n"/>
       <c r="H30" s="2" t="n"/>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I30" s="2" t="n"/>
       <c r="J30" s="2" t="n"/>
       <c r="K30" s="2" t="n"/>
-      <c r="L30" s="2" t="n"/>
-      <c r="M30" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="n"/>
       <c r="N30" s="2" t="n"/>
       <c r="O30" s="2" t="n"/>
-      <c r="P30" s="2" t="n"/>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q30" s="2" t="n"/>
-      <c r="R30" s="2" t="n"/>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S30" s="2" t="n"/>
-      <c r="T30" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T30" s="2" t="n"/>
       <c r="U30" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2453,45 +2453,45 @@
           <t>BCI tailoring</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>Tailoring the dose of pharmacotherapy for smoking cessation to the prior level of nicotine dependence of the smoker (static) or to the smokers' current strength of urges to smoke during a quit attempt (dynamic).</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>Tailoring can be static (i.e., conducted before intervention delivery in a case case), or dynamic (i.e., conducted one or more times after the intervention has started in a given case based on population or setting characteristics present at that time. Population and setting characteristics include the historical factors such as prior exposure to the intervention.</t>
         </is>
       </c>
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>Tailoring can be static (i.e., conducted before intervention delivery in a case case), or dynamic (i.e., conducted one or more times after the intervention has started in a given case based on population or setting characteristics present at that time. Population and setting characteristics include the historical factors such as prior exposure to the intervention.</t>
         </is>
       </c>
       <c r="J31" s="2" t="n"/>
       <c r="K31" s="2" t="n"/>
-      <c r="L31" s="2" t="n"/>
-      <c r="M31" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="n"/>
       <c r="N31" s="2" t="n"/>
       <c r="O31" s="2" t="n"/>
-      <c r="P31" s="2" t="n"/>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q31" s="2" t="inlineStr">
         <is>
           <t>An attribute of a behaviour change intervention (BCI) or a BCI component whereby its content or delivery is varied according to characteristics of members of the target population or setting.</t>
         </is>
       </c>
-      <c r="R31" s="2" t="n"/>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S31" s="2" t="n"/>
-      <c r="T31" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T31" s="2" t="n"/>
       <c r="U31" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2528,30 +2528,30 @@
       <c r="F32" s="2" t="n"/>
       <c r="G32" s="2" t="n"/>
       <c r="H32" s="2" t="n"/>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I32" s="2" t="n"/>
       <c r="J32" s="2" t="n"/>
       <c r="K32" s="2" t="n"/>
-      <c r="L32" s="2" t="n"/>
-      <c r="M32" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="n"/>
       <c r="N32" s="2" t="n"/>
       <c r="O32" s="2" t="n"/>
-      <c r="P32" s="2" t="n"/>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q32" s="2" t="n"/>
-      <c r="R32" s="2" t="n"/>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S32" s="2" t="n"/>
-      <c r="T32" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T32" s="2" t="n"/>
       <c r="U32" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2588,30 +2588,30 @@
       <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="n"/>
       <c r="H33" s="2" t="n"/>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I33" s="2" t="n"/>
       <c r="J33" s="2" t="n"/>
       <c r="K33" s="2" t="n"/>
-      <c r="L33" s="2" t="n"/>
-      <c r="M33" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="n"/>
       <c r="N33" s="2" t="n"/>
       <c r="O33" s="2" t="n"/>
-      <c r="P33" s="2" t="n"/>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q33" s="2" t="n"/>
-      <c r="R33" s="2" t="n"/>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S33" s="2" t="n"/>
-      <c r="T33" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T33" s="2" t="n"/>
       <c r="U33" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2648,30 +2648,30 @@
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="n"/>
       <c r="H34" s="2" t="n"/>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I34" s="2" t="n"/>
       <c r="J34" s="2" t="n"/>
       <c r="K34" s="2" t="n"/>
-      <c r="L34" s="2" t="n"/>
-      <c r="M34" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="n"/>
       <c r="N34" s="2" t="n"/>
       <c r="O34" s="2" t="n"/>
-      <c r="P34" s="2" t="n"/>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW; PS</t>
+        </is>
+      </c>
       <c r="Q34" s="2" t="n"/>
-      <c r="R34" s="2" t="n"/>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S34" s="2" t="n"/>
-      <c r="T34" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW; PS</t>
-        </is>
-      </c>
+      <c r="T34" s="2" t="n"/>
       <c r="U34" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2704,30 +2704,30 @@
       <c r="F35" s="2" t="n"/>
       <c r="G35" s="2" t="n"/>
       <c r="H35" s="2" t="n"/>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I35" s="2" t="n"/>
       <c r="J35" s="2" t="n"/>
       <c r="K35" s="2" t="n"/>
-      <c r="L35" s="2" t="n"/>
-      <c r="M35" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="n"/>
       <c r="N35" s="2" t="n"/>
       <c r="O35" s="2" t="n"/>
-      <c r="P35" s="2" t="n"/>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>JH; PS</t>
+        </is>
+      </c>
       <c r="Q35" s="2" t="n"/>
-      <c r="R35" s="2" t="n"/>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S35" s="2" t="n"/>
-      <c r="T35" s="2" t="inlineStr">
-        <is>
-          <t>JH; PS</t>
-        </is>
-      </c>
+      <c r="T35" s="2" t="n"/>
       <c r="U35" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2760,30 +2760,30 @@
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="2" t="n"/>
       <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I36" s="2" t="n"/>
       <c r="J36" s="2" t="n"/>
       <c r="K36" s="2" t="n"/>
-      <c r="L36" s="2" t="n"/>
-      <c r="M36" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="n"/>
       <c r="N36" s="2" t="n"/>
       <c r="O36" s="2" t="n"/>
-      <c r="P36" s="2" t="n"/>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>JH</t>
+        </is>
+      </c>
       <c r="Q36" s="2" t="n"/>
-      <c r="R36" s="2" t="n"/>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S36" s="2" t="n"/>
-      <c r="T36" s="2" t="inlineStr">
-        <is>
-          <t>JH</t>
-        </is>
-      </c>
+      <c r="T36" s="2" t="n"/>
       <c r="U36" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2814,36 +2814,36 @@
       </c>
       <c r="E37" s="3" t="n"/>
       <c r="F37" s="3" t="n"/>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>High cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="G37" s="3" t="n"/>
       <c r="H37" s="3" t="n"/>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>High cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J37" s="3" t="n"/>
       <c r="K37" s="3" t="n"/>
-      <c r="L37" s="3" t="n"/>
-      <c r="M37" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="L37" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="M37" s="3" t="n"/>
       <c r="N37" s="3" t="n"/>
       <c r="O37" s="3" t="n"/>
-      <c r="P37" s="3" t="n"/>
+      <c r="P37" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
       <c r="Q37" s="3" t="n"/>
-      <c r="R37" s="3" t="n"/>
+      <c r="R37" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
       <c r="S37" s="3" t="n"/>
-      <c r="T37" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="T37" s="3" t="n"/>
       <c r="U37" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -2874,36 +2874,36 @@
       </c>
       <c r="E38" s="3" t="n"/>
       <c r="F38" s="3" t="n"/>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>High emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="G38" s="3" t="n"/>
       <c r="H38" s="3" t="n"/>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>High emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J38" s="3" t="n"/>
       <c r="K38" s="3" t="n"/>
-      <c r="L38" s="3" t="n"/>
-      <c r="M38" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="L38" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="n"/>
       <c r="N38" s="3" t="n"/>
       <c r="O38" s="3" t="n"/>
-      <c r="P38" s="3" t="n"/>
+      <c r="P38" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
       <c r="Q38" s="3" t="n"/>
-      <c r="R38" s="3" t="n"/>
+      <c r="R38" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
       <c r="S38" s="3" t="n"/>
-      <c r="T38" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="T38" s="3" t="n"/>
       <c r="U38" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -2934,36 +2934,36 @@
       </c>
       <c r="E39" s="3" t="n"/>
       <c r="F39" s="3" t="n"/>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>High mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="G39" s="3" t="n"/>
       <c r="H39" s="3" t="n"/>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>High mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J39" s="3" t="n"/>
       <c r="K39" s="3" t="n"/>
-      <c r="L39" s="3" t="n"/>
-      <c r="M39" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="L39" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="M39" s="3" t="n"/>
       <c r="N39" s="3" t="n"/>
       <c r="O39" s="3" t="n"/>
-      <c r="P39" s="3" t="n"/>
+      <c r="P39" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
       <c r="Q39" s="3" t="n"/>
-      <c r="R39" s="3" t="n"/>
+      <c r="R39" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
       <c r="S39" s="3" t="n"/>
-      <c r="T39" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="T39" s="3" t="n"/>
       <c r="U39" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -2994,36 +2994,36 @@
       </c>
       <c r="E40" s="3" t="n"/>
       <c r="F40" s="3" t="n"/>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>High physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="G40" s="3" t="n"/>
       <c r="H40" s="3" t="n"/>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>High physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J40" s="3" t="n"/>
       <c r="K40" s="3" t="n"/>
-      <c r="L40" s="3" t="n"/>
-      <c r="M40" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="L40" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="M40" s="3" t="n"/>
       <c r="N40" s="3" t="n"/>
       <c r="O40" s="3" t="n"/>
-      <c r="P40" s="3" t="n"/>
+      <c r="P40" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
       <c r="Q40" s="3" t="n"/>
-      <c r="R40" s="3" t="n"/>
+      <c r="R40" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
       <c r="S40" s="3" t="n"/>
-      <c r="T40" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="T40" s="3" t="n"/>
       <c r="U40" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -3053,37 +3053,37 @@
         </is>
       </c>
       <c r="E41" s="3" t="n"/>
-      <c r="F41" s="3" t="n"/>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>"individual human behaviour" OR "population behaviour"</t>
+        </is>
+      </c>
       <c r="G41" s="3" t="n"/>
       <c r="H41" s="3" t="n"/>
-      <c r="I41" s="3" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I41" s="3" t="n"/>
       <c r="J41" s="3" t="n"/>
       <c r="K41" s="3" t="n"/>
-      <c r="L41" s="3" t="n"/>
-      <c r="M41" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M41" s="3" t="n"/>
       <c r="N41" s="3" t="n"/>
       <c r="O41" s="3" t="n"/>
       <c r="P41" s="3" t="inlineStr">
         <is>
-          <t>"individual human behaviour" OR "population behaviour"</t>
+          <t>BG; PS</t>
         </is>
       </c>
       <c r="Q41" s="3" t="n"/>
-      <c r="R41" s="3" t="n"/>
+      <c r="R41" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
       <c r="S41" s="3" t="n"/>
-      <c r="T41" s="3" t="inlineStr">
-        <is>
-          <t>BG; PS</t>
-        </is>
-      </c>
+      <c r="T41" s="3" t="n"/>
       <c r="U41" s="3" t="inlineStr">
         <is>
           <t>0</t>
@@ -3116,30 +3116,30 @@
       <c r="F42" s="2" t="n"/>
       <c r="G42" s="2" t="n"/>
       <c r="H42" s="2" t="n"/>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I42" s="2" t="n"/>
       <c r="J42" s="2" t="n"/>
       <c r="K42" s="2" t="n"/>
-      <c r="L42" s="2" t="n"/>
-      <c r="M42" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="n"/>
       <c r="N42" s="2" t="n"/>
       <c r="O42" s="2" t="n"/>
-      <c r="P42" s="2" t="n"/>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>JH; AW</t>
+        </is>
+      </c>
       <c r="Q42" s="2" t="n"/>
-      <c r="R42" s="2" t="n"/>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S42" s="2" t="n"/>
-      <c r="T42" s="2" t="inlineStr">
-        <is>
-          <t>JH; AW</t>
-        </is>
-      </c>
+      <c r="T42" s="2" t="n"/>
       <c r="U42" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3172,30 +3172,30 @@
       <c r="F43" s="2" t="n"/>
       <c r="G43" s="2" t="n"/>
       <c r="H43" s="2" t="n"/>
-      <c r="I43" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I43" s="2" t="n"/>
       <c r="J43" s="2" t="n"/>
       <c r="K43" s="2" t="n"/>
-      <c r="L43" s="2" t="n"/>
-      <c r="M43" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="n"/>
       <c r="N43" s="2" t="n"/>
       <c r="O43" s="2" t="n"/>
-      <c r="P43" s="2" t="n"/>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>JH</t>
+        </is>
+      </c>
       <c r="Q43" s="2" t="n"/>
-      <c r="R43" s="2" t="n"/>
+      <c r="R43" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S43" s="2" t="n"/>
-      <c r="T43" s="2" t="inlineStr">
-        <is>
-          <t>JH</t>
-        </is>
-      </c>
+      <c r="T43" s="2" t="n"/>
       <c r="U43" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3229,37 +3229,37 @@
           <t>human behaviour</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F44" s="2" t="n"/>
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Also referred to in definitions as human behaviour or just behaviour.</t>
         </is>
       </c>
-      <c r="G44" s="2" t="n"/>
       <c r="H44" s="2" t="n"/>
-      <c r="I44" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I44" s="2" t="n"/>
       <c r="J44" s="2" t="n"/>
       <c r="K44" s="2" t="n"/>
-      <c r="L44" s="2" t="n"/>
-      <c r="M44" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="n"/>
       <c r="N44" s="2" t="n"/>
       <c r="O44" s="2" t="n"/>
-      <c r="P44" s="2" t="n"/>
+      <c r="P44" s="2" t="inlineStr">
+        <is>
+          <t>JH</t>
+        </is>
+      </c>
       <c r="Q44" s="2" t="n"/>
-      <c r="R44" s="2" t="n"/>
+      <c r="R44" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S44" s="2" t="n"/>
-      <c r="T44" s="2" t="inlineStr">
-        <is>
-          <t>JH</t>
-        </is>
-      </c>
+      <c r="T44" s="2" t="n"/>
       <c r="U44" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3289,37 +3289,37 @@
         </is>
       </c>
       <c r="E45" s="2" t="n"/>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F45" s="2" t="n"/>
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>Examples of interventions are putting health warnings on cigarette packets, providing free stop smoking services and banning smoking in public places.</t>
         </is>
       </c>
-      <c r="G45" s="2" t="n"/>
       <c r="H45" s="2" t="n"/>
-      <c r="I45" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I45" s="2" t="n"/>
       <c r="J45" s="2" t="n"/>
       <c r="K45" s="2" t="n"/>
-      <c r="L45" s="2" t="n"/>
-      <c r="M45" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="n"/>
       <c r="N45" s="2" t="n"/>
       <c r="O45" s="2" t="n"/>
-      <c r="P45" s="2" t="n"/>
+      <c r="P45" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q45" s="2" t="n"/>
-      <c r="R45" s="2" t="n"/>
+      <c r="R45" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S45" s="2" t="n"/>
-      <c r="T45" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T45" s="2" t="n"/>
       <c r="U45" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3348,30 +3348,30 @@
           <t>process attribute</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr"/>
-      <c r="F46" s="4" t="inlineStr"/>
-      <c r="G46" s="4" t="inlineStr"/>
-      <c r="H46" s="4" t="inlineStr"/>
-      <c r="I46" s="4" t="inlineStr"/>
-      <c r="J46" s="4" t="inlineStr"/>
-      <c r="K46" s="4" t="inlineStr"/>
-      <c r="L46" s="4" t="inlineStr"/>
-      <c r="M46" s="4" t="inlineStr">
+      <c r="E46" s="4" t="n"/>
+      <c r="F46" s="4" t="n"/>
+      <c r="G46" s="4" t="n"/>
+      <c r="H46" s="4" t="n"/>
+      <c r="I46" s="4" t="n"/>
+      <c r="J46" s="4" t="n"/>
+      <c r="K46" s="4" t="n"/>
+      <c r="L46" s="4" t="n"/>
+      <c r="M46" s="4" t="n"/>
+      <c r="N46" s="4" t="n"/>
+      <c r="O46" s="4" t="n"/>
+      <c r="P46" s="4" t="n"/>
+      <c r="Q46" s="4" t="n"/>
+      <c r="R46" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="N46" s="4" t="inlineStr"/>
-      <c r="O46" s="4" t="inlineStr"/>
-      <c r="P46" s="4" t="inlineStr"/>
-      <c r="Q46" s="4" t="inlineStr"/>
-      <c r="R46" s="4" t="inlineStr"/>
-      <c r="S46" s="4" t="inlineStr"/>
-      <c r="T46" s="4" t="inlineStr"/>
+      <c r="S46" s="4" t="n"/>
+      <c r="T46" s="4" t="n"/>
       <c r="U46" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="V46" s="4" t="inlineStr"/>
+      <c r="V46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3398,30 +3398,30 @@
       <c r="F47" s="2" t="n"/>
       <c r="G47" s="2" t="n"/>
       <c r="H47" s="2" t="n"/>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I47" s="2" t="n"/>
       <c r="J47" s="2" t="n"/>
       <c r="K47" s="2" t="n"/>
-      <c r="L47" s="2" t="n"/>
-      <c r="M47" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M47" s="2" t="n"/>
       <c r="N47" s="2" t="n"/>
       <c r="O47" s="2" t="n"/>
-      <c r="P47" s="2" t="n"/>
+      <c r="P47" s="2" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
       <c r="Q47" s="2" t="n"/>
-      <c r="R47" s="2" t="n"/>
+      <c r="R47" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S47" s="2" t="n"/>
-      <c r="T47" s="2" t="inlineStr">
-        <is>
-          <t>RW</t>
-        </is>
-      </c>
+      <c r="T47" s="2" t="n"/>
       <c r="U47" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3445,7 +3445,7 @@
           <t>process context</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr">
+      <c r="R48" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -3479,30 +3479,30 @@
       <c r="F49" s="2" t="n"/>
       <c r="G49" s="2" t="n"/>
       <c r="H49" s="2" t="n"/>
-      <c r="I49" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I49" s="2" t="n"/>
       <c r="J49" s="2" t="n"/>
       <c r="K49" s="2" t="n"/>
-      <c r="L49" s="2" t="n"/>
-      <c r="M49" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="n"/>
       <c r="N49" s="2" t="n"/>
       <c r="O49" s="2" t="n"/>
-      <c r="P49" s="2" t="n"/>
+      <c r="P49" s="2" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
       <c r="Q49" s="2" t="n"/>
-      <c r="R49" s="2" t="n"/>
+      <c r="R49" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S49" s="2" t="n"/>
-      <c r="T49" s="2" t="inlineStr">
-        <is>
-          <t>RW</t>
-        </is>
-      </c>
+      <c r="T49" s="2" t="n"/>
       <c r="U49" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3535,30 +3535,30 @@
       <c r="F50" s="2" t="n"/>
       <c r="G50" s="2" t="n"/>
       <c r="H50" s="2" t="n"/>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I50" s="2" t="n"/>
       <c r="J50" s="2" t="n"/>
       <c r="K50" s="2" t="n"/>
-      <c r="L50" s="2" t="n"/>
-      <c r="M50" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="n"/>
       <c r="N50" s="2" t="n"/>
       <c r="O50" s="2" t="n"/>
-      <c r="P50" s="2" t="n"/>
+      <c r="P50" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q50" s="2" t="n"/>
-      <c r="R50" s="2" t="n"/>
+      <c r="R50" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S50" s="2" t="n"/>
-      <c r="T50" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T50" s="2" t="n"/>
       <c r="U50" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3591,30 +3591,30 @@
       <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="n"/>
       <c r="H51" s="2" t="n"/>
-      <c r="I51" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I51" s="2" t="n"/>
       <c r="J51" s="2" t="n"/>
       <c r="K51" s="2" t="n"/>
-      <c r="L51" s="2" t="n"/>
-      <c r="M51" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="n"/>
       <c r="N51" s="2" t="n"/>
       <c r="O51" s="2" t="n"/>
-      <c r="P51" s="2" t="n"/>
+      <c r="P51" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q51" s="2" t="n"/>
-      <c r="R51" s="2" t="n"/>
+      <c r="R51" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S51" s="2" t="n"/>
-      <c r="T51" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T51" s="2" t="n"/>
       <c r="U51" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3644,37 +3644,37 @@
         </is>
       </c>
       <c r="E52" s="2" t="n"/>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F52" s="2" t="n"/>
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Includes individual human behaviour, mental activity and physiological activity. Also includes undesirable outcomes, such as treatment side effects, and unintended negative consequences of the intervention. </t>
         </is>
       </c>
-      <c r="G52" s="2" t="n"/>
       <c r="H52" s="2" t="n"/>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I52" s="2" t="n"/>
       <c r="J52" s="2" t="n"/>
       <c r="K52" s="2" t="n"/>
-      <c r="L52" s="2" t="n"/>
-      <c r="M52" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="n"/>
       <c r="N52" s="2" t="n"/>
       <c r="O52" s="2" t="n"/>
-      <c r="P52" s="2" t="n"/>
+      <c r="P52" s="2" t="inlineStr">
+        <is>
+          <t>JH</t>
+        </is>
+      </c>
       <c r="Q52" s="2" t="n"/>
-      <c r="R52" s="2" t="n"/>
+      <c r="R52" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S52" s="2" t="n"/>
-      <c r="T52" s="2" t="inlineStr">
-        <is>
-          <t>JH</t>
-        </is>
-      </c>
+      <c r="T52" s="2" t="n"/>
       <c r="U52" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3707,30 +3707,30 @@
       <c r="F53" s="2" t="n"/>
       <c r="G53" s="2" t="n"/>
       <c r="H53" s="2" t="n"/>
-      <c r="I53" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I53" s="2" t="n"/>
       <c r="J53" s="2" t="n"/>
       <c r="K53" s="2" t="n"/>
-      <c r="L53" s="2" t="n"/>
-      <c r="M53" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="n"/>
       <c r="N53" s="2" t="n"/>
       <c r="O53" s="2" t="n"/>
-      <c r="P53" s="2" t="n"/>
+      <c r="P53" s="2" t="inlineStr">
+        <is>
+          <t>AW; PS</t>
+        </is>
+      </c>
       <c r="Q53" s="2" t="n"/>
-      <c r="R53" s="2" t="n"/>
+      <c r="R53" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S53" s="2" t="n"/>
-      <c r="T53" s="2" t="inlineStr">
-        <is>
-          <t>AW; PS</t>
-        </is>
-      </c>
+      <c r="T53" s="2" t="n"/>
       <c r="U53" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3764,41 +3764,41 @@
           <t>BCI schedule of delivery</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F54" s="2" t="n"/>
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>Includes the start and end of the BCI and its parts.</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
         </is>
       </c>
       <c r="H54" s="2" t="n"/>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>Upper level</t>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
         </is>
       </c>
       <c r="J54" s="2" t="n"/>
       <c r="K54" s="2" t="n"/>
-      <c r="L54" s="2" t="n"/>
-      <c r="M54" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="n"/>
       <c r="N54" s="2" t="n"/>
       <c r="O54" s="2" t="n"/>
-      <c r="P54" s="2" t="n"/>
+      <c r="P54" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
       <c r="Q54" s="2" t="n"/>
-      <c r="R54" s="2" t="n"/>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S54" s="2" t="n"/>
-      <c r="T54" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
+      <c r="T54" s="2" t="n"/>
       <c r="U54" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3822,7 +3822,7 @@
           <t>intervention context</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr">
+      <c r="R55" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -3854,36 +3854,36 @@
       </c>
       <c r="E56" s="3" t="n"/>
       <c r="F56" s="3" t="n"/>
-      <c r="G56" s="3" t="inlineStr">
-        <is>
-          <t>Low cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="G56" s="3" t="n"/>
       <c r="H56" s="3" t="n"/>
       <c r="I56" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Low cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J56" s="3" t="n"/>
       <c r="K56" s="3" t="n"/>
-      <c r="L56" s="3" t="n"/>
-      <c r="M56" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="L56" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="M56" s="3" t="n"/>
       <c r="N56" s="3" t="n"/>
       <c r="O56" s="3" t="n"/>
-      <c r="P56" s="3" t="n"/>
+      <c r="P56" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
       <c r="Q56" s="3" t="n"/>
-      <c r="R56" s="3" t="n"/>
+      <c r="R56" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
       <c r="S56" s="3" t="n"/>
-      <c r="T56" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="T56" s="3" t="n"/>
       <c r="U56" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -3914,36 +3914,36 @@
       </c>
       <c r="E57" s="3" t="n"/>
       <c r="F57" s="3" t="n"/>
-      <c r="G57" s="3" t="inlineStr">
-        <is>
-          <t>Low emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="G57" s="3" t="n"/>
       <c r="H57" s="3" t="n"/>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Low emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J57" s="3" t="n"/>
       <c r="K57" s="3" t="n"/>
-      <c r="L57" s="3" t="n"/>
-      <c r="M57" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="L57" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="M57" s="3" t="n"/>
       <c r="N57" s="3" t="n"/>
       <c r="O57" s="3" t="n"/>
-      <c r="P57" s="3" t="n"/>
+      <c r="P57" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
       <c r="Q57" s="3" t="n"/>
-      <c r="R57" s="3" t="n"/>
+      <c r="R57" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
       <c r="S57" s="3" t="n"/>
-      <c r="T57" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="T57" s="3" t="n"/>
       <c r="U57" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -3974,36 +3974,36 @@
       </c>
       <c r="E58" s="3" t="n"/>
       <c r="F58" s="3" t="n"/>
-      <c r="G58" s="3" t="inlineStr">
-        <is>
-          <t>Low mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="G58" s="3" t="n"/>
       <c r="H58" s="3" t="n"/>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Low mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J58" s="3" t="n"/>
       <c r="K58" s="3" t="n"/>
-      <c r="L58" s="3" t="n"/>
-      <c r="M58" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="L58" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="M58" s="3" t="n"/>
       <c r="N58" s="3" t="n"/>
       <c r="O58" s="3" t="n"/>
-      <c r="P58" s="3" t="n"/>
+      <c r="P58" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
       <c r="Q58" s="3" t="n"/>
-      <c r="R58" s="3" t="n"/>
+      <c r="R58" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
       <c r="S58" s="3" t="n"/>
-      <c r="T58" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="T58" s="3" t="n"/>
       <c r="U58" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -4034,36 +4034,36 @@
       </c>
       <c r="E59" s="3" t="n"/>
       <c r="F59" s="3" t="n"/>
-      <c r="G59" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Low physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means </t>
-        </is>
-      </c>
+      <c r="G59" s="3" t="n"/>
       <c r="H59" s="3" t="n"/>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t xml:space="preserve">Low physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means </t>
         </is>
       </c>
       <c r="J59" s="3" t="n"/>
       <c r="K59" s="3" t="n"/>
-      <c r="L59" s="3" t="n"/>
-      <c r="M59" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="L59" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="M59" s="3" t="n"/>
       <c r="N59" s="3" t="n"/>
       <c r="O59" s="3" t="n"/>
-      <c r="P59" s="3" t="n"/>
+      <c r="P59" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
       <c r="Q59" s="3" t="n"/>
-      <c r="R59" s="3" t="n"/>
+      <c r="R59" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
       <c r="S59" s="3" t="n"/>
-      <c r="T59" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="T59" s="3" t="n"/>
       <c r="U59" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -4094,36 +4094,36 @@
       </c>
       <c r="E60" s="3" t="n"/>
       <c r="F60" s="3" t="n"/>
-      <c r="G60" s="3" t="inlineStr">
-        <is>
-          <t>Moderate cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="G60" s="3" t="n"/>
       <c r="H60" s="3" t="n"/>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Moderate cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J60" s="3" t="n"/>
       <c r="K60" s="3" t="n"/>
-      <c r="L60" s="3" t="n"/>
-      <c r="M60" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="L60" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="M60" s="3" t="n"/>
       <c r="N60" s="3" t="n"/>
       <c r="O60" s="3" t="n"/>
-      <c r="P60" s="3" t="n"/>
+      <c r="P60" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
       <c r="Q60" s="3" t="n"/>
-      <c r="R60" s="3" t="n"/>
+      <c r="R60" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
       <c r="S60" s="3" t="n"/>
-      <c r="T60" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="T60" s="3" t="n"/>
       <c r="U60" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -4154,36 +4154,36 @@
       </c>
       <c r="E61" s="3" t="n"/>
       <c r="F61" s="3" t="n"/>
-      <c r="G61" s="3" t="inlineStr">
-        <is>
-          <t>Moderate emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="G61" s="3" t="n"/>
       <c r="H61" s="3" t="n"/>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Moderate emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J61" s="3" t="n"/>
       <c r="K61" s="3" t="n"/>
-      <c r="L61" s="3" t="n"/>
-      <c r="M61" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="L61" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="M61" s="3" t="n"/>
       <c r="N61" s="3" t="n"/>
       <c r="O61" s="3" t="n"/>
-      <c r="P61" s="3" t="n"/>
+      <c r="P61" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
       <c r="Q61" s="3" t="n"/>
-      <c r="R61" s="3" t="n"/>
+      <c r="R61" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
       <c r="S61" s="3" t="n"/>
-      <c r="T61" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="T61" s="3" t="n"/>
       <c r="U61" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -4214,36 +4214,36 @@
       </c>
       <c r="E62" s="3" t="n"/>
       <c r="F62" s="3" t="n"/>
-      <c r="G62" s="3" t="inlineStr">
-        <is>
-          <t>Moderate mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="G62" s="3" t="n"/>
       <c r="H62" s="3" t="n"/>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Moderate mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J62" s="3" t="n"/>
       <c r="K62" s="3" t="n"/>
-      <c r="L62" s="3" t="n"/>
-      <c r="M62" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="L62" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="M62" s="3" t="n"/>
       <c r="N62" s="3" t="n"/>
       <c r="O62" s="3" t="n"/>
-      <c r="P62" s="3" t="n"/>
+      <c r="P62" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
       <c r="Q62" s="3" t="n"/>
-      <c r="R62" s="3" t="n"/>
+      <c r="R62" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
       <c r="S62" s="3" t="n"/>
-      <c r="T62" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="T62" s="3" t="n"/>
       <c r="U62" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -4274,36 +4274,36 @@
       </c>
       <c r="E63" s="3" t="n"/>
       <c r="F63" s="3" t="n"/>
-      <c r="G63" s="3" t="inlineStr">
-        <is>
-          <t>Moderate physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="G63" s="3" t="n"/>
       <c r="H63" s="3" t="n"/>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Moderate physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J63" s="3" t="n"/>
       <c r="K63" s="3" t="n"/>
-      <c r="L63" s="3" t="n"/>
-      <c r="M63" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="L63" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="M63" s="3" t="n"/>
       <c r="N63" s="3" t="n"/>
       <c r="O63" s="3" t="n"/>
-      <c r="P63" s="3" t="n"/>
+      <c r="P63" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
       <c r="Q63" s="3" t="n"/>
-      <c r="R63" s="3" t="n"/>
+      <c r="R63" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
       <c r="S63" s="3" t="n"/>
-      <c r="T63" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="T63" s="3" t="n"/>
       <c r="U63" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -4337,41 +4337,41 @@
           <t>BCI engagement</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr">
+      <c r="F64" s="2" t="n"/>
+      <c r="G64" s="2" t="inlineStr">
         <is>
           <t>Includes mental activities and behaviours.</t>
         </is>
       </c>
-      <c r="G64" s="2" t="n"/>
       <c r="H64" s="2" t="inlineStr">
         <is>
           <t>process</t>
         </is>
       </c>
-      <c r="I64" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I64" s="2" t="n"/>
       <c r="J64" s="2" t="n"/>
       <c r="K64" s="2" t="n"/>
-      <c r="L64" s="2" t="n"/>
-      <c r="M64" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M64" s="2" t="n"/>
       <c r="N64" s="2" t="n"/>
       <c r="O64" s="2" t="n"/>
-      <c r="P64" s="2" t="n"/>
+      <c r="P64" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW; PS</t>
+        </is>
+      </c>
       <c r="Q64" s="2" t="n"/>
-      <c r="R64" s="2" t="n"/>
+      <c r="R64" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S64" s="2" t="n"/>
-      <c r="T64" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW; PS</t>
-        </is>
-      </c>
+      <c r="T64" s="2" t="n"/>
       <c r="U64" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -4404,34 +4404,34 @@
       <c r="F65" s="2" t="n"/>
       <c r="G65" s="2" t="n"/>
       <c r="H65" s="2" t="n"/>
-      <c r="I65" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I65" s="2" t="n"/>
       <c r="J65" s="2" t="n"/>
       <c r="K65" s="2" t="n"/>
-      <c r="L65" s="2" t="n"/>
-      <c r="M65" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M65" s="2" t="n"/>
       <c r="N65" s="2" t="n"/>
       <c r="O65" s="2" t="n"/>
-      <c r="P65" s="2" t="n"/>
+      <c r="P65" s="2" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
       <c r="Q65" s="2" t="inlineStr">
         <is>
           <t>The extend to someone interacts with an intervention, including their cognitive, emotional and behavioural response (e.g., attending intervention session) to the intervention itself.</t>
         </is>
       </c>
-      <c r="R65" s="2" t="n"/>
+      <c r="R65" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S65" s="2" t="n"/>
-      <c r="T65" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="T65" s="2" t="n"/>
       <c r="U65" s="2" t="n">
         <v>0</v>
       </c>
@@ -4466,30 +4466,30 @@
       <c r="F66" s="2" t="n"/>
       <c r="G66" s="2" t="n"/>
       <c r="H66" s="2" t="n"/>
-      <c r="I66" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I66" s="2" t="n"/>
       <c r="J66" s="2" t="n"/>
       <c r="K66" s="2" t="n"/>
-      <c r="L66" s="2" t="n"/>
-      <c r="M66" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M66" s="2" t="n"/>
       <c r="N66" s="2" t="n"/>
       <c r="O66" s="2" t="n"/>
-      <c r="P66" s="2" t="n"/>
+      <c r="P66" s="2" t="inlineStr">
+        <is>
+          <t>JH</t>
+        </is>
+      </c>
       <c r="Q66" s="2" t="n"/>
-      <c r="R66" s="2" t="n"/>
+      <c r="R66" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S66" s="2" t="n"/>
-      <c r="T66" s="2" t="inlineStr">
-        <is>
-          <t>JH</t>
-        </is>
-      </c>
+      <c r="T66" s="2" t="n"/>
       <c r="U66" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -4519,41 +4519,41 @@
         </is>
       </c>
       <c r="E67" s="2" t="n"/>
-      <c r="F67" s="2" t="inlineStr">
+      <c r="F67" s="2" t="n"/>
+      <c r="G67" s="2" t="inlineStr">
         <is>
           <t>This is intended to provide a user-friendly way of representing the way in which processes are manifest. This is somewhat similar to, but not the same as, the class 'specifically dependent continuant' in Basic Formal Ontology which provides a way of representing features of material entities such as age and size. It is formally equivalent to process profile in Basic Formal Ontology.</t>
         </is>
       </c>
-      <c r="G67" s="2" t="n"/>
       <c r="H67" s="2" t="n"/>
-      <c r="I67" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I67" s="2" t="n"/>
       <c r="J67" s="2" t="n"/>
       <c r="K67" s="2" t="n"/>
-      <c r="L67" s="2" t="n"/>
-      <c r="M67" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M67" s="2" t="n"/>
       <c r="N67" s="2" t="n"/>
       <c r="O67" s="2" t="n"/>
-      <c r="P67" s="2" t="n"/>
+      <c r="P67" s="2" t="inlineStr">
+        <is>
+          <t>JH</t>
+        </is>
+      </c>
       <c r="Q67" s="2" t="inlineStr">
         <is>
           <t>An attribute of a process.</t>
         </is>
       </c>
-      <c r="R67" s="2" t="n"/>
+      <c r="R67" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S67" s="2" t="n"/>
-      <c r="T67" s="2" t="inlineStr">
-        <is>
-          <t>JH</t>
-        </is>
-      </c>
+      <c r="T67" s="2" t="n"/>
       <c r="U67" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -4577,7 +4577,7 @@
           <t>entity</t>
         </is>
       </c>
-      <c r="M68" t="inlineStr">
+      <c r="R68" t="inlineStr">
         <is>
           <t>External</t>
         </is>
@@ -4611,30 +4611,30 @@
       <c r="F69" s="2" t="n"/>
       <c r="G69" s="2" t="n"/>
       <c r="H69" s="2" t="n"/>
-      <c r="I69" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="I69" s="2" t="n"/>
       <c r="J69" s="2" t="n"/>
       <c r="K69" s="2" t="n"/>
-      <c r="L69" s="2" t="n"/>
-      <c r="M69" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="n"/>
       <c r="N69" s="2" t="n"/>
       <c r="O69" s="2" t="n"/>
-      <c r="P69" s="2" t="n"/>
+      <c r="P69" s="2" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
       <c r="Q69" s="2" t="n"/>
-      <c r="R69" s="2" t="n"/>
+      <c r="R69" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="S69" s="2" t="n"/>
-      <c r="T69" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="T69" s="2" t="n"/>
       <c r="U69" s="2" t="inlineStr">
         <is>
           <t>0</t>

</xml_diff>

<commit_message>
Update intervention evaluation study risk of bias or error in BCIO_Upper_Defs.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
@@ -1430,34 +1430,34 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>BCIO:020000</t>
+          <t>BCIO:006000</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention evaluation study risk of bias or error</t>
+          <t>behaviour change intervention mechanism of action</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>An information content entity that is about the likelihood of the BCI evaluation finding misrepresenting the outcome behaviour.</t>
+          <t xml:space="preserve">A process that is causally active in the relationship between a BCI scenario and its outcome behaviour. </t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>information content entity</t>
+          <t>process</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>BCI evaluation study risk of bias or error</t>
+          <t>BCI mechanism of action; MOA; BCI MOA</t>
         </is>
       </c>
       <c r="F15" s="2" t="n"/>
       <c r="G15" s="2" t="n"/>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>information content entity</t>
+          <t>process</t>
         </is>
       </c>
       <c r="I15" s="2" t="n"/>
@@ -1473,7 +1473,7 @@
       <c r="O15" s="2" t="n"/>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>JH; RW</t>
+          <t>PS; JH; RW</t>
         </is>
       </c>
       <c r="Q15" s="2" t="n"/>
@@ -1494,27 +1494,27 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>BCIO:006000</t>
+          <t>BCIO:011000</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention mechanism of action</t>
+          <t>behaviour change intervention mode of delivery</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A process that is causally active in the relationship between a BCI scenario and its outcome behaviour. </t>
+          <t>An attribute of a BCI delivery that is the physical or informational medium through which a BCI is provided.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>process</t>
+          <t>BCI attribute</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>BCI mechanism of action; MOA; BCI MOA</t>
+          <t>BCI mode of delivery; BCI MOD; MOD</t>
         </is>
       </c>
       <c r="F16" s="2" t="n"/>
@@ -1537,7 +1537,7 @@
       <c r="O16" s="2" t="n"/>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>PS; JH; RW</t>
+          <t>JH; RW</t>
         </is>
       </c>
       <c r="Q16" s="2" t="n"/>
@@ -1558,36 +1558,32 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>BCIO:011000</t>
+          <t>BCIO:002000</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention mode of delivery</t>
+          <t>behaviour change intervention outcome behaviour</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>An attribute of a BCI delivery that is the physical or informational medium through which a BCI is provided.</t>
+          <t>Human behaviour that is an intervention outcome.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>BCI attribute</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>BCI mode of delivery; BCI MOD; MOD</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="n"/>
+          <t>individual human behaviour</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>'individual human behaviour' AND 'intervention outcome'</t>
+        </is>
+      </c>
       <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
+      <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="n"/>
       <c r="J17" s="2" t="n"/>
       <c r="K17" s="2" t="n"/>
@@ -1601,7 +1597,7 @@
       <c r="O17" s="2" t="n"/>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>JH; RW</t>
+          <t>JH; BG; PS</t>
         </is>
       </c>
       <c r="Q17" s="2" t="n"/>
@@ -1622,32 +1618,40 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>BCIO:002000</t>
+          <t>BCIO:025000</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention outcome behaviour</t>
+          <t>behaviour change intervention outcome estimate</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Human behaviour that is an intervention outcome.</t>
+          <t>A BCI evaluation finding that is about an outcome behaviour.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>individual human behaviour</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>'individual human behaviour' AND 'intervention outcome'</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="n"/>
+          <t>behaviour change intervention evaluation finding</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>BCI outcome estimate</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>This includes as subclasses 1) type of outcome estimate (e.g. mean, percentage), 2) value of outcome estimate (e.g. 1.5 cigs per day, 23%), 3) uncertainty estimate type (e.g. 95% CI), and 4) uncertainty estimate value (e.g. 12.0%-45.0%).</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>information content entoty</t>
+        </is>
+      </c>
       <c r="I18" s="2" t="n"/>
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
@@ -1661,7 +1665,7 @@
       <c r="O18" s="2" t="n"/>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>JH; BG; PS</t>
+          <t>JH; RW</t>
         </is>
       </c>
       <c r="Q18" s="2" t="n"/>
@@ -1682,40 +1686,32 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>BCIO:025000</t>
+          <t>BCIO:026000</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention outcome estimate</t>
+          <t>behaviour change intervention physical setting</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>A BCI evaluation finding that is about an outcome behaviour.</t>
+          <t>A physical environment in which a BCI is delivered.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention evaluation finding</t>
+          <t>environmental system</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>BCI outcome estimate</t>
+          <t>BCI physical setting</t>
         </is>
       </c>
       <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>This includes as subclasses 1) type of outcome estimate (e.g. mean, percentage), 2) value of outcome estimate (e.g. 1.5 cigs per day, 23%), 3) uncertainty estimate type (e.g. 95% CI), and 4) uncertainty estimate value (e.g. 12.0%-45.0%).</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>information content entoty</t>
-        </is>
-      </c>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
       <c r="I19" s="2" t="n"/>
       <c r="J19" s="2" t="n"/>
       <c r="K19" s="2" t="n"/>
@@ -1750,27 +1746,27 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>BCIO:026000</t>
+          <t>BCIO:015000</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention physical setting</t>
+          <t>behaviour change intervention population</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>A physical environment in which a BCI is delivered.</t>
+          <t>An intervention population who are exposed to a behaviour change intervention.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>environmental system</t>
+          <t>intervention population</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>BCI physical setting</t>
+          <t>BCI population</t>
         </is>
       </c>
       <c r="F20" s="2" t="n"/>
@@ -1789,7 +1785,7 @@
       <c r="O20" s="2" t="n"/>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>JH; RW</t>
+          <t>JH; RW; PS</t>
         </is>
       </c>
       <c r="Q20" s="2" t="n"/>
@@ -1810,34 +1806,38 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>BCIO:015000</t>
+          <t>BCIO:001000</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention population</t>
+          <t>behaviour change intervention scenario</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>An intervention population who are exposed to a behaviour change intervention.</t>
+          <t>A planned process in which a BCI is applied in a given context, including BCI engagement and outcome behaviour.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>intervention population</t>
+          <t>planned process</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>BCI population</t>
+          <t>BCI scenario</t>
         </is>
       </c>
       <c r="F21" s="2" t="n"/>
       <c r="G21" s="2" t="n"/>
       <c r="H21" s="2" t="n"/>
       <c r="I21" s="2" t="n"/>
-      <c r="J21" s="2" t="n"/>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>behaviour change intervention outcome behaviour</t>
+        </is>
+      </c>
       <c r="K21" s="2" t="n"/>
       <c r="L21" s="2" t="inlineStr">
         <is>
@@ -1849,7 +1849,7 @@
       <c r="O21" s="2" t="n"/>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>JH; RW; PS</t>
+          <t>JH; RW</t>
         </is>
       </c>
       <c r="Q21" s="2" t="n"/>
@@ -1870,38 +1870,34 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>BCIO:001000</t>
+          <t>BCIO:028000</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention scenario</t>
+          <t>behaviour change intervention scenario plan</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>A planned process in which a BCI is applied in a given context, including BCI engagement and outcome behaviour.</t>
+          <t>A plan that is realized in a BCI scenario process.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>planned process</t>
+          <t>plan</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>BCI scenario</t>
+          <t>BCI scenario plan</t>
         </is>
       </c>
       <c r="F22" s="2" t="n"/>
       <c r="G22" s="2" t="n"/>
       <c r="H22" s="2" t="n"/>
       <c r="I22" s="2" t="n"/>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>behaviour change intervention outcome behaviour</t>
-        </is>
-      </c>
+      <c r="J22" s="2" t="n"/>
       <c r="K22" s="2" t="n"/>
       <c r="L22" s="2" t="inlineStr">
         <is>
@@ -1934,27 +1930,27 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>BCIO:028000</t>
+          <t>BCIO:027000</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention scenario plan</t>
+          <t>behaviour change intervention scenario report</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>A plan that is realized in a BCI scenario process.</t>
+          <t>A report that describes a BCI scenario.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>plan</t>
+          <t>report</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>BCI scenario plan</t>
+          <t>BCI scenario report</t>
         </is>
       </c>
       <c r="F23" s="2" t="n"/>
@@ -1994,31 +1990,35 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>BCIO:027000</t>
+          <t>BCIO:014000</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention scenario report</t>
+          <t>behaviour change intervention setting</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>A report that describes a BCI scenario.</t>
+          <t xml:space="preserve">An aggregate of entities that form the environment in which a BCI is provided. </t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>report</t>
+          <t>object aggregate</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>BCI scenario report</t>
+          <t>BCI setting</t>
         </is>
       </c>
       <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Includes as parts social setting and physical setting.</t>
+        </is>
+      </c>
       <c r="H24" s="2" t="n"/>
       <c r="I24" s="2" t="n"/>
       <c r="J24" s="2" t="n"/>
@@ -2054,35 +2054,31 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>BCIO:014000</t>
+          <t>BCIO:029000</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention setting</t>
+          <t>behaviour change intervention social setting</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">An aggregate of entities that form the environment in which a BCI is provided. </t>
+          <t>An aggregate of people with whom a BCI population interacts.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>object aggregate</t>
+          <t>human population</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>BCI setting</t>
+          <t>BCI social setting</t>
         </is>
       </c>
       <c r="F25" s="2" t="n"/>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>Includes as parts social setting and physical setting.</t>
-        </is>
-      </c>
+      <c r="G25" s="2" t="n"/>
       <c r="H25" s="2" t="n"/>
       <c r="I25" s="2" t="n"/>
       <c r="J25" s="2" t="n"/>
@@ -2118,31 +2114,35 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>BCIO:029000</t>
+          <t>BCIO:010000</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention social setting</t>
+          <t>behaviour change intervention source</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>An aggregate of people with whom a BCI population interacts.</t>
+          <t>A role played by a person, population or organisation that provides a BCI.</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>human population</t>
+          <t>role</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>BCI social setting</t>
+          <t>BCI source</t>
         </is>
       </c>
       <c r="F26" s="2" t="n"/>
-      <c r="G26" s="2" t="n"/>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>This includes individual people, groups of people, and organisations.</t>
+        </is>
+      </c>
       <c r="H26" s="2" t="n"/>
       <c r="I26" s="2" t="n"/>
       <c r="J26" s="2" t="n"/>
@@ -2178,33 +2178,33 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>BCIO:010000</t>
+          <t>BCIO:030000</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention source</t>
+          <t>behaviour change intervention study investigator role</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>A role played by a person, population or organisation that provides a BCI.</t>
+          <t>A researcher role played by a person that contributes substantively to production or reporting of a BCI evaluation study.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>role</t>
+          <t>researcher role</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>BCI source</t>
+          <t>BCI study investigator</t>
         </is>
       </c>
       <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>This includes individual people, groups of people, and organisations.</t>
+          <t xml:space="preserve">What counts as substantively is subject to judgement. The level and nature of the contribution can be defined using the CReDiT taxonomy (https://casrai.org/credit/). </t>
         </is>
       </c>
       <c r="H27" s="2" t="n"/>
@@ -2242,35 +2242,31 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>BCIO:030000</t>
+          <t>BCIO:031000</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention study investigator role</t>
+          <t>behaviour change intervention study sample</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>A researcher role played by a person that contributes substantively to production or reporting of a BCI evaluation study.</t>
+          <t>A research study sample whose behaviour is studied in a BCI evaluation study.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>researcher role</t>
+          <t>research study participants</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>BCI study investigator</t>
+          <t>BCI study sample</t>
         </is>
       </c>
       <c r="F28" s="2" t="n"/>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">What counts as substantively is subject to judgement. The level and nature of the contribution can be defined using the CReDiT taxonomy (https://casrai.org/credit/). </t>
-        </is>
-      </c>
+      <c r="G28" s="2" t="n"/>
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="2" t="n"/>
       <c r="J28" s="2" t="n"/>
@@ -2285,7 +2281,7 @@
       <c r="O28" s="2" t="n"/>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>JH; RW</t>
+          <t>JH; RW; PS</t>
         </is>
       </c>
       <c r="Q28" s="2" t="n"/>
@@ -2306,31 +2302,35 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>BCIO:031000</t>
+          <t>BCIO:044000</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention study sample</t>
+          <t>behaviour change intervention style of delivery</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>A research study sample whose behaviour is studied in a BCI evaluation study.</t>
+          <t>A communication style that is an attribute of a BCI content communication process.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>research study participants</t>
+          <t>communication style</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>BCI study sample</t>
+          <t>BCI style of delivery</t>
         </is>
       </c>
       <c r="F29" s="2" t="n"/>
-      <c r="G29" s="2" t="n"/>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>An example is cold and distant vs. warm and accepting.</t>
+        </is>
+      </c>
       <c r="H29" s="2" t="n"/>
       <c r="I29" s="2" t="n"/>
       <c r="J29" s="2" t="n"/>
@@ -2345,7 +2345,7 @@
       <c r="O29" s="2" t="n"/>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>JH; RW; PS</t>
+          <t>JH; RW</t>
         </is>
       </c>
       <c r="Q29" s="2" t="n"/>
@@ -2366,37 +2366,41 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>BCIO:044000</t>
+          <t>BCIO:032000</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention style of delivery</t>
+          <t>behaviour change intervention tailoring</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>A communication style that is an attribute of a BCI content communication process.</t>
+          <t>A BCI attribute in which the content or delivery of a BCI for some member of the BCI population varies according to their characteristics or setting.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>communication style</t>
+          <t>BCI attribute</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>BCI style of delivery</t>
+          <t>BCI tailoring</t>
         </is>
       </c>
       <c r="F30" s="2" t="n"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>An example is cold and distant vs. warm and accepting.</t>
+          <t>Tailoring the dose of pharmacotherapy for smoking cessation to the prior level of nicotine dependence of the smoker (static) or to the smokers' current strength of urges to smoke during a quit attempt (dynamic).</t>
         </is>
       </c>
       <c r="H30" s="2" t="n"/>
-      <c r="I30" s="2" t="n"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Tailoring can be static (i.e., conducted before intervention delivery in a case case), or dynamic (i.e., conducted one or more times after the intervention has started in a given case based on population or setting characteristics present at that time. Population and setting characteristics include the historical factors such as prior exposure to the intervention.</t>
+        </is>
+      </c>
       <c r="J30" s="2" t="n"/>
       <c r="K30" s="2" t="n"/>
       <c r="L30" s="2" t="inlineStr">
@@ -2412,7 +2416,11 @@
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q30" s="2" t="n"/>
+      <c r="Q30" s="2" t="inlineStr">
+        <is>
+          <t>An attribute of a behaviour change intervention (BCI) or a BCI component whereby its content or delivery is varied according to characteristics of members of the target population or setting.</t>
+        </is>
+      </c>
       <c r="R30" s="2" t="inlineStr">
         <is>
           <t>Published</t>
@@ -2430,41 +2438,33 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>BCIO:032000</t>
+          <t>BCIO:047000</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention tailoring</t>
+          <t xml:space="preserve">behaviour change intervention temporal context </t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>A BCI attribute in which the content or delivery of a BCI for some member of the BCI population varies according to their characteristics or setting.</t>
+          <t>The intervention temporal context where the process is the behaviour change intervention</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>BCI attribute</t>
+          <t>intervention temporal context</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>BCI tailoring</t>
+          <t>BCI temporal context</t>
         </is>
       </c>
       <c r="F31" s="2" t="n"/>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>Tailoring the dose of pharmacotherapy for smoking cessation to the prior level of nicotine dependence of the smoker (static) or to the smokers' current strength of urges to smoke during a quit attempt (dynamic).</t>
-        </is>
-      </c>
+      <c r="G31" s="2" t="n"/>
       <c r="H31" s="2" t="n"/>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>Tailoring can be static (i.e., conducted before intervention delivery in a case case), or dynamic (i.e., conducted one or more times after the intervention has started in a given case based on population or setting characteristics present at that time. Population and setting characteristics include the historical factors such as prior exposure to the intervention.</t>
-        </is>
-      </c>
+      <c r="I31" s="2" t="n"/>
       <c r="J31" s="2" t="n"/>
       <c r="K31" s="2" t="n"/>
       <c r="L31" s="2" t="inlineStr">
@@ -2480,11 +2480,7 @@
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q31" s="2" t="inlineStr">
-        <is>
-          <t>An attribute of a behaviour change intervention (BCI) or a BCI component whereby its content or delivery is varied according to characteristics of members of the target population or setting.</t>
-        </is>
-      </c>
+      <c r="Q31" s="2" t="n"/>
       <c r="R31" s="2" t="inlineStr">
         <is>
           <t>Published</t>
@@ -2502,27 +2498,27 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>BCIO:047000</t>
+          <t>BCIO:047001</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">behaviour change intervention temporal context </t>
+          <t>behaviour change intervention temporal context event</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>The intervention temporal context where the process is the behaviour change intervention</t>
+          <t xml:space="preserve">An event which occurs during a behaviour change intervention temporal context. </t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>intervention temporal context</t>
+          <t>behaviour change intervention temporal context</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal context</t>
+          <t>BCI temporal context event</t>
         </is>
       </c>
       <c r="F32" s="2" t="n"/>
@@ -2562,27 +2558,27 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>BCIO:047001</t>
+          <t>BCIO:033000</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention temporal context event</t>
+          <t>behaviour change technique</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">An event which occurs during a behaviour change intervention temporal context. </t>
+          <t>A &lt;planned process&gt; that is the smallest part of BCI content that is observable, replicable and on its own has the potential to bring about behaviour change.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>behaviour change intervention temporal context</t>
+          <t>planned process</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>BCI temporal context event</t>
+          <t>BCT</t>
         </is>
       </c>
       <c r="F33" s="2" t="n"/>
@@ -2601,7 +2597,7 @@
       <c r="O33" s="2" t="n"/>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>JH; RW</t>
+          <t>JH; RW; PS</t>
         </is>
       </c>
       <c r="Q33" s="2" t="n"/>
@@ -2622,29 +2618,25 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>BCIO:033000</t>
+          <t>BCIO:044003</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>behaviour change technique</t>
+          <t>communication process attribute</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>A &lt;planned process&gt; that is the smallest part of BCI content that is observable, replicable and on its own has the potential to bring about behaviour change.</t>
+          <t>An attribute of a communication process.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>planned process</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>BCT</t>
-        </is>
-      </c>
+          <t>process attribute</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="n"/>
       <c r="F34" s="2" t="n"/>
       <c r="G34" s="2" t="n"/>
       <c r="H34" s="2" t="n"/>
@@ -2661,7 +2653,7 @@
       <c r="O34" s="2" t="n"/>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>JH; RW; PS</t>
+          <t>JH; PS</t>
         </is>
       </c>
       <c r="Q34" s="2" t="n"/>
@@ -2682,22 +2674,22 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>BCIO:044003</t>
+          <t>BCIO:044004</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
+          <t>communication style</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>A particular manner of communicating aimed at inducing or avoiding certain kinds of responses in others, or demonstrating certain characteristics of the initiator.</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
           <t>communication process attribute</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>An attribute of a communication process.</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>process attribute</t>
         </is>
       </c>
       <c r="E35" s="2" t="n"/>
@@ -2717,7 +2709,7 @@
       <c r="O35" s="2" t="n"/>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>JH; PS</t>
+          <t>JH</t>
         </is>
       </c>
       <c r="Q35" s="2" t="n"/>
@@ -2736,80 +2728,84 @@
       <c r="V35" s="2" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:044004</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>communication style</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>A particular manner of communicating aimed at inducing or avoiding certain kinds of responses in others, or demonstrating certain characteristics of the initiator.</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>communication process attribute</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
-      <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="n"/>
-      <c r="J36" s="2" t="n"/>
-      <c r="K36" s="2" t="n"/>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
-      <c r="M36" s="2" t="n"/>
-      <c r="N36" s="2" t="n"/>
-      <c r="O36" s="2" t="n"/>
-      <c r="P36" s="2" t="inlineStr">
-        <is>
-          <t>JH</t>
-        </is>
-      </c>
-      <c r="Q36" s="2" t="n"/>
-      <c r="R36" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S36" s="2" t="n"/>
-      <c r="T36" s="2" t="n"/>
-      <c r="U36" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V36" s="2" t="n"/>
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:050462</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>high cognitive exertion expended on a behaviour</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Cognitive exertion expended on a behaviour that is high.</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>cognitive exertion expended on a behaviour</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="n"/>
+      <c r="F36" s="3" t="n"/>
+      <c r="G36" s="3" t="n"/>
+      <c r="H36" s="3" t="n"/>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>High cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="n"/>
+      <c r="K36" s="3" t="n"/>
+      <c r="L36" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="M36" s="3" t="n"/>
+      <c r="N36" s="3" t="n"/>
+      <c r="O36" s="3" t="n"/>
+      <c r="P36" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="Q36" s="3" t="n"/>
+      <c r="R36" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="S36" s="3" t="n"/>
+      <c r="T36" s="3" t="n"/>
+      <c r="U36" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="V36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050462</t>
+          <t>BCIO:050463</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>high cognitive exertion expended on a behaviour</t>
+          <t>high emotional management  exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Cognitive exertion expended on a behaviour that is high.</t>
+          <t>Emotional management exertion expended on a behaviour that is high.</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>cognitive exertion expended on a behaviour</t>
+          <t>emotional management exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E37" s="3" t="n"/>
@@ -2818,7 +2814,7 @@
       <c r="H37" s="3" t="n"/>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>High cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
+          <t>High emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J37" s="3" t="n"/>
@@ -2854,22 +2850,22 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050463</t>
+          <t>BCIO:050464</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>high emotional management  exertion expended on a behaviour</t>
+          <t>high mental exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Emotional management exertion expended on a behaviour that is high.</t>
+          <t>Mental exertion expended on a behaviour that is high.</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>emotional management exertion expended on a behaviour</t>
+          <t>mental exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E38" s="3" t="n"/>
@@ -2878,7 +2874,7 @@
       <c r="H38" s="3" t="n"/>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>High emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
+          <t>High mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J38" s="3" t="n"/>
@@ -2914,22 +2910,22 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050464</t>
+          <t>BCIO:050465</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>high mental exertion expended on a behaviour</t>
+          <t>high physical exertion expended on behaviour</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Mental exertion expended on a behaviour that is high.</t>
+          <t>Physical exertion expended on a behaviour that is high</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>mental exertion expended on a behaviour</t>
+          <t>physical exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E39" s="3" t="n"/>
@@ -2938,7 +2934,7 @@
       <c r="H39" s="3" t="n"/>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>High mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
+          <t>High physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J39" s="3" t="n"/>
@@ -2974,38 +2970,38 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050465</t>
+          <t>BCIO:042000</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>high physical exertion expended on behaviour</t>
+          <t>human behaviour</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Physical exertion expended on a behaviour that is high</t>
+          <t>A process that is an individual human behaviour or a population behaviour.</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>physical exertion expended on a behaviour</t>
+          <t>process</t>
         </is>
       </c>
       <c r="E40" s="3" t="n"/>
-      <c r="F40" s="3" t="n"/>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>"individual human behaviour" OR "population behaviour"</t>
+        </is>
+      </c>
       <c r="G40" s="3" t="n"/>
       <c r="H40" s="3" t="n"/>
-      <c r="I40" s="3" t="inlineStr">
-        <is>
-          <t>High physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what high exertion means based on the measurement you use).</t>
-        </is>
-      </c>
+      <c r="I40" s="3" t="n"/>
       <c r="J40" s="3" t="n"/>
       <c r="K40" s="3" t="n"/>
       <c r="L40" s="3" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Upper level</t>
         </is>
       </c>
       <c r="M40" s="3" t="n"/>
@@ -3013,7 +3009,7 @@
       <c r="O40" s="3" t="n"/>
       <c r="P40" s="3" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>BG; PS</t>
         </is>
       </c>
       <c r="Q40" s="3" t="n"/>
@@ -3026,90 +3022,86 @@
       <c r="T40" s="3" t="n"/>
       <c r="U40" s="3" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>0</t>
         </is>
       </c>
       <c r="V40" s="3" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:042000</t>
-        </is>
-      </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>human behaviour</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>A process that is an individual human behaviour or a population behaviour.</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="n"/>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>"individual human behaviour" OR "population behaviour"</t>
-        </is>
-      </c>
-      <c r="G41" s="3" t="n"/>
-      <c r="H41" s="3" t="n"/>
-      <c r="I41" s="3" t="n"/>
-      <c r="J41" s="3" t="n"/>
-      <c r="K41" s="3" t="n"/>
-      <c r="L41" s="3" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
-      <c r="M41" s="3" t="n"/>
-      <c r="N41" s="3" t="n"/>
-      <c r="O41" s="3" t="n"/>
-      <c r="P41" s="3" t="inlineStr">
-        <is>
-          <t>BG; PS</t>
-        </is>
-      </c>
-      <c r="Q41" s="3" t="n"/>
-      <c r="R41" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="S41" s="3" t="n"/>
-      <c r="T41" s="3" t="n"/>
-      <c r="U41" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V41" s="3" t="n"/>
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:041000</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>human population</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>An object aggregate that consists of two or more people.</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>object aggregate</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2" t="n"/>
+      <c r="H41" s="2" t="n"/>
+      <c r="I41" s="2" t="n"/>
+      <c r="J41" s="2" t="n"/>
+      <c r="K41" s="2" t="n"/>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="n"/>
+      <c r="N41" s="2" t="n"/>
+      <c r="O41" s="2" t="n"/>
+      <c r="P41" s="2" t="inlineStr">
+        <is>
+          <t>JH; AW</t>
+        </is>
+      </c>
+      <c r="Q41" s="2" t="n"/>
+      <c r="R41" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="S41" s="2" t="n"/>
+      <c r="T41" s="2" t="n"/>
+      <c r="U41" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>BCIO:041000</t>
+          <t>BCIO:040000</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>human population</t>
+          <t>individual human activity</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>An object aggregate that consists of two or more people.</t>
+          <t>A process that is produced by a person.</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>object aggregate</t>
+          <t>process</t>
         </is>
       </c>
       <c r="E42" s="2" t="n"/>
@@ -3129,7 +3121,7 @@
       <c r="O42" s="2" t="n"/>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>JH; AW</t>
+          <t>JH</t>
         </is>
       </c>
       <c r="Q42" s="2" t="n"/>
@@ -3150,27 +3142,35 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>BCIO:040000</t>
+          <t>BCIO:036000</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>individual human activity</t>
+          <t>individual human behaviour</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>A process that is produced by a person.</t>
+          <t xml:space="preserve">A bodily process of a human that involves co-ordinated contraction of striated muscles controlled by the brain. </t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="n"/>
+          <t>bodily process</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>human behaviour</t>
+        </is>
+      </c>
       <c r="F43" s="2" t="n"/>
-      <c r="G43" s="2" t="n"/>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Also referred to in definitions as human behaviour or just behaviour.</t>
+        </is>
+      </c>
       <c r="H43" s="2" t="n"/>
       <c r="I43" s="2" t="n"/>
       <c r="J43" s="2" t="n"/>
@@ -3206,33 +3206,29 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>BCIO:036000</t>
+          <t>BCIO:037000</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>individual human behaviour</t>
+          <t>intervention</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A bodily process of a human that involves co-ordinated contraction of striated muscles controlled by the brain. </t>
+          <t>A planned process that has the aim of influencing an outcome.</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>bodily process</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>human behaviour</t>
-        </is>
-      </c>
+          <t>planned process</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="n"/>
       <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Also referred to in definitions as human behaviour or just behaviour.</t>
+          <t>Examples of interventions are putting health warnings on cigarette packets, providing free stop smoking services and banning smoking in public places.</t>
         </is>
       </c>
       <c r="H44" s="2" t="n"/>
@@ -3249,7 +3245,7 @@
       <c r="O44" s="2" t="n"/>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>JH</t>
+          <t>JH; RW</t>
         </is>
       </c>
       <c r="Q44" s="2" t="n"/>
@@ -3268,211 +3264,207 @@
       <c r="V44" s="2" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:037000</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>intervention</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>A planned process that has the aim of influencing an outcome.</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:051010</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>intervention attribute</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>A &lt;process attribute&gt; whose bearer is an intervention.</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>process attribute</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="n"/>
+      <c r="F45" s="4" t="n"/>
+      <c r="G45" s="4" t="n"/>
+      <c r="H45" s="4" t="n"/>
+      <c r="I45" s="4" t="n"/>
+      <c r="J45" s="4" t="n"/>
+      <c r="K45" s="4" t="n"/>
+      <c r="L45" s="4" t="n"/>
+      <c r="M45" s="4" t="n"/>
+      <c r="N45" s="4" t="n"/>
+      <c r="O45" s="4" t="n"/>
+      <c r="P45" s="4" t="n"/>
+      <c r="Q45" s="4" t="n"/>
+      <c r="R45" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="S45" s="4" t="n"/>
+      <c r="T45" s="4" t="n"/>
+      <c r="U45" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V45" s="4" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:046000</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>intervention content</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>A planned process that is part of an intervention and is intended to be causally active in influencing the intervention outcome.</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>planned process</t>
         </is>
       </c>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="2" t="n"/>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>Examples of interventions are putting health warnings on cigarette packets, providing free stop smoking services and banning smoking in public places.</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="n"/>
-      <c r="I45" s="2" t="n"/>
-      <c r="J45" s="2" t="n"/>
-      <c r="K45" s="2" t="n"/>
-      <c r="L45" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
-      <c r="M45" s="2" t="n"/>
-      <c r="N45" s="2" t="n"/>
-      <c r="O45" s="2" t="n"/>
-      <c r="P45" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW</t>
-        </is>
-      </c>
-      <c r="Q45" s="2" t="n"/>
-      <c r="R45" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S45" s="2" t="n"/>
-      <c r="T45" s="2" t="n"/>
-      <c r="U45" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V45" s="2" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:051010</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>intervention attribute</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>A &lt;process attribute&gt; whose bearer is an intervention.</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>process attribute</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="n"/>
-      <c r="F46" s="4" t="n"/>
-      <c r="G46" s="4" t="n"/>
-      <c r="H46" s="4" t="n"/>
-      <c r="I46" s="4" t="n"/>
-      <c r="J46" s="4" t="n"/>
-      <c r="K46" s="4" t="n"/>
-      <c r="L46" s="4" t="n"/>
-      <c r="M46" s="4" t="n"/>
-      <c r="N46" s="4" t="n"/>
-      <c r="O46" s="4" t="n"/>
-      <c r="P46" s="4" t="n"/>
-      <c r="Q46" s="4" t="n"/>
-      <c r="R46" s="4" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="S46" s="4" t="n"/>
-      <c r="T46" s="4" t="n"/>
-      <c r="U46" s="4" t="n">
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
+      <c r="G46" s="2" t="n"/>
+      <c r="H46" s="2" t="n"/>
+      <c r="I46" s="2" t="n"/>
+      <c r="J46" s="2" t="n"/>
+      <c r="K46" s="2" t="n"/>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="n"/>
+      <c r="N46" s="2" t="n"/>
+      <c r="O46" s="2" t="n"/>
+      <c r="P46" s="2" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="Q46" s="2" t="n"/>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="S46" s="2" t="n"/>
+      <c r="T46" s="2" t="n"/>
+      <c r="U46" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>GMHO:0000253</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>intervention context</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>process context</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="U47" t="n">
         <v>0</v>
       </c>
-      <c r="V46" s="4" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:046000</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>intervention content</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>A planned process that is part of an intervention and is intended to be causally active in influencing the intervention outcome.</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:045000</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>intervention delivery</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>A planned process by which intervention content is delivered.</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>planned process</t>
         </is>
       </c>
-      <c r="E47" s="2" t="n"/>
-      <c r="F47" s="2" t="n"/>
-      <c r="G47" s="2" t="n"/>
-      <c r="H47" s="2" t="n"/>
-      <c r="I47" s="2" t="n"/>
-      <c r="J47" s="2" t="n"/>
-      <c r="K47" s="2" t="n"/>
-      <c r="L47" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
-      <c r="M47" s="2" t="n"/>
-      <c r="N47" s="2" t="n"/>
-      <c r="O47" s="2" t="n"/>
-      <c r="P47" s="2" t="inlineStr">
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
+      <c r="G48" s="2" t="n"/>
+      <c r="H48" s="2" t="n"/>
+      <c r="I48" s="2" t="n"/>
+      <c r="J48" s="2" t="n"/>
+      <c r="K48" s="2" t="n"/>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="n"/>
+      <c r="N48" s="2" t="n"/>
+      <c r="O48" s="2" t="n"/>
+      <c r="P48" s="2" t="inlineStr">
         <is>
           <t>RW</t>
         </is>
       </c>
-      <c r="Q47" s="2" t="n"/>
-      <c r="R47" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S47" s="2" t="n"/>
-      <c r="T47" s="2" t="n"/>
-      <c r="U47" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V47" s="2" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>GMHO:0000253</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>intervention context</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>process context</t>
-        </is>
-      </c>
-      <c r="R48" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="U48" t="n">
-        <v>0</v>
-      </c>
+      <c r="Q48" s="2" t="n"/>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="S48" s="2" t="n"/>
+      <c r="T48" s="2" t="n"/>
+      <c r="U48" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>BCIO:045000</t>
+          <t>BCIO:035000</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>intervention delivery</t>
+          <t>intervention evaluation finding</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>A planned process by which intervention content is delivered.</t>
+          <t>A data item that is the output of an intervention evaluation study.</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>planned process</t>
+          <t>data item</t>
         </is>
       </c>
       <c r="E49" s="2" t="n"/>
@@ -3492,7 +3484,7 @@
       <c r="O49" s="2" t="n"/>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>JH; RW</t>
         </is>
       </c>
       <c r="Q49" s="2" t="n"/>
@@ -3513,22 +3505,22 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>BCIO:035000</t>
+          <t>BCIO:038000</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>intervention evaluation finding</t>
+          <t>intervention evaluation study</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>A data item that is the output of an intervention evaluation study.</t>
+          <t>A research study that aims to assess attributes of an intervention with regards to their positive or negative value.</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>data item</t>
+          <t>research study</t>
         </is>
       </c>
       <c r="E50" s="2" t="n"/>
@@ -3569,28 +3561,36 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>BCIO:038000</t>
+          <t>BCIO:020000</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>intervention evaluation study</t>
+          <t>intervention evaluation study risk of bias or error</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>A research study that aims to assess attributes of an intervention with regards to their positive or negative value.</t>
+          <t>An information content entity that is about the likelihood of the intervention evaluation finding misrepresenting the outcome behaviour.</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>research study</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="n"/>
+          <t>information content entity</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>intervention evaluation study risk of bias or error</t>
+        </is>
+      </c>
       <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="n"/>
-      <c r="H51" s="2" t="n"/>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>information content entity</t>
+        </is>
+      </c>
       <c r="I51" s="2" t="n"/>
       <c r="J51" s="2" t="n"/>
       <c r="K51" s="2" t="n"/>

</xml_diff>

<commit_message>
Update Curation status of intervention attribute in BCIO_Upper_Defs.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
@@ -30,7 +30,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,11 +47,6 @@
         <fgColor rgb="002f4f4f"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00ffffff"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -65,12 +60,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3264,50 +3258,50 @@
       <c r="V44" s="2" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>BCIO:051010</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>intervention attribute</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>A &lt;process attribute&gt; whose bearer is an intervention.</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>process attribute</t>
         </is>
       </c>
-      <c r="E45" s="4" t="n"/>
-      <c r="F45" s="4" t="n"/>
-      <c r="G45" s="4" t="n"/>
-      <c r="H45" s="4" t="n"/>
-      <c r="I45" s="4" t="n"/>
-      <c r="J45" s="4" t="n"/>
-      <c r="K45" s="4" t="n"/>
-      <c r="L45" s="4" t="n"/>
-      <c r="M45" s="4" t="n"/>
-      <c r="N45" s="4" t="n"/>
-      <c r="O45" s="4" t="n"/>
-      <c r="P45" s="4" t="n"/>
-      <c r="Q45" s="4" t="n"/>
-      <c r="R45" s="4" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="S45" s="4" t="n"/>
-      <c r="T45" s="4" t="n"/>
-      <c r="U45" s="4" t="n">
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
+      <c r="G45" s="2" t="n"/>
+      <c r="H45" s="2" t="n"/>
+      <c r="I45" s="2" t="n"/>
+      <c r="J45" s="2" t="n"/>
+      <c r="K45" s="2" t="n"/>
+      <c r="L45" s="2" t="n"/>
+      <c r="M45" s="2" t="n"/>
+      <c r="N45" s="2" t="n"/>
+      <c r="O45" s="2" t="n"/>
+      <c r="P45" s="2" t="n"/>
+      <c r="Q45" s="2" t="n"/>
+      <c r="R45" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="S45" s="2" t="n"/>
+      <c r="T45" s="2" t="n"/>
+      <c r="U45" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="V45" s="4" t="n"/>
+      <c r="V45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add 4 terms to BCIO_Upper_Defs.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
@@ -30,7 +30,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +47,11 @@
         <fgColor rgb="002f4f4f"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ffffff"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -60,11 +65,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V69"/>
+  <dimension ref="A1:V73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3385,80 +3391,70 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:045000</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>intervention delivery</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>A planned process by which intervention content is delivered.</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>planned process</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="n"/>
-      <c r="F48" s="2" t="n"/>
-      <c r="G48" s="2" t="n"/>
-      <c r="H48" s="2" t="n"/>
-      <c r="I48" s="2" t="n"/>
-      <c r="J48" s="2" t="n"/>
-      <c r="K48" s="2" t="n"/>
-      <c r="L48" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
-      <c r="M48" s="2" t="n"/>
-      <c r="N48" s="2" t="n"/>
-      <c r="O48" s="2" t="n"/>
-      <c r="P48" s="2" t="inlineStr">
-        <is>
-          <t>RW</t>
-        </is>
-      </c>
-      <c r="Q48" s="2" t="n"/>
-      <c r="R48" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S48" s="2" t="n"/>
-      <c r="T48" s="2" t="n"/>
-      <c r="U48" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V48" s="2" t="n"/>
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:051025</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>intervention context</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>A process context in which the process is an intervention.</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>process context</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr"/>
+      <c r="F48" s="4" t="inlineStr"/>
+      <c r="G48" s="4" t="inlineStr"/>
+      <c r="H48" s="4" t="inlineStr"/>
+      <c r="I48" s="4" t="inlineStr"/>
+      <c r="J48" s="4" t="inlineStr"/>
+      <c r="K48" s="4" t="inlineStr"/>
+      <c r="L48" s="4" t="inlineStr"/>
+      <c r="M48" s="4" t="inlineStr"/>
+      <c r="N48" s="4" t="inlineStr"/>
+      <c r="O48" s="4" t="inlineStr"/>
+      <c r="P48" s="4" t="inlineStr"/>
+      <c r="Q48" s="4" t="inlineStr"/>
+      <c r="R48" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="S48" s="4" t="inlineStr"/>
+      <c r="T48" s="4" t="inlineStr"/>
+      <c r="U48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V48" s="4" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>BCIO:035000</t>
+          <t>BCIO:045000</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>intervention evaluation finding</t>
+          <t>intervention delivery</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>A data item that is the output of an intervention evaluation study.</t>
+          <t>A planned process by which intervention content is delivered.</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>data item</t>
+          <t>planned process</t>
         </is>
       </c>
       <c r="E49" s="2" t="n"/>
@@ -3478,7 +3474,7 @@
       <c r="O49" s="2" t="n"/>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>JH; RW</t>
+          <t>RW</t>
         </is>
       </c>
       <c r="Q49" s="2" t="n"/>
@@ -3499,22 +3495,22 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>BCIO:038000</t>
+          <t>BCIO:035000</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>intervention evaluation study</t>
+          <t>intervention evaluation finding</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>A research study that aims to assess attributes of an intervention with regards to their positive or negative value.</t>
+          <t>A data item that is the output of an intervention evaluation study.</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>research study</t>
+          <t>data item</t>
         </is>
       </c>
       <c r="E50" s="2" t="n"/>
@@ -3555,36 +3551,28 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>BCIO:020000</t>
+          <t>BCIO:038000</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>intervention evaluation study risk of bias or error</t>
+          <t>intervention evaluation study</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>An information content entity that is about the likelihood of the intervention evaluation finding misrepresenting the intervention outcome.</t>
+          <t>A research study that aims to assess attributes of an intervention with regards to their positive or negative value.</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>information content entity</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>intervention evaluation study risk of bias or error</t>
-        </is>
-      </c>
+          <t>research study</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="n"/>
       <c r="F51" s="2" t="n"/>
       <c r="G51" s="2" t="n"/>
-      <c r="H51" s="2" t="inlineStr">
-        <is>
-          <t>information content entity</t>
-        </is>
-      </c>
+      <c r="H51" s="2" t="n"/>
       <c r="I51" s="2" t="n"/>
       <c r="J51" s="2" t="n"/>
       <c r="K51" s="2" t="n"/>
@@ -3619,32 +3607,36 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>BCIO:039000</t>
+          <t>BCIO:020000</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>intervention outcome</t>
+          <t>intervention evaluation study risk of bias or error</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>An entity that is influenced by an intervention</t>
+          <t>An information content entity that is about the likelihood of the intervention evaluation finding misrepresenting the intervention outcome.</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>entity</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="n"/>
+          <t>information content entity</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>intervention evaluation study risk of bias or error</t>
+        </is>
+      </c>
       <c r="F52" s="2" t="n"/>
-      <c r="G52" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Includes individual human behaviour, mental activity and physiological activity. Also includes undesirable outcomes, such as treatment side effects, and unintended negative consequences of the intervention. </t>
-        </is>
-      </c>
-      <c r="H52" s="2" t="n"/>
+      <c r="G52" s="2" t="n"/>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>information content entity</t>
+        </is>
+      </c>
       <c r="I52" s="2" t="n"/>
       <c r="J52" s="2" t="n"/>
       <c r="K52" s="2" t="n"/>
@@ -3658,7 +3650,7 @@
       <c r="O52" s="2" t="n"/>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>JH</t>
+          <t>JH; RW</t>
         </is>
       </c>
       <c r="Q52" s="2" t="n"/>
@@ -3679,27 +3671,31 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>BCIO:015095</t>
+          <t>BCIO:039000</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>intervention population</t>
+          <t>intervention outcome</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>A human population who are exposed to an intervention.</t>
+          <t>An entity that is influenced by an intervention</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>human population</t>
+          <t>entity</t>
         </is>
       </c>
       <c r="E53" s="2" t="n"/>
       <c r="F53" s="2" t="n"/>
-      <c r="G53" s="2" t="n"/>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Includes individual human behaviour, mental activity and physiological activity. Also includes undesirable outcomes, such as treatment side effects, and unintended negative consequences of the intervention. </t>
+        </is>
+      </c>
       <c r="H53" s="2" t="n"/>
       <c r="I53" s="2" t="n"/>
       <c r="J53" s="2" t="n"/>
@@ -3714,7 +3710,7 @@
       <c r="O53" s="2" t="n"/>
       <c r="P53" s="2" t="inlineStr">
         <is>
-          <t>AW; PS</t>
+          <t>JH</t>
         </is>
       </c>
       <c r="Q53" s="2" t="n"/>
@@ -3735,41 +3731,29 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>BCIO:009000</t>
+          <t>BCIO:015095</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>intervention schedule of delivery</t>
+          <t>intervention population</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>An intervention attribute that is its temporal organisation.</t>
+          <t>A human population who are exposed to an intervention.</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>intervention attribute</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>BCI schedule of delivery</t>
-        </is>
-      </c>
+          <t>human population</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="n"/>
       <c r="F54" s="2" t="n"/>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>Includes the start and end of the BCI and its parts.</t>
-        </is>
-      </c>
+      <c r="G54" s="2" t="n"/>
       <c r="H54" s="2" t="n"/>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
-        </is>
-      </c>
+      <c r="I54" s="2" t="n"/>
       <c r="J54" s="2" t="n"/>
       <c r="K54" s="2" t="n"/>
       <c r="L54" s="2" t="inlineStr">
@@ -3782,7 +3766,7 @@
       <c r="O54" s="2" t="n"/>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>JH; RW</t>
+          <t>AW; PS</t>
         </is>
       </c>
       <c r="Q54" s="2" t="n"/>
@@ -3801,169 +3785,163 @@
       <c r="V54" s="2" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:009000</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>intervention schedule of delivery</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>An intervention attribute that is its temporal organisation.</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>intervention attribute</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>BCI schedule of delivery</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="n"/>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Includes the start and end of the BCI and its parts.</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="n"/>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>This class was previously specific to behaviour change interventions, but was expanded to be relevant to other types of interventions, allowing it to be applied more broadly. It can still be used for behaviour change interventions in the same way as before.</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="n"/>
+      <c r="K55" s="2" t="n"/>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="n"/>
+      <c r="N55" s="2" t="n"/>
+      <c r="O55" s="2" t="n"/>
+      <c r="P55" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW</t>
+        </is>
+      </c>
+      <c r="Q55" s="2" t="n"/>
+      <c r="R55" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="S55" s="2" t="n"/>
+      <c r="T55" s="2" t="n"/>
+      <c r="U55" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
         <is>
           <t>GMHO:0000254</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>intervention temporal context</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>intervention context</t>
         </is>
       </c>
-      <c r="R55" t="inlineStr">
+      <c r="R56" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="U55" t="n">
+      <c r="U56" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:050466</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="inlineStr">
-        <is>
-          <t>low cognitive exertion expended on a behaviour</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t>Cognitive exertion expended on a behaviour that is low.</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>cognitive exertion expended on a behaviour</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="n"/>
-      <c r="F56" s="3" t="n"/>
-      <c r="G56" s="3" t="n"/>
-      <c r="H56" s="3" t="n"/>
-      <c r="I56" s="3" t="inlineStr">
-        <is>
-          <t>Low cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
-        </is>
-      </c>
-      <c r="J56" s="3" t="n"/>
-      <c r="K56" s="3" t="n"/>
-      <c r="L56" s="3" t="inlineStr">
-        <is>
-          <t>behaviour</t>
-        </is>
-      </c>
-      <c r="M56" s="3" t="n"/>
-      <c r="N56" s="3" t="n"/>
-      <c r="O56" s="3" t="n"/>
-      <c r="P56" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="Q56" s="3" t="n"/>
-      <c r="R56" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="S56" s="3" t="n"/>
-      <c r="T56" s="3" t="n"/>
-      <c r="U56" s="3" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="V56" s="3" t="n"/>
-    </row>
     <row r="57">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:050467</t>
-        </is>
-      </c>
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>low emotional management exertion expended on a behaviour</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>Emotional management exertion expended on a behaviour that is low.</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>emotional management exertion expended on a behaviour</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="n"/>
-      <c r="F57" s="3" t="n"/>
-      <c r="G57" s="3" t="n"/>
-      <c r="H57" s="3" t="n"/>
-      <c r="I57" s="3" t="inlineStr">
-        <is>
-          <t>Low emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
-        </is>
-      </c>
-      <c r="J57" s="3" t="n"/>
-      <c r="K57" s="3" t="n"/>
-      <c r="L57" s="3" t="inlineStr">
-        <is>
-          <t>behaviour</t>
-        </is>
-      </c>
-      <c r="M57" s="3" t="n"/>
-      <c r="N57" s="3" t="n"/>
-      <c r="O57" s="3" t="n"/>
-      <c r="P57" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="Q57" s="3" t="n"/>
-      <c r="R57" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="S57" s="3" t="n"/>
-      <c r="T57" s="3" t="n"/>
-      <c r="U57" s="3" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="V57" s="3" t="n"/>
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:051026</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>intervention temporal context</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A temporal context of a process where the process is the intervention. </t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>temporal context of process</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr"/>
+      <c r="F57" s="4" t="inlineStr"/>
+      <c r="G57" s="4" t="inlineStr"/>
+      <c r="H57" s="4" t="inlineStr"/>
+      <c r="I57" s="4" t="inlineStr"/>
+      <c r="J57" s="4" t="inlineStr"/>
+      <c r="K57" s="4" t="inlineStr"/>
+      <c r="L57" s="4" t="inlineStr"/>
+      <c r="M57" s="4" t="inlineStr"/>
+      <c r="N57" s="4" t="inlineStr"/>
+      <c r="O57" s="4" t="inlineStr"/>
+      <c r="P57" s="4" t="inlineStr"/>
+      <c r="Q57" s="4" t="inlineStr"/>
+      <c r="R57" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="S57" s="4" t="inlineStr"/>
+      <c r="T57" s="4" t="inlineStr"/>
+      <c r="U57" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V57" s="4" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050468</t>
+          <t>BCIO:050466</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>low mental exertion expended on a behaviour</t>
+          <t>low cognitive exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Mental exertion expended on a behaviour that is low.</t>
+          <t>Cognitive exertion expended on a behaviour that is low.</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>mental exertion expended on a behaviour</t>
+          <t>cognitive exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E58" s="3" t="n"/>
@@ -3972,7 +3950,7 @@
       <c r="H58" s="3" t="n"/>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>Low mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
+          <t>Low cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J58" s="3" t="n"/>
@@ -4008,22 +3986,22 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050469</t>
+          <t>BCIO:050467</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>low physical exertion expended on behaviour</t>
+          <t>low emotional management exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Physical exertion expended on a behaviour that is low.</t>
+          <t>Emotional management exertion expended on a behaviour that is low.</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>physical exertion expended on a behaviour</t>
+          <t>emotional management exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E59" s="3" t="n"/>
@@ -4032,7 +4010,7 @@
       <c r="H59" s="3" t="n"/>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means </t>
+          <t>Low emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J59" s="3" t="n"/>
@@ -4068,22 +4046,22 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050470</t>
+          <t>BCIO:050468</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>moderate cognitive exertion expended on a behaviour</t>
+          <t>low mental exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Cognitive exertion expended on a behaviour that is medium.</t>
+          <t>Mental exertion expended on a behaviour that is low.</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>cognitive exertion expended on a behaviour</t>
+          <t>mental exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E60" s="3" t="n"/>
@@ -4092,7 +4070,7 @@
       <c r="H60" s="3" t="n"/>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>Moderate cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
+          <t>Low mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J60" s="3" t="n"/>
@@ -4128,22 +4106,22 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050471</t>
+          <t>BCIO:050469</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>moderate emotional management exertion expended on a behaviour</t>
+          <t>low physical exertion expended on behaviour</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Emotional management exertion expended on a behaviour that is medium.</t>
+          <t>Physical exertion expended on a behaviour that is low.</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>emotional management exertion expended on a behaviour</t>
+          <t>physical exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E61" s="3" t="n"/>
@@ -4152,7 +4130,7 @@
       <c r="H61" s="3" t="n"/>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>Moderate emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
+          <t xml:space="preserve">Low physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what low exertion means </t>
         </is>
       </c>
       <c r="J61" s="3" t="n"/>
@@ -4188,22 +4166,22 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050472</t>
+          <t>BCIO:050470</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>moderate mental exertion expended on a behaviour</t>
+          <t>moderate cognitive exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Mental exertion expended on a behaviour that is medium.</t>
+          <t>Cognitive exertion expended on a behaviour that is medium.</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>mental exertion expended on a behaviour</t>
+          <t>cognitive exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E62" s="3" t="n"/>
@@ -4212,7 +4190,7 @@
       <c r="H62" s="3" t="n"/>
       <c r="I62" s="3" t="inlineStr">
         <is>
-          <t>Moderate mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
+          <t>Moderate cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J62" s="3" t="n"/>
@@ -4248,22 +4226,22 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050473</t>
+          <t>BCIO:050471</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>moderate physical exertion expended on behaviour</t>
+          <t>moderate emotional management exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Physical exertion expended on a behaviour that is medium.</t>
+          <t>Emotional management exertion expended on a behaviour that is medium.</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>physical exertion expended on a behaviour</t>
+          <t>emotional management exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E63" s="3" t="n"/>
@@ -4272,7 +4250,7 @@
       <c r="H63" s="3" t="n"/>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>Moderate physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
+          <t>Moderate emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J63" s="3" t="n"/>
@@ -4306,160 +4284,162 @@
       <c r="V63" s="3" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:013000</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>participant engagement with behaviour change intervention</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>Participant engagement with intervention, where the intervention focuses on changing behaviour.</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>participant engagement with intervention</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>BCI engagement</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="n"/>
-      <c r="G64" s="2" t="inlineStr">
-        <is>
-          <t>Includes mental activities and behaviours.</t>
-        </is>
-      </c>
-      <c r="H64" s="2" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="I64" s="2" t="n"/>
-      <c r="J64" s="2" t="n"/>
-      <c r="K64" s="2" t="n"/>
-      <c r="L64" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
-      <c r="M64" s="2" t="n"/>
-      <c r="N64" s="2" t="n"/>
-      <c r="O64" s="2" t="n"/>
-      <c r="P64" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW; PS</t>
-        </is>
-      </c>
-      <c r="Q64" s="2" t="n"/>
-      <c r="R64" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S64" s="2" t="n"/>
-      <c r="T64" s="2" t="n"/>
-      <c r="U64" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V64" s="2" t="n"/>
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:050472</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>moderate mental exertion expended on a behaviour</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Mental exertion expended on a behaviour that is medium.</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>mental exertion expended on a behaviour</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="n"/>
+      <c r="F64" s="3" t="n"/>
+      <c r="G64" s="3" t="n"/>
+      <c r="H64" s="3" t="n"/>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>Moderate mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
+        </is>
+      </c>
+      <c r="J64" s="3" t="n"/>
+      <c r="K64" s="3" t="n"/>
+      <c r="L64" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="M64" s="3" t="n"/>
+      <c r="N64" s="3" t="n"/>
+      <c r="O64" s="3" t="n"/>
+      <c r="P64" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="Q64" s="3" t="n"/>
+      <c r="R64" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="S64" s="3" t="n"/>
+      <c r="T64" s="3" t="n"/>
+      <c r="U64" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="V64" s="3" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:050916</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>participant engagement with intervention</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>An individual human activity of an intervention participant within one or more parts of the intervention.</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>individual human activity</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="n"/>
-      <c r="F65" s="2" t="n"/>
-      <c r="G65" s="2" t="n"/>
-      <c r="H65" s="2" t="n"/>
-      <c r="I65" s="2" t="n"/>
-      <c r="J65" s="2" t="n"/>
-      <c r="K65" s="2" t="n"/>
-      <c r="L65" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
-      <c r="M65" s="2" t="n"/>
-      <c r="N65" s="2" t="n"/>
-      <c r="O65" s="2" t="n"/>
-      <c r="P65" s="2" t="inlineStr">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:050473</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>moderate physical exertion expended on behaviour</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Physical exertion expended on a behaviour that is medium.</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>physical exertion expended on a behaviour</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="n"/>
+      <c r="F65" s="3" t="n"/>
+      <c r="G65" s="3" t="n"/>
+      <c r="H65" s="3" t="n"/>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>Moderate physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="n"/>
+      <c r="K65" s="3" t="n"/>
+      <c r="L65" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="M65" s="3" t="n"/>
+      <c r="N65" s="3" t="n"/>
+      <c r="O65" s="3" t="n"/>
+      <c r="P65" s="3" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="Q65" s="2" t="inlineStr">
-        <is>
-          <t>The extend to someone interacts with an intervention, including their cognitive, emotional and behavioural response (e.g., attending intervention session) to the intervention itself.</t>
-        </is>
-      </c>
-      <c r="R65" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S65" s="2" t="n"/>
-      <c r="T65" s="2" t="n"/>
-      <c r="U65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="V65" s="2" t="n"/>
+      <c r="Q65" s="3" t="n"/>
+      <c r="R65" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="S65" s="3" t="n"/>
+      <c r="T65" s="3" t="n"/>
+      <c r="U65" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="V65" s="3" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>BCIO:034000</t>
+          <t>BCIO:013000</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>population behaviour</t>
+          <t>participant engagement with behaviour change intervention</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>An aggregate of individual human behaviours of members of a population.</t>
+          <t>Participant engagement with intervention, where the intervention focuses on changing behaviour.</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
+          <t>participant engagement with intervention</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>BCI engagement</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="n"/>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Includes mental activities and behaviours.</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
           <t>process</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>human behaviour</t>
-        </is>
-      </c>
-      <c r="F66" s="2" t="n"/>
-      <c r="G66" s="2" t="n"/>
-      <c r="H66" s="2" t="n"/>
       <c r="I66" s="2" t="n"/>
       <c r="J66" s="2" t="n"/>
       <c r="K66" s="2" t="n"/>
@@ -4473,7 +4453,7 @@
       <c r="O66" s="2" t="n"/>
       <c r="P66" s="2" t="inlineStr">
         <is>
-          <t>JH</t>
+          <t>JH; RW; PS</t>
         </is>
       </c>
       <c r="Q66" s="2" t="n"/>
@@ -4494,31 +4474,27 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>BCIO:043000</t>
+          <t>BCIO:050916</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>process attribute</t>
+          <t>participant engagement with intervention</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>A process profile that is an attribute of a process.</t>
+          <t>An individual human activity of an intervention participant within one or more parts of the intervention.</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>process profile</t>
+          <t>individual human activity</t>
         </is>
       </c>
       <c r="E67" s="2" t="n"/>
       <c r="F67" s="2" t="n"/>
-      <c r="G67" s="2" t="inlineStr">
-        <is>
-          <t>This is intended to provide a user-friendly way of representing the way in which processes are manifest. This is somewhat similar to, but not the same as, the class 'specifically dependent continuant' in Basic Formal Ontology which provides a way of representing features of material entities such as age and size. It is formally equivalent to process profile in Basic Formal Ontology.</t>
-        </is>
-      </c>
+      <c r="G67" s="2" t="n"/>
       <c r="H67" s="2" t="n"/>
       <c r="I67" s="2" t="n"/>
       <c r="J67" s="2" t="n"/>
@@ -4533,12 +4509,12 @@
       <c r="O67" s="2" t="n"/>
       <c r="P67" s="2" t="inlineStr">
         <is>
-          <t>JH</t>
+          <t>PS</t>
         </is>
       </c>
       <c r="Q67" s="2" t="inlineStr">
         <is>
-          <t>An attribute of a process.</t>
+          <t>The extend to someone interacts with an intervention, including their cognitive, emotional and behavioural response (e.g., attending intervention session) to the intervention itself.</t>
         </is>
       </c>
       <c r="R67" s="2" t="inlineStr">
@@ -4548,62 +4524,99 @@
       </c>
       <c r="S67" s="2" t="n"/>
       <c r="T67" s="2" t="n"/>
-      <c r="U67" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="U67" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="V67" s="2" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>GMHO:0000268</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>process context</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>entity</t>
-        </is>
-      </c>
-      <c r="R68" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="U68" t="n">
-        <v>0</v>
-      </c>
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:034000</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>population behaviour</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>An aggregate of individual human behaviours of members of a population.</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>human behaviour</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="n"/>
+      <c r="G68" s="2" t="n"/>
+      <c r="H68" s="2" t="n"/>
+      <c r="I68" s="2" t="n"/>
+      <c r="J68" s="2" t="n"/>
+      <c r="K68" s="2" t="n"/>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="n"/>
+      <c r="N68" s="2" t="n"/>
+      <c r="O68" s="2" t="n"/>
+      <c r="P68" s="2" t="inlineStr">
+        <is>
+          <t>JH</t>
+        </is>
+      </c>
+      <c r="Q68" s="2" t="n"/>
+      <c r="R68" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="S68" s="2" t="n"/>
+      <c r="T68" s="2" t="n"/>
+      <c r="U68" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V68" s="2" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050551</t>
+          <t>BCIO:043000</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>research study participants</t>
+          <t>process attribute</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>A population that is studied in a research study.</t>
+          <t>A process profile that is an attribute of a process.</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>human population</t>
+          <t>process profile</t>
         </is>
       </c>
       <c r="E69" s="2" t="n"/>
       <c r="F69" s="2" t="n"/>
-      <c r="G69" s="2" t="n"/>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>This is intended to provide a user-friendly way of representing the way in which processes are manifest. This is somewhat similar to, but not the same as, the class 'specifically dependent continuant' in Basic Formal Ontology which provides a way of representing features of material entities such as age and size. It is formally equivalent to process profile in Basic Formal Ontology.</t>
+        </is>
+      </c>
       <c r="H69" s="2" t="n"/>
       <c r="I69" s="2" t="n"/>
       <c r="J69" s="2" t="n"/>
@@ -4618,10 +4631,14 @@
       <c r="O69" s="2" t="n"/>
       <c r="P69" s="2" t="inlineStr">
         <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="Q69" s="2" t="n"/>
+          <t>JH</t>
+        </is>
+      </c>
+      <c r="Q69" s="2" t="inlineStr">
+        <is>
+          <t>An attribute of a process.</t>
+        </is>
+      </c>
       <c r="R69" s="2" t="inlineStr">
         <is>
           <t>Published</t>
@@ -4635,6 +4652,187 @@
         </is>
       </c>
       <c r="V69" s="2" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>GMHO:0000268</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>process context</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>entity</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="U70" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:051027</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>process context</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>An entity that includes the material and temporal contexts that are not part of but may influence the outcome of a process.</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>entity</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr"/>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>'temporal context of process' OR 'material context of process'</t>
+        </is>
+      </c>
+      <c r="G71" s="4" t="inlineStr"/>
+      <c r="H71" s="4" t="inlineStr"/>
+      <c r="I71" s="4" t="inlineStr"/>
+      <c r="J71" s="4" t="inlineStr"/>
+      <c r="K71" s="4" t="inlineStr"/>
+      <c r="L71" s="4" t="inlineStr"/>
+      <c r="M71" s="4" t="inlineStr"/>
+      <c r="N71" s="4" t="inlineStr"/>
+      <c r="O71" s="4" t="inlineStr"/>
+      <c r="P71" s="4" t="inlineStr"/>
+      <c r="Q71" s="4" t="inlineStr"/>
+      <c r="R71" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="S71" s="4" t="inlineStr"/>
+      <c r="T71" s="4" t="inlineStr"/>
+      <c r="U71" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V71" s="4" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:050551</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>research study participants</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>A population that is studied in a research study.</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>human population</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="n"/>
+      <c r="F72" s="2" t="n"/>
+      <c r="G72" s="2" t="n"/>
+      <c r="H72" s="2" t="n"/>
+      <c r="I72" s="2" t="n"/>
+      <c r="J72" s="2" t="n"/>
+      <c r="K72" s="2" t="n"/>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M72" s="2" t="n"/>
+      <c r="N72" s="2" t="n"/>
+      <c r="O72" s="2" t="n"/>
+      <c r="P72" s="2" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="Q72" s="2" t="n"/>
+      <c r="R72" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="S72" s="2" t="n"/>
+      <c r="T72" s="2" t="n"/>
+      <c r="U72" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V72" s="2" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:051028</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>temporal context of process</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>An occurrent that is not dependent on a process but may influence the effect of the process on its outcome.</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>occurrent</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr"/>
+      <c r="F73" s="4" t="inlineStr"/>
+      <c r="G73" s="4" t="inlineStr"/>
+      <c r="H73" s="4" t="inlineStr"/>
+      <c r="I73" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This entity includes time periods, events, etc. </t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="inlineStr"/>
+      <c r="K73" s="4" t="inlineStr"/>
+      <c r="L73" s="4" t="inlineStr"/>
+      <c r="M73" s="4" t="inlineStr"/>
+      <c r="N73" s="4" t="inlineStr"/>
+      <c r="O73" s="4" t="inlineStr"/>
+      <c r="P73" s="4" t="inlineStr"/>
+      <c r="Q73" s="4" t="inlineStr"/>
+      <c r="R73" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="S73" s="4" t="inlineStr"/>
+      <c r="T73" s="4" t="inlineStr"/>
+      <c r="U73" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V73" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 3 terms in BCIO_Upper_Defs.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
@@ -3366,29 +3366,46 @@
       <c r="V46" s="2" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000253</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>intervention context</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="C47" s="3" t="n"/>
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>process context</t>
         </is>
       </c>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="U47" t="n">
+      <c r="E47" s="3" t="n"/>
+      <c r="F47" s="3" t="n"/>
+      <c r="G47" s="3" t="n"/>
+      <c r="H47" s="3" t="n"/>
+      <c r="I47" s="3" t="n"/>
+      <c r="J47" s="3" t="n"/>
+      <c r="K47" s="3" t="n"/>
+      <c r="L47" s="3" t="n"/>
+      <c r="M47" s="3" t="n"/>
+      <c r="N47" s="3" t="n"/>
+      <c r="O47" s="3" t="n"/>
+      <c r="P47" s="3" t="n"/>
+      <c r="Q47" s="3" t="n"/>
+      <c r="R47" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="S47" s="3" t="n"/>
+      <c r="T47" s="3" t="n"/>
+      <c r="U47" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="V47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -3411,30 +3428,30 @@
           <t>process context</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr"/>
-      <c r="F48" s="4" t="inlineStr"/>
-      <c r="G48" s="4" t="inlineStr"/>
-      <c r="H48" s="4" t="inlineStr"/>
-      <c r="I48" s="4" t="inlineStr"/>
-      <c r="J48" s="4" t="inlineStr"/>
-      <c r="K48" s="4" t="inlineStr"/>
-      <c r="L48" s="4" t="inlineStr"/>
-      <c r="M48" s="4" t="inlineStr"/>
-      <c r="N48" s="4" t="inlineStr"/>
-      <c r="O48" s="4" t="inlineStr"/>
-      <c r="P48" s="4" t="inlineStr"/>
-      <c r="Q48" s="4" t="inlineStr"/>
+      <c r="E48" s="4" t="n"/>
+      <c r="F48" s="4" t="n"/>
+      <c r="G48" s="4" t="n"/>
+      <c r="H48" s="4" t="n"/>
+      <c r="I48" s="4" t="n"/>
+      <c r="J48" s="4" t="n"/>
+      <c r="K48" s="4" t="n"/>
+      <c r="L48" s="4" t="n"/>
+      <c r="M48" s="4" t="n"/>
+      <c r="N48" s="4" t="n"/>
+      <c r="O48" s="4" t="n"/>
+      <c r="P48" s="4" t="n"/>
+      <c r="Q48" s="4" t="n"/>
       <c r="R48" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="S48" s="4" t="inlineStr"/>
-      <c r="T48" s="4" t="inlineStr"/>
+      <c r="S48" s="4" t="n"/>
+      <c r="T48" s="4" t="n"/>
       <c r="U48" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="V48" s="4" t="inlineStr"/>
+      <c r="V48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3853,29 +3870,46 @@
       <c r="V55" s="2" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000254</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>intervention temporal context</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="C56" s="3" t="n"/>
+      <c r="D56" s="3" t="inlineStr">
         <is>
           <t>intervention context</t>
         </is>
       </c>
-      <c r="R56" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="U56" t="n">
+      <c r="E56" s="3" t="n"/>
+      <c r="F56" s="3" t="n"/>
+      <c r="G56" s="3" t="n"/>
+      <c r="H56" s="3" t="n"/>
+      <c r="I56" s="3" t="n"/>
+      <c r="J56" s="3" t="n"/>
+      <c r="K56" s="3" t="n"/>
+      <c r="L56" s="3" t="n"/>
+      <c r="M56" s="3" t="n"/>
+      <c r="N56" s="3" t="n"/>
+      <c r="O56" s="3" t="n"/>
+      <c r="P56" s="3" t="n"/>
+      <c r="Q56" s="3" t="n"/>
+      <c r="R56" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="S56" s="3" t="n"/>
+      <c r="T56" s="3" t="n"/>
+      <c r="U56" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="V56" s="3" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -3898,30 +3932,30 @@
           <t>temporal context of process</t>
         </is>
       </c>
-      <c r="E57" s="4" t="inlineStr"/>
-      <c r="F57" s="4" t="inlineStr"/>
-      <c r="G57" s="4" t="inlineStr"/>
-      <c r="H57" s="4" t="inlineStr"/>
-      <c r="I57" s="4" t="inlineStr"/>
-      <c r="J57" s="4" t="inlineStr"/>
-      <c r="K57" s="4" t="inlineStr"/>
-      <c r="L57" s="4" t="inlineStr"/>
-      <c r="M57" s="4" t="inlineStr"/>
-      <c r="N57" s="4" t="inlineStr"/>
-      <c r="O57" s="4" t="inlineStr"/>
-      <c r="P57" s="4" t="inlineStr"/>
-      <c r="Q57" s="4" t="inlineStr"/>
+      <c r="E57" s="4" t="n"/>
+      <c r="F57" s="4" t="n"/>
+      <c r="G57" s="4" t="n"/>
+      <c r="H57" s="4" t="n"/>
+      <c r="I57" s="4" t="n"/>
+      <c r="J57" s="4" t="n"/>
+      <c r="K57" s="4" t="n"/>
+      <c r="L57" s="4" t="n"/>
+      <c r="M57" s="4" t="n"/>
+      <c r="N57" s="4" t="n"/>
+      <c r="O57" s="4" t="n"/>
+      <c r="P57" s="4" t="n"/>
+      <c r="Q57" s="4" t="n"/>
       <c r="R57" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="S57" s="4" t="inlineStr"/>
-      <c r="T57" s="4" t="inlineStr"/>
+      <c r="S57" s="4" t="n"/>
+      <c r="T57" s="4" t="n"/>
       <c r="U57" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="V57" s="4" t="inlineStr"/>
+      <c r="V57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -4654,29 +4688,46 @@
       <c r="V69" s="2" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
+      <c r="A70" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000268</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
+      <c r="B70" s="3" t="inlineStr">
         <is>
           <t>process context</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="C70" s="3" t="n"/>
+      <c r="D70" s="3" t="inlineStr">
         <is>
           <t>entity</t>
         </is>
       </c>
-      <c r="R70" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="U70" t="n">
+      <c r="E70" s="3" t="n"/>
+      <c r="F70" s="3" t="n"/>
+      <c r="G70" s="3" t="n"/>
+      <c r="H70" s="3" t="n"/>
+      <c r="I70" s="3" t="n"/>
+      <c r="J70" s="3" t="n"/>
+      <c r="K70" s="3" t="n"/>
+      <c r="L70" s="3" t="n"/>
+      <c r="M70" s="3" t="n"/>
+      <c r="N70" s="3" t="n"/>
+      <c r="O70" s="3" t="n"/>
+      <c r="P70" s="3" t="n"/>
+      <c r="Q70" s="3" t="n"/>
+      <c r="R70" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="S70" s="3" t="n"/>
+      <c r="T70" s="3" t="n"/>
+      <c r="U70" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="V70" s="3" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -4699,34 +4750,34 @@
           <t>entity</t>
         </is>
       </c>
-      <c r="E71" s="4" t="inlineStr"/>
+      <c r="E71" s="4" t="n"/>
       <c r="F71" s="4" t="inlineStr">
         <is>
           <t>'temporal context of process' OR 'material context of process'</t>
         </is>
       </c>
-      <c r="G71" s="4" t="inlineStr"/>
-      <c r="H71" s="4" t="inlineStr"/>
-      <c r="I71" s="4" t="inlineStr"/>
-      <c r="J71" s="4" t="inlineStr"/>
-      <c r="K71" s="4" t="inlineStr"/>
-      <c r="L71" s="4" t="inlineStr"/>
-      <c r="M71" s="4" t="inlineStr"/>
-      <c r="N71" s="4" t="inlineStr"/>
-      <c r="O71" s="4" t="inlineStr"/>
-      <c r="P71" s="4" t="inlineStr"/>
-      <c r="Q71" s="4" t="inlineStr"/>
+      <c r="G71" s="4" t="n"/>
+      <c r="H71" s="4" t="n"/>
+      <c r="I71" s="4" t="n"/>
+      <c r="J71" s="4" t="n"/>
+      <c r="K71" s="4" t="n"/>
+      <c r="L71" s="4" t="n"/>
+      <c r="M71" s="4" t="n"/>
+      <c r="N71" s="4" t="n"/>
+      <c r="O71" s="4" t="n"/>
+      <c r="P71" s="4" t="n"/>
+      <c r="Q71" s="4" t="n"/>
       <c r="R71" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="S71" s="4" t="inlineStr"/>
-      <c r="T71" s="4" t="inlineStr"/>
+      <c r="S71" s="4" t="n"/>
+      <c r="T71" s="4" t="n"/>
       <c r="U71" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="V71" s="4" t="inlineStr"/>
+      <c r="V71" s="4" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4805,34 +4856,34 @@
           <t>occurrent</t>
         </is>
       </c>
-      <c r="E73" s="4" t="inlineStr"/>
-      <c r="F73" s="4" t="inlineStr"/>
-      <c r="G73" s="4" t="inlineStr"/>
-      <c r="H73" s="4" t="inlineStr"/>
+      <c r="E73" s="4" t="n"/>
+      <c r="F73" s="4" t="n"/>
+      <c r="G73" s="4" t="n"/>
+      <c r="H73" s="4" t="n"/>
       <c r="I73" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">This entity includes time periods, events, etc. </t>
         </is>
       </c>
-      <c r="J73" s="4" t="inlineStr"/>
-      <c r="K73" s="4" t="inlineStr"/>
-      <c r="L73" s="4" t="inlineStr"/>
-      <c r="M73" s="4" t="inlineStr"/>
-      <c r="N73" s="4" t="inlineStr"/>
-      <c r="O73" s="4" t="inlineStr"/>
-      <c r="P73" s="4" t="inlineStr"/>
-      <c r="Q73" s="4" t="inlineStr"/>
+      <c r="J73" s="4" t="n"/>
+      <c r="K73" s="4" t="n"/>
+      <c r="L73" s="4" t="n"/>
+      <c r="M73" s="4" t="n"/>
+      <c r="N73" s="4" t="n"/>
+      <c r="O73" s="4" t="n"/>
+      <c r="P73" s="4" t="n"/>
+      <c r="Q73" s="4" t="n"/>
       <c r="R73" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="S73" s="4" t="inlineStr"/>
-      <c r="T73" s="4" t="inlineStr"/>
+      <c r="S73" s="4" t="n"/>
+      <c r="T73" s="4" t="n"/>
       <c r="U73" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="V73" s="4" t="inlineStr"/>
+      <c r="V73" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 4 terms in BCIO_Upper_Defs.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
@@ -30,7 +30,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,11 +47,6 @@
         <fgColor rgb="002f4f4f"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00ffffff"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -65,12 +60,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3408,50 +3402,50 @@
       <c r="V47" s="3" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="inlineStr">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>BCIO:051025</t>
         </is>
       </c>
-      <c r="B48" s="4" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>intervention context</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>A process context in which the process is an intervention.</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>process context</t>
         </is>
       </c>
-      <c r="E48" s="4" t="n"/>
-      <c r="F48" s="4" t="n"/>
-      <c r="G48" s="4" t="n"/>
-      <c r="H48" s="4" t="n"/>
-      <c r="I48" s="4" t="n"/>
-      <c r="J48" s="4" t="n"/>
-      <c r="K48" s="4" t="n"/>
-      <c r="L48" s="4" t="n"/>
-      <c r="M48" s="4" t="n"/>
-      <c r="N48" s="4" t="n"/>
-      <c r="O48" s="4" t="n"/>
-      <c r="P48" s="4" t="n"/>
-      <c r="Q48" s="4" t="n"/>
-      <c r="R48" s="4" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="S48" s="4" t="n"/>
-      <c r="T48" s="4" t="n"/>
-      <c r="U48" s="4" t="n">
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
+      <c r="G48" s="2" t="n"/>
+      <c r="H48" s="2" t="n"/>
+      <c r="I48" s="2" t="n"/>
+      <c r="J48" s="2" t="n"/>
+      <c r="K48" s="2" t="n"/>
+      <c r="L48" s="2" t="n"/>
+      <c r="M48" s="2" t="n"/>
+      <c r="N48" s="2" t="n"/>
+      <c r="O48" s="2" t="n"/>
+      <c r="P48" s="2" t="n"/>
+      <c r="Q48" s="2" t="n"/>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="S48" s="2" t="n"/>
+      <c r="T48" s="2" t="n"/>
+      <c r="U48" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="V48" s="4" t="n"/>
+      <c r="V48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3912,50 +3906,50 @@
       <c r="V56" s="3" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="4" t="inlineStr">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>BCIO:051026</t>
         </is>
       </c>
-      <c r="B57" s="4" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>intervention temporal context</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">A temporal context of a process where the process is the intervention. </t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>temporal context of process</t>
         </is>
       </c>
-      <c r="E57" s="4" t="n"/>
-      <c r="F57" s="4" t="n"/>
-      <c r="G57" s="4" t="n"/>
-      <c r="H57" s="4" t="n"/>
-      <c r="I57" s="4" t="n"/>
-      <c r="J57" s="4" t="n"/>
-      <c r="K57" s="4" t="n"/>
-      <c r="L57" s="4" t="n"/>
-      <c r="M57" s="4" t="n"/>
-      <c r="N57" s="4" t="n"/>
-      <c r="O57" s="4" t="n"/>
-      <c r="P57" s="4" t="n"/>
-      <c r="Q57" s="4" t="n"/>
-      <c r="R57" s="4" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="S57" s="4" t="n"/>
-      <c r="T57" s="4" t="n"/>
-      <c r="U57" s="4" t="n">
+      <c r="E57" s="2" t="n"/>
+      <c r="F57" s="2" t="n"/>
+      <c r="G57" s="2" t="n"/>
+      <c r="H57" s="2" t="n"/>
+      <c r="I57" s="2" t="n"/>
+      <c r="J57" s="2" t="n"/>
+      <c r="K57" s="2" t="n"/>
+      <c r="L57" s="2" t="n"/>
+      <c r="M57" s="2" t="n"/>
+      <c r="N57" s="2" t="n"/>
+      <c r="O57" s="2" t="n"/>
+      <c r="P57" s="2" t="n"/>
+      <c r="Q57" s="2" t="n"/>
+      <c r="R57" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="S57" s="2" t="n"/>
+      <c r="T57" s="2" t="n"/>
+      <c r="U57" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="V57" s="4" t="n"/>
+      <c r="V57" s="2" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -4730,54 +4724,54 @@
       <c r="V70" s="3" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="4" t="inlineStr">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>BCIO:051027</t>
         </is>
       </c>
-      <c r="B71" s="4" t="inlineStr">
+      <c r="B71" s="2" t="inlineStr">
         <is>
           <t>process context</t>
         </is>
       </c>
-      <c r="C71" s="4" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
         <is>
           <t>An entity that includes the material and temporal contexts that are not part of but may influence the outcome of a process.</t>
         </is>
       </c>
-      <c r="D71" s="4" t="inlineStr">
+      <c r="D71" s="2" t="inlineStr">
         <is>
           <t>entity</t>
         </is>
       </c>
-      <c r="E71" s="4" t="n"/>
-      <c r="F71" s="4" t="inlineStr">
+      <c r="E71" s="2" t="n"/>
+      <c r="F71" s="2" t="inlineStr">
         <is>
           <t>'temporal context of process' OR 'material context of process'</t>
         </is>
       </c>
-      <c r="G71" s="4" t="n"/>
-      <c r="H71" s="4" t="n"/>
-      <c r="I71" s="4" t="n"/>
-      <c r="J71" s="4" t="n"/>
-      <c r="K71" s="4" t="n"/>
-      <c r="L71" s="4" t="n"/>
-      <c r="M71" s="4" t="n"/>
-      <c r="N71" s="4" t="n"/>
-      <c r="O71" s="4" t="n"/>
-      <c r="P71" s="4" t="n"/>
-      <c r="Q71" s="4" t="n"/>
-      <c r="R71" s="4" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="S71" s="4" t="n"/>
-      <c r="T71" s="4" t="n"/>
-      <c r="U71" s="4" t="n">
+      <c r="G71" s="2" t="n"/>
+      <c r="H71" s="2" t="n"/>
+      <c r="I71" s="2" t="n"/>
+      <c r="J71" s="2" t="n"/>
+      <c r="K71" s="2" t="n"/>
+      <c r="L71" s="2" t="n"/>
+      <c r="M71" s="2" t="n"/>
+      <c r="N71" s="2" t="n"/>
+      <c r="O71" s="2" t="n"/>
+      <c r="P71" s="2" t="n"/>
+      <c r="Q71" s="2" t="n"/>
+      <c r="R71" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="S71" s="2" t="n"/>
+      <c r="T71" s="2" t="n"/>
+      <c r="U71" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="V71" s="4" t="n"/>
+      <c r="V71" s="2" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4836,54 +4830,54 @@
       <c r="V72" s="2" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="4" t="inlineStr">
+      <c r="A73" s="2" t="inlineStr">
         <is>
           <t>BCIO:051028</t>
         </is>
       </c>
-      <c r="B73" s="4" t="inlineStr">
+      <c r="B73" s="2" t="inlineStr">
         <is>
           <t>temporal context of process</t>
         </is>
       </c>
-      <c r="C73" s="4" t="inlineStr">
+      <c r="C73" s="2" t="inlineStr">
         <is>
           <t>An occurrent that is not dependent on a process but may influence the effect of the process on its outcome.</t>
         </is>
       </c>
-      <c r="D73" s="4" t="inlineStr">
+      <c r="D73" s="2" t="inlineStr">
         <is>
           <t>occurrent</t>
         </is>
       </c>
-      <c r="E73" s="4" t="n"/>
-      <c r="F73" s="4" t="n"/>
-      <c r="G73" s="4" t="n"/>
-      <c r="H73" s="4" t="n"/>
-      <c r="I73" s="4" t="inlineStr">
+      <c r="E73" s="2" t="n"/>
+      <c r="F73" s="2" t="n"/>
+      <c r="G73" s="2" t="n"/>
+      <c r="H73" s="2" t="n"/>
+      <c r="I73" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">This entity includes time periods, events, etc. </t>
         </is>
       </c>
-      <c r="J73" s="4" t="n"/>
-      <c r="K73" s="4" t="n"/>
-      <c r="L73" s="4" t="n"/>
-      <c r="M73" s="4" t="n"/>
-      <c r="N73" s="4" t="n"/>
-      <c r="O73" s="4" t="n"/>
-      <c r="P73" s="4" t="n"/>
-      <c r="Q73" s="4" t="n"/>
-      <c r="R73" s="4" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="S73" s="4" t="n"/>
-      <c r="T73" s="4" t="n"/>
-      <c r="U73" s="4" t="n">
+      <c r="J73" s="2" t="n"/>
+      <c r="K73" s="2" t="n"/>
+      <c r="L73" s="2" t="n"/>
+      <c r="M73" s="2" t="n"/>
+      <c r="N73" s="2" t="n"/>
+      <c r="O73" s="2" t="n"/>
+      <c r="P73" s="2" t="n"/>
+      <c r="Q73" s="2" t="n"/>
+      <c r="R73" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="S73" s="2" t="n"/>
+      <c r="T73" s="2" t="n"/>
+      <c r="U73" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="V73" s="4" t="n"/>
+      <c r="V73" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 3 terms to BCIO_Upper_Defs.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
@@ -30,7 +30,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +47,11 @@
         <fgColor rgb="002f4f4f"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ffffff"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -60,11 +65,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V73"/>
+  <dimension ref="A1:V76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,27 +517,27 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>Curation status</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Informal definition</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>To be reviewed by</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Reviewer query</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>Curator</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Informal definition</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Curation status</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>To be reviewed by</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Reviewer query</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
@@ -591,21 +597,21 @@
       <c r="O2" s="2" t="n"/>
       <c r="P2" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>An attribute of a behaviour change intervention.</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
           <t>RW</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>An attribute of a behaviour change intervention.</t>
-        </is>
-      </c>
-      <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="n"/>
       <c r="U2" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -655,21 +661,21 @@
       <c r="O3" s="2" t="n"/>
       <c r="P3" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>A criterion for selecting people for a BCI population.</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="n"/>
+      <c r="S3" s="2" t="n"/>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
           <t>RW; JH</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="inlineStr">
-        <is>
-          <t>A criterion for selecting people for a BCI population.</t>
-        </is>
-      </c>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S3" s="2" t="n"/>
-      <c r="T3" s="2" t="n"/>
       <c r="U3" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -735,17 +741,17 @@
       <c r="O4" s="2" t="n"/>
       <c r="P4" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="n"/>
+      <c r="R4" s="2" t="n"/>
+      <c r="S4" s="2" t="n"/>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
           <t>JH; BG; PS</t>
         </is>
       </c>
-      <c r="Q4" s="2" t="n"/>
-      <c r="R4" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S4" s="2" t="n"/>
-      <c r="T4" s="2" t="n"/>
       <c r="U4" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -803,17 +809,17 @@
       <c r="O5" s="2" t="n"/>
       <c r="P5" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="n"/>
+      <c r="R5" s="2" t="n"/>
+      <c r="S5" s="2" t="n"/>
+      <c r="T5" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q5" s="2" t="n"/>
-      <c r="R5" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S5" s="2" t="n"/>
-      <c r="T5" s="2" t="n"/>
       <c r="U5" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -871,17 +877,17 @@
       <c r="O6" s="2" t="n"/>
       <c r="P6" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="n"/>
+      <c r="R6" s="2" t="n"/>
+      <c r="S6" s="2" t="n"/>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
           <t>RW</t>
         </is>
       </c>
-      <c r="Q6" s="2" t="n"/>
-      <c r="R6" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S6" s="2" t="n"/>
-      <c r="T6" s="2" t="n"/>
       <c r="U6" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -939,17 +945,17 @@
       <c r="O7" s="2" t="n"/>
       <c r="P7" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="n"/>
+      <c r="R7" s="2" t="n"/>
+      <c r="S7" s="2" t="n"/>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q7" s="2" t="n"/>
-      <c r="R7" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S7" s="2" t="n"/>
-      <c r="T7" s="2" t="n"/>
       <c r="U7" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1003,17 +1009,17 @@
       <c r="O8" s="2" t="n"/>
       <c r="P8" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="n"/>
+      <c r="R8" s="2" t="n"/>
+      <c r="S8" s="2" t="n"/>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q8" s="2" t="n"/>
-      <c r="R8" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S8" s="2" t="n"/>
-      <c r="T8" s="2" t="n"/>
       <c r="U8" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1075,17 +1081,17 @@
       <c r="O9" s="2" t="n"/>
       <c r="P9" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="n"/>
+      <c r="R9" s="2" t="n"/>
+      <c r="S9" s="2" t="n"/>
+      <c r="T9" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q9" s="2" t="n"/>
-      <c r="R9" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S9" s="2" t="n"/>
-      <c r="T9" s="2" t="n"/>
       <c r="U9" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1143,17 +1149,17 @@
       <c r="O10" s="2" t="n"/>
       <c r="P10" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="n"/>
+      <c r="R10" s="2" t="n"/>
+      <c r="S10" s="2" t="n"/>
+      <c r="T10" s="2" t="inlineStr">
+        <is>
           <t>JH; RW; BG</t>
         </is>
       </c>
-      <c r="Q10" s="2" t="n"/>
-      <c r="R10" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S10" s="2" t="n"/>
-      <c r="T10" s="2" t="n"/>
       <c r="U10" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1207,17 +1213,17 @@
       <c r="O11" s="2" t="n"/>
       <c r="P11" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="n"/>
+      <c r="R11" s="2" t="n"/>
+      <c r="S11" s="2" t="n"/>
+      <c r="T11" s="2" t="inlineStr">
+        <is>
           <t>JH; RW; BG</t>
         </is>
       </c>
-      <c r="Q11" s="2" t="n"/>
-      <c r="R11" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S11" s="2" t="n"/>
-      <c r="T11" s="2" t="n"/>
       <c r="U11" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1275,17 +1281,17 @@
       <c r="O12" s="2" t="n"/>
       <c r="P12" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="n"/>
+      <c r="R12" s="2" t="n"/>
+      <c r="S12" s="2" t="n"/>
+      <c r="T12" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q12" s="2" t="n"/>
-      <c r="R12" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S12" s="2" t="n"/>
-      <c r="T12" s="2" t="n"/>
       <c r="U12" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1339,17 +1345,17 @@
       <c r="O13" s="2" t="n"/>
       <c r="P13" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="n"/>
+      <c r="R13" s="2" t="n"/>
+      <c r="S13" s="2" t="n"/>
+      <c r="T13" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q13" s="2" t="n"/>
-      <c r="R13" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S13" s="2" t="n"/>
-      <c r="T13" s="2" t="n"/>
       <c r="U13" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1403,17 +1409,17 @@
       <c r="O14" s="2" t="n"/>
       <c r="P14" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="n"/>
+      <c r="R14" s="2" t="n"/>
+      <c r="S14" s="2" t="n"/>
+      <c r="T14" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q14" s="2" t="n"/>
-      <c r="R14" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S14" s="2" t="n"/>
-      <c r="T14" s="2" t="n"/>
       <c r="U14" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1467,17 +1473,17 @@
       <c r="O15" s="2" t="n"/>
       <c r="P15" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="n"/>
+      <c r="R15" s="2" t="n"/>
+      <c r="S15" s="2" t="n"/>
+      <c r="T15" s="2" t="inlineStr">
+        <is>
           <t>PS; JH; RW</t>
         </is>
       </c>
-      <c r="Q15" s="2" t="n"/>
-      <c r="R15" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S15" s="2" t="n"/>
-      <c r="T15" s="2" t="n"/>
       <c r="U15" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1531,17 +1537,17 @@
       <c r="O16" s="2" t="n"/>
       <c r="P16" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="n"/>
+      <c r="R16" s="2" t="n"/>
+      <c r="S16" s="2" t="n"/>
+      <c r="T16" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q16" s="2" t="n"/>
-      <c r="R16" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S16" s="2" t="n"/>
-      <c r="T16" s="2" t="n"/>
       <c r="U16" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1591,17 +1597,17 @@
       <c r="O17" s="2" t="n"/>
       <c r="P17" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="n"/>
+      <c r="R17" s="2" t="n"/>
+      <c r="S17" s="2" t="n"/>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
           <t>JH; BG; PS</t>
         </is>
       </c>
-      <c r="Q17" s="2" t="n"/>
-      <c r="R17" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S17" s="2" t="n"/>
-      <c r="T17" s="2" t="n"/>
       <c r="U17" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1659,17 +1665,17 @@
       <c r="O18" s="2" t="n"/>
       <c r="P18" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="n"/>
+      <c r="R18" s="2" t="n"/>
+      <c r="S18" s="2" t="n"/>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q18" s="2" t="n"/>
-      <c r="R18" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S18" s="2" t="n"/>
-      <c r="T18" s="2" t="n"/>
       <c r="U18" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1719,17 +1725,17 @@
       <c r="O19" s="2" t="n"/>
       <c r="P19" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q19" s="2" t="n"/>
+      <c r="R19" s="2" t="n"/>
+      <c r="S19" s="2" t="n"/>
+      <c r="T19" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q19" s="2" t="n"/>
-      <c r="R19" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S19" s="2" t="n"/>
-      <c r="T19" s="2" t="n"/>
       <c r="U19" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1779,17 +1785,17 @@
       <c r="O20" s="2" t="n"/>
       <c r="P20" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="n"/>
+      <c r="R20" s="2" t="n"/>
+      <c r="S20" s="2" t="n"/>
+      <c r="T20" s="2" t="inlineStr">
+        <is>
           <t>JH; RW; PS</t>
         </is>
       </c>
-      <c r="Q20" s="2" t="n"/>
-      <c r="R20" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S20" s="2" t="n"/>
-      <c r="T20" s="2" t="n"/>
       <c r="U20" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1843,17 +1849,17 @@
       <c r="O21" s="2" t="n"/>
       <c r="P21" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="n"/>
+      <c r="R21" s="2" t="n"/>
+      <c r="S21" s="2" t="n"/>
+      <c r="T21" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q21" s="2" t="n"/>
-      <c r="R21" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S21" s="2" t="n"/>
-      <c r="T21" s="2" t="n"/>
       <c r="U21" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1903,17 +1909,17 @@
       <c r="O22" s="2" t="n"/>
       <c r="P22" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="n"/>
+      <c r="R22" s="2" t="n"/>
+      <c r="S22" s="2" t="n"/>
+      <c r="T22" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q22" s="2" t="n"/>
-      <c r="R22" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S22" s="2" t="n"/>
-      <c r="T22" s="2" t="n"/>
       <c r="U22" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1963,17 +1969,17 @@
       <c r="O23" s="2" t="n"/>
       <c r="P23" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q23" s="2" t="n"/>
+      <c r="R23" s="2" t="n"/>
+      <c r="S23" s="2" t="n"/>
+      <c r="T23" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q23" s="2" t="n"/>
-      <c r="R23" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S23" s="2" t="n"/>
-      <c r="T23" s="2" t="n"/>
       <c r="U23" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2027,17 +2033,17 @@
       <c r="O24" s="2" t="n"/>
       <c r="P24" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q24" s="2" t="n"/>
+      <c r="R24" s="2" t="n"/>
+      <c r="S24" s="2" t="n"/>
+      <c r="T24" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q24" s="2" t="n"/>
-      <c r="R24" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S24" s="2" t="n"/>
-      <c r="T24" s="2" t="n"/>
       <c r="U24" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2087,17 +2093,17 @@
       <c r="O25" s="2" t="n"/>
       <c r="P25" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q25" s="2" t="n"/>
+      <c r="R25" s="2" t="n"/>
+      <c r="S25" s="2" t="n"/>
+      <c r="T25" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q25" s="2" t="n"/>
-      <c r="R25" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S25" s="2" t="n"/>
-      <c r="T25" s="2" t="n"/>
       <c r="U25" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2151,17 +2157,17 @@
       <c r="O26" s="2" t="n"/>
       <c r="P26" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="n"/>
+      <c r="R26" s="2" t="n"/>
+      <c r="S26" s="2" t="n"/>
+      <c r="T26" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q26" s="2" t="n"/>
-      <c r="R26" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S26" s="2" t="n"/>
-      <c r="T26" s="2" t="n"/>
       <c r="U26" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2215,17 +2221,17 @@
       <c r="O27" s="2" t="n"/>
       <c r="P27" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q27" s="2" t="n"/>
+      <c r="R27" s="2" t="n"/>
+      <c r="S27" s="2" t="n"/>
+      <c r="T27" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q27" s="2" t="n"/>
-      <c r="R27" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S27" s="2" t="n"/>
-      <c r="T27" s="2" t="n"/>
       <c r="U27" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2275,17 +2281,17 @@
       <c r="O28" s="2" t="n"/>
       <c r="P28" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q28" s="2" t="n"/>
+      <c r="R28" s="2" t="n"/>
+      <c r="S28" s="2" t="n"/>
+      <c r="T28" s="2" t="inlineStr">
+        <is>
           <t>JH; RW; PS</t>
         </is>
       </c>
-      <c r="Q28" s="2" t="n"/>
-      <c r="R28" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S28" s="2" t="n"/>
-      <c r="T28" s="2" t="n"/>
       <c r="U28" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2339,17 +2345,17 @@
       <c r="O29" s="2" t="n"/>
       <c r="P29" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q29" s="2" t="n"/>
+      <c r="R29" s="2" t="n"/>
+      <c r="S29" s="2" t="n"/>
+      <c r="T29" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q29" s="2" t="n"/>
-      <c r="R29" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S29" s="2" t="n"/>
-      <c r="T29" s="2" t="n"/>
       <c r="U29" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2407,21 +2413,21 @@
       <c r="O30" s="2" t="n"/>
       <c r="P30" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q30" s="2" t="inlineStr">
+        <is>
+          <t>An attribute of a behaviour change intervention (BCI) or a BCI component whereby its content or delivery is varied according to characteristics of members of the target population or setting.</t>
+        </is>
+      </c>
+      <c r="R30" s="2" t="n"/>
+      <c r="S30" s="2" t="n"/>
+      <c r="T30" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q30" s="2" t="inlineStr">
-        <is>
-          <t>An attribute of a behaviour change intervention (BCI) or a BCI component whereby its content or delivery is varied according to characteristics of members of the target population or setting.</t>
-        </is>
-      </c>
-      <c r="R30" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S30" s="2" t="n"/>
-      <c r="T30" s="2" t="n"/>
       <c r="U30" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2471,17 +2477,17 @@
       <c r="O31" s="2" t="n"/>
       <c r="P31" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q31" s="2" t="n"/>
+      <c r="R31" s="2" t="n"/>
+      <c r="S31" s="2" t="n"/>
+      <c r="T31" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q31" s="2" t="n"/>
-      <c r="R31" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S31" s="2" t="n"/>
-      <c r="T31" s="2" t="n"/>
       <c r="U31" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2531,17 +2537,17 @@
       <c r="O32" s="2" t="n"/>
       <c r="P32" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q32" s="2" t="n"/>
+      <c r="R32" s="2" t="n"/>
+      <c r="S32" s="2" t="n"/>
+      <c r="T32" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q32" s="2" t="n"/>
-      <c r="R32" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S32" s="2" t="n"/>
-      <c r="T32" s="2" t="n"/>
       <c r="U32" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2591,17 +2597,17 @@
       <c r="O33" s="2" t="n"/>
       <c r="P33" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q33" s="2" t="n"/>
+      <c r="R33" s="2" t="n"/>
+      <c r="S33" s="2" t="n"/>
+      <c r="T33" s="2" t="inlineStr">
+        <is>
           <t>JH; RW; PS</t>
         </is>
       </c>
-      <c r="Q33" s="2" t="n"/>
-      <c r="R33" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S33" s="2" t="n"/>
-      <c r="T33" s="2" t="n"/>
       <c r="U33" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2647,17 +2653,17 @@
       <c r="O34" s="2" t="n"/>
       <c r="P34" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q34" s="2" t="n"/>
+      <c r="R34" s="2" t="n"/>
+      <c r="S34" s="2" t="n"/>
+      <c r="T34" s="2" t="inlineStr">
+        <is>
           <t>JH; PS</t>
         </is>
       </c>
-      <c r="Q34" s="2" t="n"/>
-      <c r="R34" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S34" s="2" t="n"/>
-      <c r="T34" s="2" t="n"/>
       <c r="U34" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2703,17 +2709,17 @@
       <c r="O35" s="2" t="n"/>
       <c r="P35" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q35" s="2" t="n"/>
+      <c r="R35" s="2" t="n"/>
+      <c r="S35" s="2" t="n"/>
+      <c r="T35" s="2" t="inlineStr">
+        <is>
           <t>JH</t>
         </is>
       </c>
-      <c r="Q35" s="2" t="n"/>
-      <c r="R35" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S35" s="2" t="n"/>
-      <c r="T35" s="2" t="n"/>
       <c r="U35" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -2763,17 +2769,17 @@
       <c r="O36" s="3" t="n"/>
       <c r="P36" s="3" t="inlineStr">
         <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Q36" s="3" t="n"/>
+      <c r="R36" s="3" t="n"/>
+      <c r="S36" s="3" t="n"/>
+      <c r="T36" s="3" t="inlineStr">
+        <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="Q36" s="3" t="n"/>
-      <c r="R36" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="S36" s="3" t="n"/>
-      <c r="T36" s="3" t="n"/>
       <c r="U36" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -2823,17 +2829,17 @@
       <c r="O37" s="3" t="n"/>
       <c r="P37" s="3" t="inlineStr">
         <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Q37" s="3" t="n"/>
+      <c r="R37" s="3" t="n"/>
+      <c r="S37" s="3" t="n"/>
+      <c r="T37" s="3" t="inlineStr">
+        <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="Q37" s="3" t="n"/>
-      <c r="R37" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="S37" s="3" t="n"/>
-      <c r="T37" s="3" t="n"/>
       <c r="U37" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -2883,17 +2889,17 @@
       <c r="O38" s="3" t="n"/>
       <c r="P38" s="3" t="inlineStr">
         <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Q38" s="3" t="n"/>
+      <c r="R38" s="3" t="n"/>
+      <c r="S38" s="3" t="n"/>
+      <c r="T38" s="3" t="inlineStr">
+        <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="Q38" s="3" t="n"/>
-      <c r="R38" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="S38" s="3" t="n"/>
-      <c r="T38" s="3" t="n"/>
       <c r="U38" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -2943,17 +2949,17 @@
       <c r="O39" s="3" t="n"/>
       <c r="P39" s="3" t="inlineStr">
         <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Q39" s="3" t="n"/>
+      <c r="R39" s="3" t="n"/>
+      <c r="S39" s="3" t="n"/>
+      <c r="T39" s="3" t="inlineStr">
+        <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="Q39" s="3" t="n"/>
-      <c r="R39" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="S39" s="3" t="n"/>
-      <c r="T39" s="3" t="n"/>
       <c r="U39" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -3003,17 +3009,17 @@
       <c r="O40" s="3" t="n"/>
       <c r="P40" s="3" t="inlineStr">
         <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Q40" s="3" t="n"/>
+      <c r="R40" s="3" t="n"/>
+      <c r="S40" s="3" t="n"/>
+      <c r="T40" s="3" t="inlineStr">
+        <is>
           <t>BG; PS</t>
         </is>
       </c>
-      <c r="Q40" s="3" t="n"/>
-      <c r="R40" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="S40" s="3" t="n"/>
-      <c r="T40" s="3" t="n"/>
       <c r="U40" s="3" t="inlineStr">
         <is>
           <t>0</t>
@@ -3059,17 +3065,17 @@
       <c r="O41" s="2" t="n"/>
       <c r="P41" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q41" s="2" t="n"/>
+      <c r="R41" s="2" t="n"/>
+      <c r="S41" s="2" t="n"/>
+      <c r="T41" s="2" t="inlineStr">
+        <is>
           <t>JH; AW</t>
         </is>
       </c>
-      <c r="Q41" s="2" t="n"/>
-      <c r="R41" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S41" s="2" t="n"/>
-      <c r="T41" s="2" t="n"/>
       <c r="U41" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3115,17 +3121,17 @@
       <c r="O42" s="2" t="n"/>
       <c r="P42" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q42" s="2" t="n"/>
+      <c r="R42" s="2" t="n"/>
+      <c r="S42" s="2" t="n"/>
+      <c r="T42" s="2" t="inlineStr">
+        <is>
           <t>JH</t>
         </is>
       </c>
-      <c r="Q42" s="2" t="n"/>
-      <c r="R42" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S42" s="2" t="n"/>
-      <c r="T42" s="2" t="n"/>
       <c r="U42" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3179,17 +3185,17 @@
       <c r="O43" s="2" t="n"/>
       <c r="P43" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q43" s="2" t="n"/>
+      <c r="R43" s="2" t="n"/>
+      <c r="S43" s="2" t="n"/>
+      <c r="T43" s="2" t="inlineStr">
+        <is>
           <t>JH</t>
         </is>
       </c>
-      <c r="Q43" s="2" t="n"/>
-      <c r="R43" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S43" s="2" t="n"/>
-      <c r="T43" s="2" t="n"/>
       <c r="U43" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3239,17 +3245,17 @@
       <c r="O44" s="2" t="n"/>
       <c r="P44" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q44" s="2" t="n"/>
+      <c r="R44" s="2" t="n"/>
+      <c r="S44" s="2" t="n"/>
+      <c r="T44" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q44" s="2" t="n"/>
-      <c r="R44" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S44" s="2" t="n"/>
-      <c r="T44" s="2" t="n"/>
       <c r="U44" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3289,13 +3295,13 @@
       <c r="M45" s="2" t="n"/>
       <c r="N45" s="2" t="n"/>
       <c r="O45" s="2" t="n"/>
-      <c r="P45" s="2" t="n"/>
+      <c r="P45" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="Q45" s="2" t="n"/>
-      <c r="R45" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="R45" s="2" t="n"/>
       <c r="S45" s="2" t="n"/>
       <c r="T45" s="2" t="n"/>
       <c r="U45" s="2" t="n">
@@ -3341,17 +3347,17 @@
       <c r="O46" s="2" t="n"/>
       <c r="P46" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q46" s="2" t="n"/>
+      <c r="R46" s="2" t="n"/>
+      <c r="S46" s="2" t="n"/>
+      <c r="T46" s="2" t="inlineStr">
+        <is>
           <t>RW</t>
         </is>
       </c>
-      <c r="Q46" s="2" t="n"/>
-      <c r="R46" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S46" s="2" t="n"/>
-      <c r="T46" s="2" t="n"/>
       <c r="U46" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3387,13 +3393,13 @@
       <c r="M47" s="3" t="n"/>
       <c r="N47" s="3" t="n"/>
       <c r="O47" s="3" t="n"/>
-      <c r="P47" s="3" t="n"/>
+      <c r="P47" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
       <c r="Q47" s="3" t="n"/>
-      <c r="R47" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="R47" s="3" t="n"/>
       <c r="S47" s="3" t="n"/>
       <c r="T47" s="3" t="n"/>
       <c r="U47" s="3" t="n">
@@ -3433,13 +3439,13 @@
       <c r="M48" s="2" t="n"/>
       <c r="N48" s="2" t="n"/>
       <c r="O48" s="2" t="n"/>
-      <c r="P48" s="2" t="n"/>
+      <c r="P48" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="Q48" s="2" t="n"/>
-      <c r="R48" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="R48" s="2" t="n"/>
       <c r="S48" s="2" t="n"/>
       <c r="T48" s="2" t="n"/>
       <c r="U48" s="2" t="n">
@@ -3485,17 +3491,17 @@
       <c r="O49" s="2" t="n"/>
       <c r="P49" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q49" s="2" t="n"/>
+      <c r="R49" s="2" t="n"/>
+      <c r="S49" s="2" t="n"/>
+      <c r="T49" s="2" t="inlineStr">
+        <is>
           <t>RW</t>
         </is>
       </c>
-      <c r="Q49" s="2" t="n"/>
-      <c r="R49" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S49" s="2" t="n"/>
-      <c r="T49" s="2" t="n"/>
       <c r="U49" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3541,17 +3547,17 @@
       <c r="O50" s="2" t="n"/>
       <c r="P50" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q50" s="2" t="n"/>
+      <c r="R50" s="2" t="n"/>
+      <c r="S50" s="2" t="n"/>
+      <c r="T50" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q50" s="2" t="n"/>
-      <c r="R50" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S50" s="2" t="n"/>
-      <c r="T50" s="2" t="n"/>
       <c r="U50" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3597,17 +3603,17 @@
       <c r="O51" s="2" t="n"/>
       <c r="P51" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q51" s="2" t="n"/>
+      <c r="R51" s="2" t="n"/>
+      <c r="S51" s="2" t="n"/>
+      <c r="T51" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q51" s="2" t="n"/>
-      <c r="R51" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S51" s="2" t="n"/>
-      <c r="T51" s="2" t="n"/>
       <c r="U51" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3661,17 +3667,17 @@
       <c r="O52" s="2" t="n"/>
       <c r="P52" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q52" s="2" t="n"/>
+      <c r="R52" s="2" t="n"/>
+      <c r="S52" s="2" t="n"/>
+      <c r="T52" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q52" s="2" t="n"/>
-      <c r="R52" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S52" s="2" t="n"/>
-      <c r="T52" s="2" t="n"/>
       <c r="U52" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3721,17 +3727,17 @@
       <c r="O53" s="2" t="n"/>
       <c r="P53" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q53" s="2" t="n"/>
+      <c r="R53" s="2" t="n"/>
+      <c r="S53" s="2" t="n"/>
+      <c r="T53" s="2" t="inlineStr">
+        <is>
           <t>JH</t>
         </is>
       </c>
-      <c r="Q53" s="2" t="n"/>
-      <c r="R53" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S53" s="2" t="n"/>
-      <c r="T53" s="2" t="n"/>
       <c r="U53" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3777,17 +3783,17 @@
       <c r="O54" s="2" t="n"/>
       <c r="P54" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q54" s="2" t="n"/>
+      <c r="R54" s="2" t="n"/>
+      <c r="S54" s="2" t="n"/>
+      <c r="T54" s="2" t="inlineStr">
+        <is>
           <t>AW; PS</t>
         </is>
       </c>
-      <c r="Q54" s="2" t="n"/>
-      <c r="R54" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S54" s="2" t="n"/>
-      <c r="T54" s="2" t="n"/>
       <c r="U54" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3845,17 +3851,17 @@
       <c r="O55" s="2" t="n"/>
       <c r="P55" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q55" s="2" t="n"/>
+      <c r="R55" s="2" t="n"/>
+      <c r="S55" s="2" t="n"/>
+      <c r="T55" s="2" t="inlineStr">
+        <is>
           <t>JH; RW</t>
         </is>
       </c>
-      <c r="Q55" s="2" t="n"/>
-      <c r="R55" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S55" s="2" t="n"/>
-      <c r="T55" s="2" t="n"/>
       <c r="U55" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -3891,13 +3897,13 @@
       <c r="M56" s="3" t="n"/>
       <c r="N56" s="3" t="n"/>
       <c r="O56" s="3" t="n"/>
-      <c r="P56" s="3" t="n"/>
+      <c r="P56" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
       <c r="Q56" s="3" t="n"/>
-      <c r="R56" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
+      <c r="R56" s="3" t="n"/>
       <c r="S56" s="3" t="n"/>
       <c r="T56" s="3" t="n"/>
       <c r="U56" s="3" t="n">
@@ -3937,13 +3943,13 @@
       <c r="M57" s="2" t="n"/>
       <c r="N57" s="2" t="n"/>
       <c r="O57" s="2" t="n"/>
-      <c r="P57" s="2" t="n"/>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="Q57" s="2" t="n"/>
-      <c r="R57" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="R57" s="2" t="n"/>
       <c r="S57" s="2" t="n"/>
       <c r="T57" s="2" t="n"/>
       <c r="U57" s="2" t="n">
@@ -3993,17 +3999,17 @@
       <c r="O58" s="3" t="n"/>
       <c r="P58" s="3" t="inlineStr">
         <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Q58" s="3" t="n"/>
+      <c r="R58" s="3" t="n"/>
+      <c r="S58" s="3" t="n"/>
+      <c r="T58" s="3" t="inlineStr">
+        <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="Q58" s="3" t="n"/>
-      <c r="R58" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="S58" s="3" t="n"/>
-      <c r="T58" s="3" t="n"/>
       <c r="U58" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -4053,17 +4059,17 @@
       <c r="O59" s="3" t="n"/>
       <c r="P59" s="3" t="inlineStr">
         <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Q59" s="3" t="n"/>
+      <c r="R59" s="3" t="n"/>
+      <c r="S59" s="3" t="n"/>
+      <c r="T59" s="3" t="inlineStr">
+        <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="Q59" s="3" t="n"/>
-      <c r="R59" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="S59" s="3" t="n"/>
-      <c r="T59" s="3" t="n"/>
       <c r="U59" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -4113,17 +4119,17 @@
       <c r="O60" s="3" t="n"/>
       <c r="P60" s="3" t="inlineStr">
         <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Q60" s="3" t="n"/>
+      <c r="R60" s="3" t="n"/>
+      <c r="S60" s="3" t="n"/>
+      <c r="T60" s="3" t="inlineStr">
+        <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="Q60" s="3" t="n"/>
-      <c r="R60" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="S60" s="3" t="n"/>
-      <c r="T60" s="3" t="n"/>
       <c r="U60" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -4173,17 +4179,17 @@
       <c r="O61" s="3" t="n"/>
       <c r="P61" s="3" t="inlineStr">
         <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Q61" s="3" t="n"/>
+      <c r="R61" s="3" t="n"/>
+      <c r="S61" s="3" t="n"/>
+      <c r="T61" s="3" t="inlineStr">
+        <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="Q61" s="3" t="n"/>
-      <c r="R61" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="S61" s="3" t="n"/>
-      <c r="T61" s="3" t="n"/>
       <c r="U61" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -4233,17 +4239,17 @@
       <c r="O62" s="3" t="n"/>
       <c r="P62" s="3" t="inlineStr">
         <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Q62" s="3" t="n"/>
+      <c r="R62" s="3" t="n"/>
+      <c r="S62" s="3" t="n"/>
+      <c r="T62" s="3" t="inlineStr">
+        <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="Q62" s="3" t="n"/>
-      <c r="R62" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="S62" s="3" t="n"/>
-      <c r="T62" s="3" t="n"/>
       <c r="U62" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -4293,17 +4299,17 @@
       <c r="O63" s="3" t="n"/>
       <c r="P63" s="3" t="inlineStr">
         <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Q63" s="3" t="n"/>
+      <c r="R63" s="3" t="n"/>
+      <c r="S63" s="3" t="n"/>
+      <c r="T63" s="3" t="inlineStr">
+        <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="Q63" s="3" t="n"/>
-      <c r="R63" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="S63" s="3" t="n"/>
-      <c r="T63" s="3" t="n"/>
       <c r="U63" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -4353,17 +4359,17 @@
       <c r="O64" s="3" t="n"/>
       <c r="P64" s="3" t="inlineStr">
         <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Q64" s="3" t="n"/>
+      <c r="R64" s="3" t="n"/>
+      <c r="S64" s="3" t="n"/>
+      <c r="T64" s="3" t="inlineStr">
+        <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="Q64" s="3" t="n"/>
-      <c r="R64" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="S64" s="3" t="n"/>
-      <c r="T64" s="3" t="n"/>
       <c r="U64" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -4413,17 +4419,17 @@
       <c r="O65" s="3" t="n"/>
       <c r="P65" s="3" t="inlineStr">
         <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Q65" s="3" t="n"/>
+      <c r="R65" s="3" t="n"/>
+      <c r="S65" s="3" t="n"/>
+      <c r="T65" s="3" t="inlineStr">
+        <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="Q65" s="3" t="n"/>
-      <c r="R65" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="S65" s="3" t="n"/>
-      <c r="T65" s="3" t="n"/>
       <c r="U65" s="3" t="inlineStr">
         <is>
           <t>true</t>
@@ -4432,98 +4438,88 @@
       <c r="V65" s="3" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:013000</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>participant engagement with behaviour change intervention</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>Participant engagement with intervention, where the intervention focuses on changing behaviour.</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>participant engagement with intervention</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>BCI engagement</t>
-        </is>
-      </c>
-      <c r="F66" s="2" t="n"/>
-      <c r="G66" s="2" t="inlineStr">
-        <is>
-          <t>Includes mental activities and behaviours.</t>
-        </is>
-      </c>
-      <c r="H66" s="2" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="I66" s="2" t="n"/>
-      <c r="J66" s="2" t="n"/>
-      <c r="K66" s="2" t="n"/>
-      <c r="L66" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
-      <c r="M66" s="2" t="n"/>
-      <c r="N66" s="2" t="n"/>
-      <c r="O66" s="2" t="n"/>
-      <c r="P66" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW; PS</t>
-        </is>
-      </c>
-      <c r="Q66" s="2" t="n"/>
-      <c r="R66" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S66" s="2" t="n"/>
-      <c r="T66" s="2" t="n"/>
-      <c r="U66" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V66" s="2" t="n"/>
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:010004</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>occupational role of source</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>A personal role of source that is realised by doing a specified type of work or working in a specified way.</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>personal role of source</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr"/>
+      <c r="F66" s="4" t="inlineStr"/>
+      <c r="G66" s="4" t="inlineStr"/>
+      <c r="H66" s="4" t="inlineStr"/>
+      <c r="I66" s="4" t="inlineStr"/>
+      <c r="J66" s="4" t="inlineStr"/>
+      <c r="K66" s="4" t="inlineStr"/>
+      <c r="L66" s="4" t="inlineStr"/>
+      <c r="M66" s="4" t="inlineStr"/>
+      <c r="N66" s="4" t="inlineStr"/>
+      <c r="O66" s="4" t="inlineStr"/>
+      <c r="P66" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="Q66" s="4" t="inlineStr"/>
+      <c r="R66" s="4" t="inlineStr"/>
+      <c r="S66" s="4" t="inlineStr"/>
+      <c r="T66" s="4" t="inlineStr"/>
+      <c r="U66" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V66" s="4" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050916</t>
+          <t>BCIO:013000</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
+          <t>participant engagement with behaviour change intervention</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Participant engagement with intervention, where the intervention focuses on changing behaviour.</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
           <t>participant engagement with intervention</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>An individual human activity of an intervention participant within one or more parts of the intervention.</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>individual human activity</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="n"/>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>BCI engagement</t>
+        </is>
+      </c>
       <c r="F67" s="2" t="n"/>
-      <c r="G67" s="2" t="n"/>
-      <c r="H67" s="2" t="n"/>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Includes mental activities and behaviours.</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
       <c r="I67" s="2" t="n"/>
       <c r="J67" s="2" t="n"/>
       <c r="K67" s="2" t="n"/>
@@ -4537,52 +4533,46 @@
       <c r="O67" s="2" t="n"/>
       <c r="P67" s="2" t="inlineStr">
         <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="Q67" s="2" t="inlineStr">
-        <is>
-          <t>The extend to someone interacts with an intervention, including their cognitive, emotional and behavioural response (e.g., attending intervention session) to the intervention itself.</t>
-        </is>
-      </c>
-      <c r="R67" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q67" s="2" t="n"/>
+      <c r="R67" s="2" t="n"/>
       <c r="S67" s="2" t="n"/>
-      <c r="T67" s="2" t="n"/>
-      <c r="U67" s="2" t="n">
-        <v>0</v>
+      <c r="T67" s="2" t="inlineStr">
+        <is>
+          <t>JH; RW; PS</t>
+        </is>
+      </c>
+      <c r="U67" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="V67" s="2" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>BCIO:034000</t>
+          <t>BCIO:050916</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>population behaviour</t>
+          <t>participant engagement with intervention</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>An aggregate of individual human behaviours of members of a population.</t>
+          <t>An individual human activity of an intervention participant within one or more parts of the intervention.</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>human behaviour</t>
-        </is>
-      </c>
+          <t>individual human activity</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="n"/>
       <c r="F68" s="2" t="n"/>
       <c r="G68" s="2" t="n"/>
       <c r="H68" s="2" t="n"/>
@@ -4599,279 +4589,281 @@
       <c r="O68" s="2" t="n"/>
       <c r="P68" s="2" t="inlineStr">
         <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q68" s="2" t="inlineStr">
+        <is>
+          <t>The extend to someone interacts with an intervention, including their cognitive, emotional and behavioural response (e.g., attending intervention session) to the intervention itself.</t>
+        </is>
+      </c>
+      <c r="R68" s="2" t="n"/>
+      <c r="S68" s="2" t="n"/>
+      <c r="T68" s="2" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V68" s="2" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:010003</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>personal role of source</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>A role that inheres in a person source.</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr"/>
+      <c r="F69" s="4" t="inlineStr"/>
+      <c r="G69" s="4" t="inlineStr"/>
+      <c r="H69" s="4" t="inlineStr"/>
+      <c r="I69" s="4" t="inlineStr"/>
+      <c r="J69" s="4" t="inlineStr"/>
+      <c r="K69" s="4" t="inlineStr"/>
+      <c r="L69" s="4" t="inlineStr"/>
+      <c r="M69" s="4" t="inlineStr"/>
+      <c r="N69" s="4" t="inlineStr"/>
+      <c r="O69" s="4" t="inlineStr"/>
+      <c r="P69" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="Q69" s="4" t="inlineStr"/>
+      <c r="R69" s="4" t="inlineStr"/>
+      <c r="S69" s="4" t="inlineStr"/>
+      <c r="T69" s="4" t="inlineStr"/>
+      <c r="U69" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V69" s="4" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:034000</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>population behaviour</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>An aggregate of individual human behaviours of members of a population.</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>human behaviour</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="n"/>
+      <c r="G70" s="2" t="n"/>
+      <c r="H70" s="2" t="n"/>
+      <c r="I70" s="2" t="n"/>
+      <c r="J70" s="2" t="n"/>
+      <c r="K70" s="2" t="n"/>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M70" s="2" t="n"/>
+      <c r="N70" s="2" t="n"/>
+      <c r="O70" s="2" t="n"/>
+      <c r="P70" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q70" s="2" t="n"/>
+      <c r="R70" s="2" t="n"/>
+      <c r="S70" s="2" t="n"/>
+      <c r="T70" s="2" t="inlineStr">
+        <is>
           <t>JH</t>
         </is>
       </c>
-      <c r="Q68" s="2" t="n"/>
-      <c r="R68" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S68" s="2" t="n"/>
-      <c r="T68" s="2" t="n"/>
-      <c r="U68" s="2" t="inlineStr">
+      <c r="U70" s="2" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="V68" s="2" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:043000</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>process attribute</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>A process profile that is an attribute of a process.</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>process profile</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="n"/>
-      <c r="F69" s="2" t="n"/>
-      <c r="G69" s="2" t="inlineStr">
-        <is>
-          <t>This is intended to provide a user-friendly way of representing the way in which processes are manifest. This is somewhat similar to, but not the same as, the class 'specifically dependent continuant' in Basic Formal Ontology which provides a way of representing features of material entities such as age and size. It is formally equivalent to process profile in Basic Formal Ontology.</t>
-        </is>
-      </c>
-      <c r="H69" s="2" t="n"/>
-      <c r="I69" s="2" t="n"/>
-      <c r="J69" s="2" t="n"/>
-      <c r="K69" s="2" t="n"/>
-      <c r="L69" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
-      <c r="M69" s="2" t="n"/>
-      <c r="N69" s="2" t="n"/>
-      <c r="O69" s="2" t="n"/>
-      <c r="P69" s="2" t="inlineStr">
-        <is>
-          <t>JH</t>
-        </is>
-      </c>
-      <c r="Q69" s="2" t="inlineStr">
-        <is>
-          <t>An attribute of a process.</t>
-        </is>
-      </c>
-      <c r="R69" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S69" s="2" t="n"/>
-      <c r="T69" s="2" t="n"/>
-      <c r="U69" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V69" s="2" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="3" t="inlineStr">
-        <is>
-          <t>GMHO:0000268</t>
-        </is>
-      </c>
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>process context</t>
-        </is>
-      </c>
-      <c r="C70" s="3" t="n"/>
-      <c r="D70" s="3" t="inlineStr">
-        <is>
-          <t>entity</t>
-        </is>
-      </c>
-      <c r="E70" s="3" t="n"/>
-      <c r="F70" s="3" t="n"/>
-      <c r="G70" s="3" t="n"/>
-      <c r="H70" s="3" t="n"/>
-      <c r="I70" s="3" t="n"/>
-      <c r="J70" s="3" t="n"/>
-      <c r="K70" s="3" t="n"/>
-      <c r="L70" s="3" t="n"/>
-      <c r="M70" s="3" t="n"/>
-      <c r="N70" s="3" t="n"/>
-      <c r="O70" s="3" t="n"/>
-      <c r="P70" s="3" t="n"/>
-      <c r="Q70" s="3" t="n"/>
-      <c r="R70" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="S70" s="3" t="n"/>
-      <c r="T70" s="3" t="n"/>
-      <c r="U70" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="V70" s="3" t="n"/>
+      <c r="V70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>BCIO:051027</t>
+          <t>BCIO:043000</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>process context</t>
+          <t>process attribute</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>An entity that includes the material and temporal contexts that are not part of but may influence the outcome of a process.</t>
+          <t>A process profile that is an attribute of a process.</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>entity</t>
+          <t>process profile</t>
         </is>
       </c>
       <c r="E71" s="2" t="n"/>
-      <c r="F71" s="2" t="inlineStr">
-        <is>
-          <t>'temporal context of process' OR 'material context of process'</t>
-        </is>
-      </c>
-      <c r="G71" s="2" t="n"/>
+      <c r="F71" s="2" t="n"/>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>This is intended to provide a user-friendly way of representing the way in which processes are manifest. This is somewhat similar to, but not the same as, the class 'specifically dependent continuant' in Basic Formal Ontology which provides a way of representing features of material entities such as age and size. It is formally equivalent to process profile in Basic Formal Ontology.</t>
+        </is>
+      </c>
       <c r="H71" s="2" t="n"/>
       <c r="I71" s="2" t="n"/>
       <c r="J71" s="2" t="n"/>
       <c r="K71" s="2" t="n"/>
-      <c r="L71" s="2" t="n"/>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="M71" s="2" t="n"/>
       <c r="N71" s="2" t="n"/>
       <c r="O71" s="2" t="n"/>
-      <c r="P71" s="2" t="n"/>
-      <c r="Q71" s="2" t="n"/>
-      <c r="R71" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="P71" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q71" s="2" t="inlineStr">
+        <is>
+          <t>An attribute of a process.</t>
+        </is>
+      </c>
+      <c r="R71" s="2" t="n"/>
       <c r="S71" s="2" t="n"/>
-      <c r="T71" s="2" t="n"/>
-      <c r="U71" s="2" t="n">
+      <c r="T71" s="2" t="inlineStr">
+        <is>
+          <t>JH</t>
+        </is>
+      </c>
+      <c r="U71" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V71" s="2" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>GMHO:0000268</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>process context</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="n"/>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>entity</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="n"/>
+      <c r="F72" s="3" t="n"/>
+      <c r="G72" s="3" t="n"/>
+      <c r="H72" s="3" t="n"/>
+      <c r="I72" s="3" t="n"/>
+      <c r="J72" s="3" t="n"/>
+      <c r="K72" s="3" t="n"/>
+      <c r="L72" s="3" t="n"/>
+      <c r="M72" s="3" t="n"/>
+      <c r="N72" s="3" t="n"/>
+      <c r="O72" s="3" t="n"/>
+      <c r="P72" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Q72" s="3" t="n"/>
+      <c r="R72" s="3" t="n"/>
+      <c r="S72" s="3" t="n"/>
+      <c r="T72" s="3" t="n"/>
+      <c r="U72" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="V71" s="2" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:050551</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="inlineStr">
-        <is>
-          <t>research study participants</t>
-        </is>
-      </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>A population that is studied in a research study.</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>human population</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="n"/>
-      <c r="F72" s="2" t="n"/>
-      <c r="G72" s="2" t="n"/>
-      <c r="H72" s="2" t="n"/>
-      <c r="I72" s="2" t="n"/>
-      <c r="J72" s="2" t="n"/>
-      <c r="K72" s="2" t="n"/>
-      <c r="L72" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
-      <c r="M72" s="2" t="n"/>
-      <c r="N72" s="2" t="n"/>
-      <c r="O72" s="2" t="n"/>
-      <c r="P72" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="Q72" s="2" t="n"/>
-      <c r="R72" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="S72" s="2" t="n"/>
-      <c r="T72" s="2" t="n"/>
-      <c r="U72" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="V72" s="2" t="n"/>
+      <c r="V72" s="3" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>BCIO:051028</t>
+          <t>BCIO:051027</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>temporal context of process</t>
+          <t>process context</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>An occurrent that is not dependent on a process but may influence the effect of the process on its outcome.</t>
+          <t>An entity that includes the material and temporal contexts that are not part of but may influence the outcome of a process.</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>occurrent</t>
+          <t>entity</t>
         </is>
       </c>
       <c r="E73" s="2" t="n"/>
-      <c r="F73" s="2" t="n"/>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>'temporal context of process' OR 'material context of process'</t>
+        </is>
+      </c>
       <c r="G73" s="2" t="n"/>
       <c r="H73" s="2" t="n"/>
-      <c r="I73" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">This entity includes time periods, events, etc. </t>
-        </is>
-      </c>
+      <c r="I73" s="2" t="n"/>
       <c r="J73" s="2" t="n"/>
       <c r="K73" s="2" t="n"/>
       <c r="L73" s="2" t="n"/>
       <c r="M73" s="2" t="n"/>
       <c r="N73" s="2" t="n"/>
       <c r="O73" s="2" t="n"/>
-      <c r="P73" s="2" t="n"/>
+      <c r="P73" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
       <c r="Q73" s="2" t="n"/>
-      <c r="R73" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
+      <c r="R73" s="2" t="n"/>
       <c r="S73" s="2" t="n"/>
       <c r="T73" s="2" t="n"/>
       <c r="U73" s="2" t="n">
@@ -4879,6 +4871,158 @@
       </c>
       <c r="V73" s="2" t="n"/>
     </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:050551</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>research study participants</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>A population that is studied in a research study.</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>human population</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="n"/>
+      <c r="F74" s="2" t="n"/>
+      <c r="G74" s="2" t="n"/>
+      <c r="H74" s="2" t="n"/>
+      <c r="I74" s="2" t="n"/>
+      <c r="J74" s="2" t="n"/>
+      <c r="K74" s="2" t="n"/>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M74" s="2" t="n"/>
+      <c r="N74" s="2" t="n"/>
+      <c r="O74" s="2" t="n"/>
+      <c r="P74" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q74" s="2" t="n"/>
+      <c r="R74" s="2" t="n"/>
+      <c r="S74" s="2" t="n"/>
+      <c r="T74" s="2" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U74" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V74" s="2" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:010083</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>researcher role</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>A occupational role played by a person that contributes substantively to production or reporting of a research study.</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>occupational role of source</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr"/>
+      <c r="F75" s="4" t="inlineStr"/>
+      <c r="G75" s="4" t="inlineStr"/>
+      <c r="H75" s="4" t="inlineStr"/>
+      <c r="I75" s="4" t="inlineStr"/>
+      <c r="J75" s="4" t="inlineStr"/>
+      <c r="K75" s="4" t="inlineStr"/>
+      <c r="L75" s="4" t="inlineStr"/>
+      <c r="M75" s="4" t="inlineStr"/>
+      <c r="N75" s="4" t="inlineStr"/>
+      <c r="O75" s="4" t="inlineStr"/>
+      <c r="P75" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="Q75" s="4" t="inlineStr"/>
+      <c r="R75" s="4" t="inlineStr"/>
+      <c r="S75" s="4" t="inlineStr"/>
+      <c r="T75" s="4" t="inlineStr"/>
+      <c r="U75" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V75" s="4" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:051028</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>temporal context of process</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>An occurrent that is not dependent on a process but may influence the effect of the process on its outcome.</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>occurrent</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="n"/>
+      <c r="F76" s="2" t="n"/>
+      <c r="G76" s="2" t="n"/>
+      <c r="H76" s="2" t="n"/>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This entity includes time periods, events, etc. </t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="n"/>
+      <c r="K76" s="2" t="n"/>
+      <c r="L76" s="2" t="n"/>
+      <c r="M76" s="2" t="n"/>
+      <c r="N76" s="2" t="n"/>
+      <c r="O76" s="2" t="n"/>
+      <c r="P76" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q76" s="2" t="n"/>
+      <c r="R76" s="2" t="n"/>
+      <c r="S76" s="2" t="n"/>
+      <c r="T76" s="2" t="n"/>
+      <c r="U76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V76" s="2" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add material context of process to BCIO_Upper_Defs.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
@@ -30,7 +30,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +47,11 @@
         <fgColor rgb="002f4f4f"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ffffff"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -60,11 +65,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V76"/>
+  <dimension ref="A1:V77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4192,84 +4198,70 @@
       <c r="V61" s="3" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:050470</t>
-        </is>
-      </c>
-      <c r="B62" s="3" t="inlineStr">
-        <is>
-          <t>moderate cognitive exertion expended on a behaviour</t>
-        </is>
-      </c>
-      <c r="C62" s="3" t="inlineStr">
-        <is>
-          <t>Cognitive exertion expended on a behaviour that is medium.</t>
-        </is>
-      </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>cognitive exertion expended on a behaviour</t>
-        </is>
-      </c>
-      <c r="E62" s="3" t="n"/>
-      <c r="F62" s="3" t="n"/>
-      <c r="G62" s="3" t="n"/>
-      <c r="H62" s="3" t="n"/>
-      <c r="I62" s="3" t="inlineStr">
-        <is>
-          <t>Moderate cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
-        </is>
-      </c>
-      <c r="J62" s="3" t="n"/>
-      <c r="K62" s="3" t="n"/>
-      <c r="L62" s="3" t="inlineStr">
-        <is>
-          <t>behaviour</t>
-        </is>
-      </c>
-      <c r="M62" s="3" t="n"/>
-      <c r="N62" s="3" t="n"/>
-      <c r="O62" s="3" t="n"/>
-      <c r="P62" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="Q62" s="3" t="n"/>
-      <c r="R62" s="3" t="n"/>
-      <c r="S62" s="3" t="n"/>
-      <c r="T62" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="U62" s="3" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="V62" s="3" t="n"/>
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:051029</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>material context of process</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>A material entity that is not dependent on a process but may influence the effect of the process on its outcome.</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr"/>
+      <c r="F62" s="4" t="inlineStr"/>
+      <c r="G62" s="4" t="inlineStr"/>
+      <c r="H62" s="4" t="inlineStr"/>
+      <c r="I62" s="4" t="inlineStr"/>
+      <c r="J62" s="4" t="inlineStr"/>
+      <c r="K62" s="4" t="inlineStr"/>
+      <c r="L62" s="4" t="inlineStr"/>
+      <c r="M62" s="4" t="inlineStr"/>
+      <c r="N62" s="4" t="inlineStr"/>
+      <c r="O62" s="4" t="inlineStr"/>
+      <c r="P62" s="4" t="inlineStr">
+        <is>
+          <t>Proposed</t>
+        </is>
+      </c>
+      <c r="Q62" s="4" t="inlineStr"/>
+      <c r="R62" s="4" t="inlineStr"/>
+      <c r="S62" s="4" t="inlineStr"/>
+      <c r="T62" s="4" t="inlineStr"/>
+      <c r="U62" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V62" s="4" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050471</t>
+          <t>BCIO:050470</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>moderate emotional management exertion expended on a behaviour</t>
+          <t>moderate cognitive exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Emotional management exertion expended on a behaviour that is medium.</t>
+          <t>Cognitive exertion expended on a behaviour that is medium.</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>emotional management exertion expended on a behaviour</t>
+          <t>cognitive exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E63" s="3" t="n"/>
@@ -4278,7 +4270,7 @@
       <c r="H63" s="3" t="n"/>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>Moderate emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
+          <t>Moderate cognitive exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J63" s="3" t="n"/>
@@ -4314,22 +4306,22 @@
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050472</t>
+          <t>BCIO:050471</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>moderate mental exertion expended on a behaviour</t>
+          <t>moderate emotional management exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Mental exertion expended on a behaviour that is medium.</t>
+          <t>Emotional management exertion expended on a behaviour that is medium.</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>mental exertion expended on a behaviour</t>
+          <t>emotional management exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E64" s="3" t="n"/>
@@ -4338,7 +4330,7 @@
       <c r="H64" s="3" t="n"/>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>Moderate mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
+          <t>Moderate emotional management exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J64" s="3" t="n"/>
@@ -4374,22 +4366,22 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>BCIO:050473</t>
+          <t>BCIO:050472</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>moderate physical exertion expended on behaviour</t>
+          <t>moderate mental exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Physical exertion expended on a behaviour that is medium.</t>
+          <t>Mental exertion expended on a behaviour that is medium.</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>physical exertion expended on a behaviour</t>
+          <t>mental exertion expended on a behaviour</t>
         </is>
       </c>
       <c r="E65" s="3" t="n"/>
@@ -4398,7 +4390,7 @@
       <c r="H65" s="3" t="n"/>
       <c r="I65" s="3" t="inlineStr">
         <is>
-          <t>Moderate physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
+          <t>Moderate mental exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
         </is>
       </c>
       <c r="J65" s="3" t="n"/>
@@ -4432,96 +4424,94 @@
       <c r="V65" s="3" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:010004</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>occupational role of source</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>A personal role of source that is realised by doing a specified type of work or working in a specified way.</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>personal role of source</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="n"/>
-      <c r="F66" s="2" t="n"/>
-      <c r="G66" s="2" t="n"/>
-      <c r="H66" s="2" t="n"/>
-      <c r="I66" s="2" t="n"/>
-      <c r="J66" s="2" t="n"/>
-      <c r="K66" s="2" t="n"/>
-      <c r="L66" s="2" t="n"/>
-      <c r="M66" s="2" t="n"/>
-      <c r="N66" s="2" t="n"/>
-      <c r="O66" s="2" t="n"/>
-      <c r="P66" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="Q66" s="2" t="n"/>
-      <c r="R66" s="2" t="n"/>
-      <c r="S66" s="2" t="n"/>
-      <c r="T66" s="2" t="n"/>
-      <c r="U66" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="V66" s="2" t="n"/>
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:050473</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>moderate physical exertion expended on behaviour</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>Physical exertion expended on a behaviour that is medium.</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>physical exertion expended on a behaviour</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="n"/>
+      <c r="F66" s="3" t="n"/>
+      <c r="G66" s="3" t="n"/>
+      <c r="H66" s="3" t="n"/>
+      <c r="I66" s="3" t="inlineStr">
+        <is>
+          <t>Moderate physical exertion will mean different things depending on how this concept is operationalised. Therefore, when using this class, you would need to operationalise it for the relevant context (e.g., specify what moderate exertion means based on the measurement you use).</t>
+        </is>
+      </c>
+      <c r="J66" s="3" t="n"/>
+      <c r="K66" s="3" t="n"/>
+      <c r="L66" s="3" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="M66" s="3" t="n"/>
+      <c r="N66" s="3" t="n"/>
+      <c r="O66" s="3" t="n"/>
+      <c r="P66" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="Q66" s="3" t="n"/>
+      <c r="R66" s="3" t="n"/>
+      <c r="S66" s="3" t="n"/>
+      <c r="T66" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U66" s="3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="V66" s="3" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>BCIO:013000</t>
+          <t>BCIO:010004</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>participant engagement with behaviour change intervention</t>
+          <t>occupational role of source</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Participant engagement with intervention, where the intervention focuses on changing behaviour.</t>
+          <t>A personal role of source that is realised by doing a specified type of work or working in a specified way.</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>participant engagement with intervention</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>BCI engagement</t>
-        </is>
-      </c>
+          <t>personal role of source</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="n"/>
       <c r="F67" s="2" t="n"/>
-      <c r="G67" s="2" t="inlineStr">
-        <is>
-          <t>Includes mental activities and behaviours.</t>
-        </is>
-      </c>
-      <c r="H67" s="2" t="inlineStr">
-        <is>
-          <t>process</t>
-        </is>
-      </c>
+      <c r="G67" s="2" t="n"/>
+      <c r="H67" s="2" t="n"/>
       <c r="I67" s="2" t="n"/>
       <c r="J67" s="2" t="n"/>
       <c r="K67" s="2" t="n"/>
-      <c r="L67" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="L67" s="2" t="n"/>
       <c r="M67" s="2" t="n"/>
       <c r="N67" s="2" t="n"/>
       <c r="O67" s="2" t="n"/>
@@ -4533,43 +4523,49 @@
       <c r="Q67" s="2" t="n"/>
       <c r="R67" s="2" t="n"/>
       <c r="S67" s="2" t="n"/>
-      <c r="T67" s="2" t="inlineStr">
-        <is>
-          <t>JH; RW; PS</t>
-        </is>
-      </c>
-      <c r="U67" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="T67" s="2" t="n"/>
+      <c r="U67" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="V67" s="2" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050916</t>
+          <t>BCIO:013000</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
+          <t>participant engagement with behaviour change intervention</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Participant engagement with intervention, where the intervention focuses on changing behaviour.</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
           <t>participant engagement with intervention</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>An individual human activity of an intervention participant within one or more parts of the intervention.</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>individual human activity</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="n"/>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>BCI engagement</t>
+        </is>
+      </c>
       <c r="F68" s="2" t="n"/>
-      <c r="G68" s="2" t="n"/>
-      <c r="H68" s="2" t="n"/>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Includes mental activities and behaviours.</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
       <c r="I68" s="2" t="n"/>
       <c r="J68" s="2" t="n"/>
       <c r="K68" s="2" t="n"/>
@@ -4586,42 +4582,40 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="Q68" s="2" t="inlineStr">
-        <is>
-          <t>The extend to someone interacts with an intervention, including their cognitive, emotional and behavioural response (e.g., attending intervention session) to the intervention itself.</t>
-        </is>
-      </c>
+      <c r="Q68" s="2" t="n"/>
       <c r="R68" s="2" t="n"/>
       <c r="S68" s="2" t="n"/>
       <c r="T68" s="2" t="inlineStr">
         <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="U68" s="2" t="n">
-        <v>0</v>
+          <t>JH; RW; PS</t>
+        </is>
+      </c>
+      <c r="U68" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="V68" s="2" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>BCIO:010003</t>
+          <t>BCIO:050916</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>personal role of source</t>
+          <t>participant engagement with intervention</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>A role that inheres in a person source.</t>
+          <t>An individual human activity of an intervention participant within one or more parts of the intervention.</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>role</t>
+          <t>individual human activity</t>
         </is>
       </c>
       <c r="E69" s="2" t="n"/>
@@ -4631,7 +4625,11 @@
       <c r="I69" s="2" t="n"/>
       <c r="J69" s="2" t="n"/>
       <c r="K69" s="2" t="n"/>
-      <c r="L69" s="2" t="n"/>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="M69" s="2" t="n"/>
       <c r="N69" s="2" t="n"/>
       <c r="O69" s="2" t="n"/>
@@ -4640,10 +4638,18 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="Q69" s="2" t="n"/>
+      <c r="Q69" s="2" t="inlineStr">
+        <is>
+          <t>The extend to someone interacts with an intervention, including their cognitive, emotional and behavioural response (e.g., attending intervention session) to the intervention itself.</t>
+        </is>
+      </c>
       <c r="R69" s="2" t="n"/>
       <c r="S69" s="2" t="n"/>
-      <c r="T69" s="2" t="n"/>
+      <c r="T69" s="2" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
       <c r="U69" s="2" t="n">
         <v>0</v>
       </c>
@@ -4652,40 +4658,32 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>BCIO:034000</t>
+          <t>BCIO:010003</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>population behaviour</t>
+          <t>personal role of source</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>An aggregate of individual human behaviours of members of a population.</t>
+          <t>A role that inheres in a person source.</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>process</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>human behaviour</t>
-        </is>
-      </c>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="n"/>
       <c r="F70" s="2" t="n"/>
       <c r="G70" s="2" t="n"/>
       <c r="H70" s="2" t="n"/>
       <c r="I70" s="2" t="n"/>
       <c r="J70" s="2" t="n"/>
       <c r="K70" s="2" t="n"/>
-      <c r="L70" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="L70" s="2" t="n"/>
       <c r="M70" s="2" t="n"/>
       <c r="N70" s="2" t="n"/>
       <c r="O70" s="2" t="n"/>
@@ -4697,46 +4695,40 @@
       <c r="Q70" s="2" t="n"/>
       <c r="R70" s="2" t="n"/>
       <c r="S70" s="2" t="n"/>
-      <c r="T70" s="2" t="inlineStr">
-        <is>
-          <t>JH</t>
-        </is>
-      </c>
-      <c r="U70" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="T70" s="2" t="n"/>
+      <c r="U70" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="V70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>BCIO:043000</t>
+          <t>BCIO:034000</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>process attribute</t>
+          <t>population behaviour</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>A process profile that is an attribute of a process.</t>
+          <t>An aggregate of individual human behaviours of members of a population.</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>process profile</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="n"/>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>human behaviour</t>
+        </is>
+      </c>
       <c r="F71" s="2" t="n"/>
-      <c r="G71" s="2" t="inlineStr">
-        <is>
-          <t>This is intended to provide a user-friendly way of representing the way in which processes are manifest. This is somewhat similar to, but not the same as, the class 'specifically dependent continuant' in Basic Formal Ontology which provides a way of representing features of material entities such as age and size. It is formally equivalent to process profile in Basic Formal Ontology.</t>
-        </is>
-      </c>
+      <c r="G71" s="2" t="n"/>
       <c r="H71" s="2" t="n"/>
       <c r="I71" s="2" t="n"/>
       <c r="J71" s="2" t="n"/>
@@ -4754,11 +4746,7 @@
           <t>Published</t>
         </is>
       </c>
-      <c r="Q71" s="2" t="inlineStr">
-        <is>
-          <t>An attribute of a process.</t>
-        </is>
-      </c>
+      <c r="Q71" s="2" t="n"/>
       <c r="R71" s="2" t="n"/>
       <c r="S71" s="2" t="n"/>
       <c r="T71" s="2" t="inlineStr">
@@ -4774,130 +4762,144 @@
       <c r="V71" s="2" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="3" t="inlineStr">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:043000</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>process attribute</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>A process profile that is an attribute of a process.</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>process profile</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="n"/>
+      <c r="F72" s="2" t="n"/>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>This is intended to provide a user-friendly way of representing the way in which processes are manifest. This is somewhat similar to, but not the same as, the class 'specifically dependent continuant' in Basic Formal Ontology which provides a way of representing features of material entities such as age and size. It is formally equivalent to process profile in Basic Formal Ontology.</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="n"/>
+      <c r="I72" s="2" t="n"/>
+      <c r="J72" s="2" t="n"/>
+      <c r="K72" s="2" t="n"/>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
+      <c r="M72" s="2" t="n"/>
+      <c r="N72" s="2" t="n"/>
+      <c r="O72" s="2" t="n"/>
+      <c r="P72" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q72" s="2" t="inlineStr">
+        <is>
+          <t>An attribute of a process.</t>
+        </is>
+      </c>
+      <c r="R72" s="2" t="n"/>
+      <c r="S72" s="2" t="n"/>
+      <c r="T72" s="2" t="inlineStr">
+        <is>
+          <t>JH</t>
+        </is>
+      </c>
+      <c r="U72" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V72" s="2" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
         <is>
           <t>GMHO:0000268</t>
         </is>
       </c>
-      <c r="B72" s="3" t="inlineStr">
+      <c r="B73" s="3" t="inlineStr">
         <is>
           <t>process context</t>
         </is>
       </c>
-      <c r="C72" s="3" t="n"/>
-      <c r="D72" s="3" t="inlineStr">
+      <c r="C73" s="3" t="n"/>
+      <c r="D73" s="3" t="inlineStr">
         <is>
           <t>entity</t>
         </is>
       </c>
-      <c r="E72" s="3" t="n"/>
-      <c r="F72" s="3" t="n"/>
-      <c r="G72" s="3" t="n"/>
-      <c r="H72" s="3" t="n"/>
-      <c r="I72" s="3" t="n"/>
-      <c r="J72" s="3" t="n"/>
-      <c r="K72" s="3" t="n"/>
-      <c r="L72" s="3" t="n"/>
-      <c r="M72" s="3" t="n"/>
-      <c r="N72" s="3" t="n"/>
-      <c r="O72" s="3" t="n"/>
-      <c r="P72" s="3" t="inlineStr">
+      <c r="E73" s="3" t="n"/>
+      <c r="F73" s="3" t="n"/>
+      <c r="G73" s="3" t="n"/>
+      <c r="H73" s="3" t="n"/>
+      <c r="I73" s="3" t="n"/>
+      <c r="J73" s="3" t="n"/>
+      <c r="K73" s="3" t="n"/>
+      <c r="L73" s="3" t="n"/>
+      <c r="M73" s="3" t="n"/>
+      <c r="N73" s="3" t="n"/>
+      <c r="O73" s="3" t="n"/>
+      <c r="P73" s="3" t="inlineStr">
         <is>
           <t>Obsolete</t>
         </is>
       </c>
-      <c r="Q72" s="3" t="n"/>
-      <c r="R72" s="3" t="n"/>
-      <c r="S72" s="3" t="n"/>
-      <c r="T72" s="3" t="n"/>
-      <c r="U72" s="3" t="n">
+      <c r="Q73" s="3" t="n"/>
+      <c r="R73" s="3" t="n"/>
+      <c r="S73" s="3" t="n"/>
+      <c r="T73" s="3" t="n"/>
+      <c r="U73" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="V72" s="3" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>BCIO:051027</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
-        <is>
-          <t>process context</t>
-        </is>
-      </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>An entity that includes the material and temporal contexts that are not part of but may influence the outcome of a process.</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="inlineStr">
-        <is>
-          <t>entity</t>
-        </is>
-      </c>
-      <c r="E73" s="2" t="n"/>
-      <c r="F73" s="2" t="inlineStr">
-        <is>
-          <t>'temporal context of process' OR 'material context of process'</t>
-        </is>
-      </c>
-      <c r="G73" s="2" t="n"/>
-      <c r="H73" s="2" t="n"/>
-      <c r="I73" s="2" t="n"/>
-      <c r="J73" s="2" t="n"/>
-      <c r="K73" s="2" t="n"/>
-      <c r="L73" s="2" t="n"/>
-      <c r="M73" s="2" t="n"/>
-      <c r="N73" s="2" t="n"/>
-      <c r="O73" s="2" t="n"/>
-      <c r="P73" s="2" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="Q73" s="2" t="n"/>
-      <c r="R73" s="2" t="n"/>
-      <c r="S73" s="2" t="n"/>
-      <c r="T73" s="2" t="n"/>
-      <c r="U73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="V73" s="2" t="n"/>
+      <c r="V73" s="3" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>BCIO:050551</t>
+          <t>BCIO:051027</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>research study participants</t>
+          <t>process context</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>A population that is studied in a research study.</t>
+          <t>An entity that includes the material and temporal contexts that are not part of but may influence the outcome of a process.</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>human population</t>
+          <t>entity</t>
         </is>
       </c>
       <c r="E74" s="2" t="n"/>
-      <c r="F74" s="2" t="n"/>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>'temporal context of process' OR 'material context of process'</t>
+        </is>
+      </c>
       <c r="G74" s="2" t="n"/>
       <c r="H74" s="2" t="n"/>
       <c r="I74" s="2" t="n"/>
       <c r="J74" s="2" t="n"/>
       <c r="K74" s="2" t="n"/>
-      <c r="L74" s="2" t="inlineStr">
-        <is>
-          <t>Upper level</t>
-        </is>
-      </c>
+      <c r="L74" s="2" t="n"/>
       <c r="M74" s="2" t="n"/>
       <c r="N74" s="2" t="n"/>
       <c r="O74" s="2" t="n"/>
@@ -4909,37 +4911,31 @@
       <c r="Q74" s="2" t="n"/>
       <c r="R74" s="2" t="n"/>
       <c r="S74" s="2" t="n"/>
-      <c r="T74" s="2" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="U74" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="T74" s="2" t="n"/>
+      <c r="U74" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="V74" s="2" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>BCIO:010083</t>
+          <t>BCIO:050551</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>researcher role</t>
+          <t>research study participants</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>A occupational role played by a person that contributes substantively to production or reporting of a research study.</t>
+          <t>A population that is studied in a research study.</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>occupational role of source</t>
+          <t>human population</t>
         </is>
       </c>
       <c r="E75" s="2" t="n"/>
@@ -4949,7 +4945,11 @@
       <c r="I75" s="2" t="n"/>
       <c r="J75" s="2" t="n"/>
       <c r="K75" s="2" t="n"/>
-      <c r="L75" s="2" t="n"/>
+      <c r="L75" s="2" t="inlineStr">
+        <is>
+          <t>Upper level</t>
+        </is>
+      </c>
       <c r="M75" s="2" t="n"/>
       <c r="N75" s="2" t="n"/>
       <c r="O75" s="2" t="n"/>
@@ -4961,42 +4961,44 @@
       <c r="Q75" s="2" t="n"/>
       <c r="R75" s="2" t="n"/>
       <c r="S75" s="2" t="n"/>
-      <c r="T75" s="2" t="n"/>
-      <c r="U75" s="2" t="n">
-        <v>0</v>
+      <c r="T75" s="2" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="U75" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="V75" s="2" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>BCIO:051028</t>
+          <t>BCIO:010083</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>temporal context of process</t>
+          <t>researcher role</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>An occurrent that is not dependent on a process but may influence the effect of the process on its outcome.</t>
+          <t>A occupational role played by a person that contributes substantively to production or reporting of a research study.</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>occurrent</t>
+          <t>occupational role of source</t>
         </is>
       </c>
       <c r="E76" s="2" t="n"/>
       <c r="F76" s="2" t="n"/>
       <c r="G76" s="2" t="n"/>
       <c r="H76" s="2" t="n"/>
-      <c r="I76" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">This entity includes time periods, events, etc. </t>
-        </is>
-      </c>
+      <c r="I76" s="2" t="n"/>
       <c r="J76" s="2" t="n"/>
       <c r="K76" s="2" t="n"/>
       <c r="L76" s="2" t="n"/>
@@ -5017,6 +5019,56 @@
       </c>
       <c r="V76" s="2" t="n"/>
     </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>BCIO:051028</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>temporal context of process</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>An occurrent that is not dependent on a process but may influence the effect of the process on its outcome.</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>occurrent</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="n"/>
+      <c r="F77" s="2" t="n"/>
+      <c r="G77" s="2" t="n"/>
+      <c r="H77" s="2" t="n"/>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This entity includes time periods, events, etc. </t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="n"/>
+      <c r="K77" s="2" t="n"/>
+      <c r="L77" s="2" t="n"/>
+      <c r="M77" s="2" t="n"/>
+      <c r="N77" s="2" t="n"/>
+      <c r="O77" s="2" t="n"/>
+      <c r="P77" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q77" s="2" t="n"/>
+      <c r="R77" s="2" t="n"/>
+      <c r="S77" s="2" t="n"/>
+      <c r="T77" s="2" t="n"/>
+      <c r="U77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V77" s="2" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update material context of process in BCIO_Upper_Defs.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_Upper_Defs.xlsx
@@ -30,7 +30,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,11 +47,6 @@
         <fgColor rgb="002f4f4f"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00ffffff"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -65,12 +60,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4198,50 +4192,50 @@
       <c r="V61" s="3" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="4" t="inlineStr">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>BCIO:051029</t>
         </is>
       </c>
-      <c r="B62" s="4" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>material context of process</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>A material entity that is not dependent on a process but may influence the effect of the process on its outcome.</t>
         </is>
       </c>
-      <c r="D62" s="4" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>material entity</t>
         </is>
       </c>
-      <c r="E62" s="4" t="inlineStr"/>
-      <c r="F62" s="4" t="inlineStr"/>
-      <c r="G62" s="4" t="inlineStr"/>
-      <c r="H62" s="4" t="inlineStr"/>
-      <c r="I62" s="4" t="inlineStr"/>
-      <c r="J62" s="4" t="inlineStr"/>
-      <c r="K62" s="4" t="inlineStr"/>
-      <c r="L62" s="4" t="inlineStr"/>
-      <c r="M62" s="4" t="inlineStr"/>
-      <c r="N62" s="4" t="inlineStr"/>
-      <c r="O62" s="4" t="inlineStr"/>
-      <c r="P62" s="4" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="Q62" s="4" t="inlineStr"/>
-      <c r="R62" s="4" t="inlineStr"/>
-      <c r="S62" s="4" t="inlineStr"/>
-      <c r="T62" s="4" t="inlineStr"/>
-      <c r="U62" s="4" t="n">
+      <c r="E62" s="2" t="n"/>
+      <c r="F62" s="2" t="n"/>
+      <c r="G62" s="2" t="n"/>
+      <c r="H62" s="2" t="n"/>
+      <c r="I62" s="2" t="n"/>
+      <c r="J62" s="2" t="n"/>
+      <c r="K62" s="2" t="n"/>
+      <c r="L62" s="2" t="n"/>
+      <c r="M62" s="2" t="n"/>
+      <c r="N62" s="2" t="n"/>
+      <c r="O62" s="2" t="n"/>
+      <c r="P62" s="2" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="Q62" s="2" t="n"/>
+      <c r="R62" s="2" t="n"/>
+      <c r="S62" s="2" t="n"/>
+      <c r="T62" s="2" t="n"/>
+      <c r="U62" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="V62" s="4" t="inlineStr"/>
+      <c r="V62" s="2" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -5043,7 +5037,7 @@
       <c r="E77" s="2" t="n"/>
       <c r="F77" s="2" t="n"/>
       <c r="G77" s="2" t="n"/>
-      <c r="H77" s="2" t="n"/>
+      <c r="H77" s="2" t="inlineStr"/>
       <c r="I77" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">This entity includes time periods, events, etc. </t>

</xml_diff>